<commit_message>
Clarify taxonomy, evidence, and ranking limits
</commit_message>
<xml_diff>
--- a/notes/01-video-to-robotics-transition/video_to_robotics_architecture_pilot.xlsx
+++ b/notes/01-video-to-robotics-transition/video_to_robotics_architecture_pilot.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Method" sheetId="1" r:id="Rc54cf1abdcde4a0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="R1b45709ed78e4fc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Researchers" sheetId="3" r:id="R0dfcf6492ae84e7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="4" r:id="R0c6c37f9bb034ad3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R239c5a1c938841fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Matrix" sheetId="6" r:id="Re4227b421d3e4e49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact_Ranking" sheetId="7" r:id="R07d913c838a94bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Method" sheetId="1" r:id="Rac15678f70e040a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="R4d68dec3ca954dcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Researchers" sheetId="3" r:id="Rf452392e6b8a4f3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="4" r:id="R4ee084819038450c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R50871ad3eb02474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Matrix" sheetId="6" r:id="R5a16de437c4e44e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact_Ranking" sheetId="7" r:id="R7dfdf2f6325c4a84"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -345,7 +345,7 @@
         <x:color rgb="FF246B3C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -600,7 +600,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6120d88870c64beb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R93e42202a1074286"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -630,7 +630,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ccacba2ce5c40fc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R843c366bb7024664"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -981,7 +981,7 @@
         <x:v>Sample</x:v>
       </x:c>
       <x:c r="B7" s="42" t="str">
-        <x:v>Purposive pilot of core bridge researchers plus controls; not a population estimate</x:v>
+        <x:v>Purposive pilot: 57 researchers and 40 papers in separate, non-1:1 tables; papers may have multiple listed researchers and researchers may span multiple papers</x:v>
       </x:c>
       <x:c r="C7" s="42"/>
       <x:c r="D7" s="42"/>
@@ -1009,7 +1009,7 @@
         <x:v>Person class</x:v>
       </x:c>
       <x:c r="B9" s="42" t="str">
-        <x:v>Switcher / Bridger / Native hybrid / Robotics-first; migration is not reduced to one binary label</x:v>
+        <x:v>Switcher 2 / Bridger 42 / Native hybrid 11 / Robotics-first 2 = 57</x:v>
       </x:c>
       <x:c r="C9" s="42"/>
       <x:c r="D9" s="42"/>
@@ -1023,7 +1023,7 @@
         <x:v>Video axis</x:v>
       </x:c>
       <x:c r="B10" s="42" t="str">
-        <x:v>G1–G3 generation is structurally separated from U1–U3 understanding/predictive representation and VL</x:v>
+        <x:v>G1-G3 are separated by output: G2 may take actions as conditions but outputs future video/state; G3 outputs video/future state and actions jointly; A outputs actions only</x:v>
       </x:c>
       <x:c r="C10" s="42"/>
       <x:c r="D10" s="42"/>
@@ -1079,7 +1079,7 @@
         <x:v>Researcher ordering</x:v>
       </x:c>
       <x:c r="B14" s="42" t="str">
-        <x:v>Important in both fields first; then geometric mean of selected video/robotics citations, with Medium evidence ×0.8</x:v>
+        <x:v>Important_both researchers are placed first, then ranked within that selected intersection by the geometric mean of representative video/robotics citations; Medium evidence x0.8</x:v>
       </x:c>
       <x:c r="C14" s="42"/>
       <x:c r="D14" s="42"/>
@@ -1093,7 +1093,7 @@
         <x:v>Limit</x:v>
       </x:c>
       <x:c r="B15" s="42" t="str">
-        <x:v>Bridge-specific ranking, not total career influence. Missing representative-paper coverage scores 0 and remains visible</x:v>
+        <x:v>Selection-aware bridge ranking, not a field-wide or career-impact ranking. High = direct authorship/project evidence on both sides; Medium = one link is team-level, recent, indirect, or not fully authorship-verified. Citation_coverage is separate</x:v>
       </x:c>
       <x:c r="C15" s="42"/>
       <x:c r="D15" s="42"/>
@@ -1157,7 +1157,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B20" s="47" t="str">
-        <x:v>Report Switcher, Bridger, and Native hybrid separately to avoid under- or over-stating migration.</x:v>
+        <x:v>Report Switcher, Bridger, Native hybrid, and Robotics-first separately to avoid under- or over-stating migration.</x:v>
       </x:c>
       <x:c r="C20" s="47"/>
       <x:c r="D20" s="47"/>
@@ -1295,7 +1295,7 @@
         <x:v>May have no robot-action conditioning</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="6" ht="43.5" hidden="0" customHeight="1">
       <x:c r="A6" s="47" t="str">
         <x:v>G2</x:v>
       </x:c>
@@ -1303,7 +1303,7 @@
         <x:v>Generation / Prediction</x:v>
       </x:c>
       <x:c r="C6" s="47" t="str">
-        <x:v>Action-conditioned or future video/state generation</x:v>
+        <x:v>Future video/state generation; actions may condition the input but are not generated</x:v>
       </x:c>
       <x:c r="D6" s="47" t="str">
         <x:v>Visual Foresight, Cosmos-Predict</x:v>
@@ -1312,10 +1312,10 @@
         <x:v>world simulation, planning</x:v>
       </x:c>
       <x:c r="F6" s="47" t="str">
-        <x:v>Separate pixel prediction from 3D-state prediction</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>GameNGen/Genie remain G2: action-conditioned video/world output, not action output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="43.5" hidden="0" customHeight="1">
       <x:c r="A7" s="47" t="str">
         <x:v>G3</x:v>
       </x:c>
@@ -1323,7 +1323,7 @@
         <x:v>Unified generation</x:v>
       </x:c>
       <x:c r="C7" s="47" t="str">
-        <x:v>Joint/shared generation of video and actions</x:v>
+        <x:v>Joint/shared output of video or future state and actions</x:v>
       </x:c>
       <x:c r="D7" s="47" t="str">
         <x:v>GR-2, Cosmos Policy</x:v>
@@ -1332,7 +1332,7 @@
         <x:v>direct policy</x:v>
       </x:c>
       <x:c r="F7" s="47" t="str">
-        <x:v>Do not equate action diffusion with generic video generation</x:v>
+        <x:v>G3 vs A distinguishes output modality/architecture, not the downstream direct-policy role</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1415,7 +1415,7 @@
         <x:v>Separate VLM from VLA</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="12" ht="36" hidden="0" customHeight="1">
       <x:c r="A12" s="47" t="str">
         <x:v>A</x:v>
       </x:c>
@@ -1432,7 +1432,7 @@
         <x:v>direct policy</x:v>
       </x:c>
       <x:c r="F12" s="47" t="str">
-        <x:v>Does not establish video-generation origin</x:v>
+        <x:v>Action-only output; unlike G3, no video/future-state output is jointly generated</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -6637,7 +6637,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf421c5cfafe64da6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7bb7b30adab455c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9219,7 +9219,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb94cd13607ee428a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b0f2d951154f6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9687,7 +9687,7 @@
     <x:mergeCell ref="A19:H19"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5371da53978e4f5b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6b7f1f9ec9d4c64"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Refresh citation snapshot for the video-to-robotics note
</commit_message>
<xml_diff>
--- a/notes/01-video-to-robotics-transition/video_to_robotics_architecture_pilot.xlsx
+++ b/notes/01-video-to-robotics-transition/video_to_robotics_architecture_pilot.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Method" sheetId="1" r:id="Rfd3e101bc0a94b2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="R1f0be2ae35884412"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Researchers" sheetId="3" r:id="R4b82c5717e9b4e9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="4" r:id="R61446d792be84fc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="Rec16dd58e7cd4b20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Matrix" sheetId="6" r:id="R28f861bec5ae4df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact_Ranking" sheetId="7" r:id="R609b629f93db4292"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Method" sheetId="1" r:id="R065d8736aa614280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="R2450fe03ee614e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Researchers" sheetId="3" r:id="Ra5ff92658d8c4aa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="4" r:id="R1838e6bc70874096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R71a115705acf4163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Matrix" sheetId="6" r:id="Re92bf41d39134994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact_Ranking" sheetId="7" r:id="R78f419c53ec14869"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -618,7 +618,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4c1f1479cd514e5a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a120482da1e4cb0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -648,7 +648,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf76b3f6e73044ed1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2e2ec02756da4672"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -985,7 +985,7 @@
         <x:v>As of</x:v>
       </x:c>
       <x:c r="B6" s="47" t="str">
-        <x:v>2026-09-02 revision; original citation snapshot 2026-08-30, added G2 audit rows 2026-09-02</x:v>
+        <x:v>2026-09-02 citation snapshot; all 55 paper rows rechecked on the same date</x:v>
       </x:c>
       <x:c r="C6" s="42"/>
       <x:c r="D6" s="42"/>
@@ -1083,7 +1083,7 @@
         <x:v>Citation basis</x:v>
       </x:c>
       <x:c r="B13" s="47" t="str">
-        <x:v>Observed scholarly-web-index counts; original rows as of 2026-08-30 and added G2 audit rows as of 2026-09-02; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index counts rechecked on 2026-09-02; title and paper identity were matched, and version-split decreases were not substituted</x:v>
       </x:c>
       <x:c r="C13" s="42"/>
       <x:c r="D13" s="42"/>
@@ -1778,7 +1778,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB2" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1866,7 +1866,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB3" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1954,7 +1954,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB4" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2042,7 +2042,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB5" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2130,7 +2130,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB6" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2218,7 +2218,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB7" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2306,7 +2306,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB8" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2394,7 +2394,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB9" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2482,7 +2482,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB10" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2559,18 +2559,18 @@
         <x:v>P019</x:v>
       </x:c>
       <x:c r="Y11" s="50" t="n">
-        <x:v>827</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="Z11" s="51" t="n">
         <x:f>IF(OR(N11&lt;&gt;"Yes",AA11&lt;&gt;"Both selected papers covered"),"",SQRT((W11+1)*(Y11+1))*IF(Q11="High",1,0.8))</x:f>
-        <x:v>671.7588853152595</x:v>
+        <x:v>674.5924695695913</x:v>
       </x:c>
       <x:c r="AA11" s="47" t="str">
         <x:f>IF(AND(V11&lt;&gt;"",ISNUMBER(W11),X11&lt;&gt;"",ISNUMBER(Y11),COUNTIF('Papers'!$C$2:$C$56,V11)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X11)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB11" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2658,7 +2658,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB12" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2729,7 +2729,7 @@
         <x:v>P003</x:v>
       </x:c>
       <x:c r="W13" s="50" t="n">
-        <x:v>554</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="X13" s="47" t="str">
         <x:v>P004</x:v>
@@ -2739,14 +2739,14 @@
       </x:c>
       <x:c r="Z13" s="51" t="n">
         <x:f>IF(OR(N13&lt;&gt;"Yes",AA13&lt;&gt;"Both selected papers covered"),"",SQRT((W13+1)*(Y13+1))*IF(Q13="High",1,0.8))</x:f>
-        <x:v>620.6206570845028</x:v>
+        <x:v>625.6324799752647</x:v>
       </x:c>
       <x:c r="AA13" s="47" t="str">
         <x:f>IF(AND(V13&lt;&gt;"",ISNUMBER(W13),X13&lt;&gt;"",ISNUMBER(Y13),COUNTIF('Papers'!$C$2:$C$56,V13)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X13)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB13" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2817,7 +2817,7 @@
         <x:v>P003</x:v>
       </x:c>
       <x:c r="W14" s="50" t="n">
-        <x:v>554</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="X14" s="47" t="str">
         <x:v>P004</x:v>
@@ -2827,14 +2827,14 @@
       </x:c>
       <x:c r="Z14" s="51" t="n">
         <x:f>IF(OR(N14&lt;&gt;"Yes",AA14&lt;&gt;"Both selected papers covered"),"",SQRT((W14+1)*(Y14+1))*IF(Q14="High",1,0.8))</x:f>
-        <x:v>620.6206570845028</x:v>
+        <x:v>625.6324799752647</x:v>
       </x:c>
       <x:c r="AA14" s="47" t="str">
         <x:f>IF(AND(V14&lt;&gt;"",ISNUMBER(W14),X14&lt;&gt;"",ISNUMBER(Y14),COUNTIF('Papers'!$C$2:$C$56,V14)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X14)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB14" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2905,7 +2905,7 @@
         <x:v>P003</x:v>
       </x:c>
       <x:c r="W15" s="50" t="n">
-        <x:v>554</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="X15" s="47" t="str">
         <x:v>P004</x:v>
@@ -2915,14 +2915,14 @@
       </x:c>
       <x:c r="Z15" s="51" t="n">
         <x:f>IF(OR(N15&lt;&gt;"Yes",AA15&lt;&gt;"Both selected papers covered"),"",SQRT((W15+1)*(Y15+1))*IF(Q15="High",1,0.8))</x:f>
-        <x:v>620.6206570845028</x:v>
+        <x:v>625.6324799752647</x:v>
       </x:c>
       <x:c r="AA15" s="47" t="str">
         <x:f>IF(AND(V15&lt;&gt;"",ISNUMBER(W15),X15&lt;&gt;"",ISNUMBER(Y15),COUNTIF('Papers'!$C$2:$C$56,V15)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X15)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB15" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2993,7 +2993,7 @@
         <x:v>P003</x:v>
       </x:c>
       <x:c r="W16" s="50" t="n">
-        <x:v>554</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="X16" s="47" t="str">
         <x:v>P004</x:v>
@@ -3003,14 +3003,14 @@
       </x:c>
       <x:c r="Z16" s="51" t="n">
         <x:f>IF(OR(N16&lt;&gt;"Yes",AA16&lt;&gt;"Both selected papers covered"),"",SQRT((W16+1)*(Y16+1))*IF(Q16="High",1,0.8))</x:f>
-        <x:v>620.6206570845028</x:v>
+        <x:v>625.6324799752647</x:v>
       </x:c>
       <x:c r="AA16" s="47" t="str">
         <x:f>IF(AND(V16&lt;&gt;"",ISNUMBER(W16),X16&lt;&gt;"",ISNUMBER(Y16),COUNTIF('Papers'!$C$2:$C$56,V16)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X16)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB16" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -3081,7 +3081,7 @@
         <x:v>P003</x:v>
       </x:c>
       <x:c r="W17" s="50" t="n">
-        <x:v>554</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="X17" s="47" t="str">
         <x:v>P004</x:v>
@@ -3091,14 +3091,14 @@
       </x:c>
       <x:c r="Z17" s="51" t="n">
         <x:f>IF(OR(N17&lt;&gt;"Yes",AA17&lt;&gt;"Both selected papers covered"),"",SQRT((W17+1)*(Y17+1))*IF(Q17="High",1,0.8))</x:f>
-        <x:v>620.6206570845028</x:v>
+        <x:v>625.6324799752647</x:v>
       </x:c>
       <x:c r="AA17" s="47" t="str">
         <x:f>IF(AND(V17&lt;&gt;"",ISNUMBER(W17),X17&lt;&gt;"",ISNUMBER(Y17),COUNTIF('Papers'!$C$2:$C$56,V17)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X17)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB17" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3169,24 +3169,24 @@
         <x:v>P001</x:v>
       </x:c>
       <x:c r="W18" s="50" t="n">
-        <x:v>388</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="X18" s="47" t="str">
         <x:v>P019</x:v>
       </x:c>
       <x:c r="Y18" s="50" t="n">
-        <x:v>827</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="Z18" s="51" t="n">
         <x:f>IF(OR(N18&lt;&gt;"Yes",AA18&lt;&gt;"Both selected papers covered"),"",SQRT((W18+1)*(Y18+1))*IF(Q18="High",1,0.8))</x:f>
-        <x:v>567.5314969232985</x:v>
+        <x:v>572.1188687676714</x:v>
       </x:c>
       <x:c r="AA18" s="47" t="str">
         <x:f>IF(AND(V18&lt;&gt;"",ISNUMBER(W18),X18&lt;&gt;"",ISNUMBER(Y18),COUNTIF('Papers'!$C$2:$C$56,V18)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X18)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB18" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3257,24 +3257,24 @@
         <x:v>P001</x:v>
       </x:c>
       <x:c r="W19" s="50" t="n">
-        <x:v>388</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="X19" s="47" t="str">
         <x:v>P019</x:v>
       </x:c>
       <x:c r="Y19" s="50" t="n">
-        <x:v>827</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="Z19" s="51" t="n">
         <x:f>IF(OR(N19&lt;&gt;"Yes",AA19&lt;&gt;"Both selected papers covered"),"",SQRT((W19+1)*(Y19+1))*IF(Q19="High",1,0.8))</x:f>
-        <x:v>567.5314969232985</x:v>
+        <x:v>572.1188687676714</x:v>
       </x:c>
       <x:c r="AA19" s="47" t="str">
         <x:f>IF(AND(V19&lt;&gt;"",ISNUMBER(W19),X19&lt;&gt;"",ISNUMBER(Y19),COUNTIF('Papers'!$C$2:$C$56,V19)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X19)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB19" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -3362,7 +3362,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB20" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -3450,7 +3450,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB21" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -3538,7 +3538,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB22" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -3626,7 +3626,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB23" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -3703,18 +3703,18 @@
         <x:v>P012</x:v>
       </x:c>
       <x:c r="Y24" s="50" t="n">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="Z24" s="51" t="n">
         <x:f>IF(OR(N24&lt;&gt;"Yes",AA24&lt;&gt;"Both selected papers covered"),"",SQRT((W24+1)*(Y24+1))*IF(Q24="High",1,0.8))</x:f>
-        <x:v>374.0588189041932</x:v>
+        <x:v>374.9399951992319</x:v>
       </x:c>
       <x:c r="AA24" s="47" t="str">
         <x:f>IF(AND(V24&lt;&gt;"",ISNUMBER(W24),X24&lt;&gt;"",ISNUMBER(Y24),COUNTIF('Papers'!$C$2:$C$56,V24)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X24)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB24" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -3802,7 +3802,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB25" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -3890,7 +3890,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB26" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -3978,7 +3978,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB27" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -4049,24 +4049,24 @@
         <x:v>P012</x:v>
       </x:c>
       <x:c r="W28" s="50" t="n">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="X28" s="47" t="str">
         <x:v>P012</x:v>
       </x:c>
       <x:c r="Y28" s="50" t="n">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="Z28" s="51" t="n">
         <x:f>IF(OR(N28&lt;&gt;"Yes",AA28&lt;&gt;"Both selected papers covered"),"",SQRT((W28+1)*(Y28+1))*IF(Q28="High",1,0.8))</x:f>
-        <x:v>212</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="AA28" s="47" t="str">
         <x:f>IF(AND(V28&lt;&gt;"",ISNUMBER(W28),X28&lt;&gt;"",ISNUMBER(Y28),COUNTIF('Papers'!$C$2:$C$56,V28)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X28)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB28" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -4154,7 +4154,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB29" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -4225,24 +4225,24 @@
         <x:v>P014</x:v>
       </x:c>
       <x:c r="W30" s="50" t="n">
-        <x:v>161</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="X30" s="47" t="str">
         <x:v>P014</x:v>
       </x:c>
       <x:c r="Y30" s="50" t="n">
-        <x:v>161</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="Z30" s="51" t="n">
         <x:f>IF(OR(N30&lt;&gt;"Yes",AA30&lt;&gt;"Both selected papers covered"),"",SQRT((W30+1)*(Y30+1))*IF(Q30="High",1,0.8))</x:f>
-        <x:v>162</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="AA30" s="47" t="str">
         <x:f>IF(AND(V30&lt;&gt;"",ISNUMBER(W30),X30&lt;&gt;"",ISNUMBER(Y30),COUNTIF('Papers'!$C$2:$C$56,V30)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X30)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB30" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -4330,7 +4330,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB31" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -4418,7 +4418,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB32" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -4495,22 +4495,22 @@
         <x:v>P026</x:v>
       </x:c>
       <x:c r="Y33" s="50" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="Z33" s="51" t="n">
         <x:f>IF(OR(N33&lt;&gt;"Yes",AA33&lt;&gt;"Both selected papers covered"),"",SQRT((W33+1)*(Y33+1))*IF(Q33="High",1,0.8))</x:f>
-        <x:v>12.569805089976535</x:v>
+        <x:v>37.70941526992961</x:v>
       </x:c>
       <x:c r="AA33" s="47" t="str">
         <x:f>IF(AND(V33&lt;&gt;"",ISNUMBER(W33),X33&lt;&gt;"",ISNUMBER(Y33),COUNTIF('Papers'!$C$2:$C$56,V33)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X33)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB33" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="50" t="str"/>
+      <x:c r="A34" s="50"/>
       <x:c r="B34" s="47" t="str">
         <x:v>R048</x:v>
       </x:c>
@@ -4575,7 +4575,7 @@
         <x:v>P033</x:v>
       </x:c>
       <x:c r="W34" s="50" t="n">
-        <x:v>716</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="X34" s="47"/>
       <x:c r="Y34" s="50"/>
@@ -4587,11 +4587,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB34" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="50" t="str"/>
+      <x:c r="A35" s="50"/>
       <x:c r="B35" s="47" t="str">
         <x:v>R006</x:v>
       </x:c>
@@ -4662,7 +4662,7 @@
         <x:v>P027</x:v>
       </x:c>
       <x:c r="Y35" s="50" t="n">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="Z35" s="51" t="str">
         <x:f>IF(OR(N35&lt;&gt;"Yes",AA35&lt;&gt;"Both selected papers covered"),"",SQRT((W35+1)*(Y35+1))*IF(Q35="High",1,0.8))</x:f>
@@ -4672,11 +4672,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB35" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="50" t="str"/>
+      <x:c r="A36" s="50"/>
       <x:c r="B36" s="47" t="str">
         <x:v>R047</x:v>
       </x:c>
@@ -4741,7 +4741,7 @@
         <x:v>P033</x:v>
       </x:c>
       <x:c r="W36" s="50" t="n">
-        <x:v>716</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="X36" s="47"/>
       <x:c r="Y36" s="50"/>
@@ -4753,11 +4753,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB36" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="50" t="str"/>
+      <x:c r="A37" s="50"/>
       <x:c r="B37" s="47" t="str">
         <x:v>R032</x:v>
       </x:c>
@@ -4830,11 +4830,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB37" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="50" t="str"/>
+      <x:c r="A38" s="50"/>
       <x:c r="B38" s="47" t="str">
         <x:v>R044</x:v>
       </x:c>
@@ -4915,11 +4915,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB38" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="50" t="str"/>
+      <x:c r="A39" s="50"/>
       <x:c r="B39" s="47" t="str">
         <x:v>R007</x:v>
       </x:c>
@@ -5000,11 +5000,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB39" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="50" t="str"/>
+      <x:c r="A40" s="50"/>
       <x:c r="B40" s="47" t="str">
         <x:v>R003</x:v>
       </x:c>
@@ -5069,7 +5069,7 @@
         <x:v>P001</x:v>
       </x:c>
       <x:c r="W40" s="50" t="n">
-        <x:v>388</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="X40" s="47"/>
       <x:c r="Y40" s="50"/>
@@ -5081,11 +5081,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB40" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="50" t="str"/>
+      <x:c r="A41" s="50"/>
       <x:c r="B41" s="47" t="str">
         <x:v>R041</x:v>
       </x:c>
@@ -5150,13 +5150,13 @@
         <x:v>P026</x:v>
       </x:c>
       <x:c r="W41" s="50" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X41" s="47" t="str">
         <x:v>P026</x:v>
       </x:c>
       <x:c r="Y41" s="50" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="Z41" s="51" t="str">
         <x:f>IF(OR(N41&lt;&gt;"Yes",AA41&lt;&gt;"Both selected papers covered"),"",SQRT((W41+1)*(Y41+1))*IF(Q41="High",1,0.8))</x:f>
@@ -5166,11 +5166,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB41" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="50" t="str"/>
+      <x:c r="A42" s="50"/>
       <x:c r="B42" s="47" t="str">
         <x:v>R038</x:v>
       </x:c>
@@ -5247,11 +5247,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB42" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="50" t="str"/>
+      <x:c r="A43" s="50"/>
       <x:c r="B43" s="47" t="str">
         <x:v>R002</x:v>
       </x:c>
@@ -5316,7 +5316,7 @@
         <x:v>P001</x:v>
       </x:c>
       <x:c r="W43" s="50" t="n">
-        <x:v>388</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="X43" s="47"/>
       <x:c r="Y43" s="50"/>
@@ -5328,11 +5328,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB43" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="50" t="str"/>
+      <x:c r="A44" s="50"/>
       <x:c r="B44" s="47" t="str">
         <x:v>R027</x:v>
       </x:c>
@@ -5397,7 +5397,7 @@
         <x:v>P008</x:v>
       </x:c>
       <x:c r="W44" s="50" t="n">
-        <x:v>758</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="X44" s="47" t="str">
         <x:v>P010</x:v>
@@ -5413,11 +5413,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB44" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="50" t="str"/>
+      <x:c r="A45" s="50"/>
       <x:c r="B45" s="47" t="str">
         <x:v>R021</x:v>
       </x:c>
@@ -5498,11 +5498,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB45" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="50" t="str"/>
+      <x:c r="A46" s="50"/>
       <x:c r="B46" s="47" t="str">
         <x:v>R050</x:v>
       </x:c>
@@ -5575,11 +5575,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB46" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="50" t="str"/>
+      <x:c r="A47" s="50"/>
       <x:c r="B47" s="47" t="str">
         <x:v>R045</x:v>
       </x:c>
@@ -5660,11 +5660,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB47" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="50" t="str"/>
+      <x:c r="A48" s="50"/>
       <x:c r="B48" s="47" t="str">
         <x:v>R039</x:v>
       </x:c>
@@ -5729,13 +5729,13 @@
         <x:v>P026</x:v>
       </x:c>
       <x:c r="W48" s="50" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X48" s="47" t="str">
         <x:v>P026</x:v>
       </x:c>
       <x:c r="Y48" s="50" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="Z48" s="51" t="str">
         <x:f>IF(OR(N48&lt;&gt;"Yes",AA48&lt;&gt;"Both selected papers covered"),"",SQRT((W48+1)*(Y48+1))*IF(Q48="High",1,0.8))</x:f>
@@ -5745,11 +5745,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB48" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="50" t="str"/>
+      <x:c r="A49" s="50"/>
       <x:c r="B49" s="47" t="str">
         <x:v>R051</x:v>
       </x:c>
@@ -5813,24 +5813,28 @@
       <x:c r="V49" s="47" t="str">
         <x:v>P032</x:v>
       </x:c>
-      <x:c r="W49" s="50"/>
+      <x:c r="W49" s="50" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="X49" s="47" t="str">
         <x:v>P032</x:v>
       </x:c>
-      <x:c r="Y49" s="50"/>
+      <x:c r="Y49" s="50" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="Z49" s="51" t="str">
         <x:f>IF(OR(N49&lt;&gt;"Yes",AA49&lt;&gt;"Both selected papers covered"),"",SQRT((W49+1)*(Y49+1))*IF(Q49="High",1,0.8))</x:f>
       </x:c>
       <x:c r="AA49" s="47" t="str">
         <x:f>IF(AND(V49&lt;&gt;"",ISNUMBER(W49),X49&lt;&gt;"",ISNUMBER(Y49),COUNTIF('Papers'!$C$2:$C$56,V49)&gt;0,COUNTIF('Papers'!$C$2:$C$56,X49)&gt;0),"Both selected papers covered","Partial / missing selected-paper coverage")</x:f>
-        <x:v>Partial / missing selected-paper coverage</x:v>
+        <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB49" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="50" t="str"/>
+      <x:c r="A50" s="50"/>
       <x:c r="B50" s="47" t="str">
         <x:v>R037</x:v>
       </x:c>
@@ -5911,11 +5915,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB50" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="50" t="str"/>
+      <x:c r="A51" s="50"/>
       <x:c r="B51" s="47" t="str">
         <x:v>R052</x:v>
       </x:c>
@@ -5988,11 +5992,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB51" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="50" t="str"/>
+      <x:c r="A52" s="50"/>
       <x:c r="B52" s="47" t="str">
         <x:v>R040</x:v>
       </x:c>
@@ -6057,13 +6061,13 @@
         <x:v>P026</x:v>
       </x:c>
       <x:c r="W52" s="50" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X52" s="47" t="str">
         <x:v>P026</x:v>
       </x:c>
       <x:c r="Y52" s="50" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="Z52" s="51" t="str">
         <x:f>IF(OR(N52&lt;&gt;"Yes",AA52&lt;&gt;"Both selected papers covered"),"",SQRT((W52+1)*(Y52+1))*IF(Q52="High",1,0.8))</x:f>
@@ -6073,11 +6077,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB52" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="50" t="str"/>
+      <x:c r="A53" s="50"/>
       <x:c r="B53" s="47" t="str">
         <x:v>R030</x:v>
       </x:c>
@@ -6150,11 +6154,11 @@
         <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB53" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="50" t="str"/>
+      <x:c r="A54" s="50"/>
       <x:c r="B54" s="47" t="str">
         <x:v>R019</x:v>
       </x:c>
@@ -6235,11 +6239,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB54" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="50" t="str"/>
+      <x:c r="A55" s="50"/>
       <x:c r="B55" s="47" t="str">
         <x:v>R023</x:v>
       </x:c>
@@ -6320,11 +6324,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB55" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="50" t="str"/>
+      <x:c r="A56" s="50"/>
       <x:c r="B56" s="47" t="str">
         <x:v>R056</x:v>
       </x:c>
@@ -6389,13 +6393,13 @@
         <x:v>P019</x:v>
       </x:c>
       <x:c r="W56" s="50" t="n">
-        <x:v>827</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="X56" s="47" t="str">
         <x:v>P019</x:v>
       </x:c>
       <x:c r="Y56" s="50" t="n">
-        <x:v>827</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="Z56" s="51" t="str">
         <x:f>IF(OR(N56&lt;&gt;"Yes",AA56&lt;&gt;"Both selected papers covered"),"",SQRT((W56+1)*(Y56+1))*IF(Q56="High",1,0.8))</x:f>
@@ -6405,11 +6409,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB56" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="50" t="str"/>
+      <x:c r="A57" s="50"/>
       <x:c r="B57" s="47" t="str">
         <x:v>R054</x:v>
       </x:c>
@@ -6474,13 +6478,13 @@
         <x:v>P019</x:v>
       </x:c>
       <x:c r="W57" s="50" t="n">
-        <x:v>827</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="X57" s="47" t="str">
         <x:v>P019</x:v>
       </x:c>
       <x:c r="Y57" s="50" t="n">
-        <x:v>827</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="Z57" s="51" t="str">
         <x:f>IF(OR(N57&lt;&gt;"Yes",AA57&lt;&gt;"Both selected papers covered"),"",SQRT((W57+1)*(Y57+1))*IF(Q57="High",1,0.8))</x:f>
@@ -6490,11 +6494,11 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB57" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="50" t="str"/>
+      <x:c r="A58" s="50"/>
       <x:c r="B58" s="47" t="str">
         <x:v>R022</x:v>
       </x:c>
@@ -6575,7 +6579,7 @@
         <x:v>Both selected papers covered</x:v>
       </x:c>
       <x:c r="AB58" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6584,7 +6588,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bd393b946ff4733"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978df3d9322548a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6724,19 +6728,20 @@
         <x:v>Video embeddings transferred across demonstrations and robots</x:v>
       </x:c>
       <x:c r="P2" s="51" t="n">
-        <x:v>1358</x:v>
+        <x:v>1359</x:v>
       </x:c>
       <x:c r="Q2" s="51" t="n">
-        <x:v>135.8</x:v>
+        <x:f>IF(P2="","",P2/MAX(1,2026-E2+1))</x:f>
+        <x:v>135.9</x:v>
       </x:c>
       <x:c r="R2" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S2" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Time-Contrastive%20Networks%3A%20Self-Supervised%20Learning%20from%20Video</x:v>
       </x:c>
       <x:c r="T2" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -6789,16 +6794,17 @@
         <x:v>1130</x:v>
       </x:c>
       <x:c r="Q3" s="51" t="n">
+        <x:f>IF(P3="","",P3/MAX(1,2026-E3+1))</x:f>
         <x:v>102.72727272727273</x:v>
       </x:c>
       <x:c r="R3" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S3" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Deep%20Visual%20Foresight%20for%20Planning%20Robot%20Motion</x:v>
       </x:c>
       <x:c r="T3" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
@@ -6848,19 +6854,20 @@
         <x:v>Important prompt-conditioned robot policy</x:v>
       </x:c>
       <x:c r="P4" s="51" t="n">
-        <x:v>827</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="Q4" s="51" t="n">
-        <x:v>206.75</x:v>
+        <x:f>IF(P4="","",P4/MAX(1,2026-E4+1))</x:f>
+        <x:v>208.5</x:v>
       </x:c>
       <x:c r="R4" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S4" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=VIMA%3A%20General%20Robot%20Manipulation%20with%20Multimodal%20Prompts</x:v>
       </x:c>
       <x:c r="T4" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
@@ -6913,16 +6920,17 @@
         <x:v>740</x:v>
       </x:c>
       <x:c r="Q5" s="51" t="n">
+        <x:f>IF(P5="","",P5/MAX(1,2026-E5+1))</x:f>
         <x:v>370</x:v>
       </x:c>
       <x:c r="R5" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S5" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Cosmos%20World%20Foundation%20Model%20Platform%20for%20Physical%20AI</x:v>
       </x:c>
       <x:c r="T5" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -6975,16 +6983,17 @@
         <x:v>693</x:v>
       </x:c>
       <x:c r="Q6" s="51" t="n">
+        <x:f>IF(P6="","",P6/MAX(1,2026-E6+1))</x:f>
         <x:v>346.5</x:v>
       </x:c>
       <x:c r="R6" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S6" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=V-JEPA%202%3A%20Self-Supervised%20Video%20Models%20Enable%20Understanding%2C%20Prediction%20and%20Planning</x:v>
       </x:c>
       <x:c r="T6" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -7037,16 +7046,17 @@
         <x:v>659</x:v>
       </x:c>
       <x:c r="Q7" s="51" t="n">
+        <x:f>IF(P7="","",P7/MAX(1,2026-E7+1))</x:f>
         <x:v>164.75</x:v>
       </x:c>
       <x:c r="R7" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S7" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=UniPi%3A%20Learning%20Universal%20Policies%20via%20Text-Guided%20Video%20Generation</x:v>
       </x:c>
       <x:c r="T7" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -7099,16 +7109,17 @@
         <x:v>544</x:v>
       </x:c>
       <x:c r="Q8" s="51" t="n">
+        <x:f>IF(P8="","",P8/MAX(1,2026-E8+1))</x:f>
         <x:v>108.8</x:v>
       </x:c>
       <x:c r="R8" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S8" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=MineDojo%3A%20Building%20Open-Ended%20Embodied%20Agents%20with%20Internet-Scale%20Knowledge</x:v>
       </x:c>
       <x:c r="T8" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -7161,10 +7172,11 @@
         <x:v>448</x:v>
       </x:c>
       <x:c r="Q9" s="51" t="n">
+        <x:f>IF(P9="","",P9/MAX(1,2026-E9+1))</x:f>
         <x:v>112</x:v>
       </x:c>
       <x:c r="R9" s="47" t="str">
-        <x:v>Observed scholarly web index; added during G2 audit; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S9" s="47" t="str">
         <x:v>https://arxiv.org/abs/2310.06114</x:v>
@@ -7223,16 +7235,17 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="Q10" s="51" t="n">
+        <x:f>IF(P10="","",P10/MAX(1,2026-E10+1))</x:f>
         <x:v>55.5</x:v>
       </x:c>
       <x:c r="R10" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S10" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=RoboNet%3A%20Large-Scale%20Multi-Robot%20Learning</x:v>
       </x:c>
       <x:c r="T10" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
@@ -7282,19 +7295,20 @@
         <x:v>Pretrains video generation then predicts actions and videos</x:v>
       </x:c>
       <x:c r="P11" s="51" t="n">
-        <x:v>294</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="Q11" s="51" t="n">
-        <x:v>98</x:v>
+        <x:f>IF(P11="","",P11/MAX(1,2026-E11+1))</x:f>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="R11" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S11" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=GR-2%3A%20A%20Generative%20Video-Language-Action%20Model%20with%20Web-Scale%20Knowledge%20for%20Robot%20Manipulation</x:v>
       </x:c>
       <x:c r="T11" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
@@ -7347,16 +7361,17 @@
         <x:v>251</x:v>
       </x:c>
       <x:c r="Q12" s="51" t="n">
+        <x:f>IF(P12="","",P12/MAX(1,2026-E12+1))</x:f>
         <x:v>50.2</x:v>
       </x:c>
       <x:c r="R12" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S12" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=WHIRL%3A%20Human-to-Robot%20Imitation%20in%20the%20Wild</x:v>
       </x:c>
       <x:c r="T12" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -7406,19 +7421,20 @@
         <x:v>Compositional video world model for robot planning</x:v>
       </x:c>
       <x:c r="P13" s="51" t="n">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="Q13" s="51" t="n">
-        <x:v>70.33333333333333</x:v>
+        <x:f>IF(P13="","",P13/MAX(1,2026-E13+1))</x:f>
+        <x:v>70.66666666666667</x:v>
       </x:c>
       <x:c r="R13" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S13" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=RoboDreamer%3A%20Learning%20Compositional%20World%20Models%20for%20Robot%20Imagination</x:v>
       </x:c>
       <x:c r="T13" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -7471,16 +7487,17 @@
         <x:v>193</x:v>
       </x:c>
       <x:c r="Q14" s="51" t="n">
+        <x:f>IF(P14="","",P14/MAX(1,2026-E14+1))</x:f>
         <x:v>193</x:v>
       </x:c>
       <x:c r="R14" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S14" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Cosmos%20Policy%3A%20Fine-Tuning%20Video%20Models%20for%20Visuomotor%20Control%20and%20Planning</x:v>
       </x:c>
       <x:c r="T14" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -7533,16 +7550,17 @@
         <x:v>189</x:v>
       </x:c>
       <x:c r="Q15" s="51" t="n">
+        <x:f>IF(P15="","",P15/MAX(1,2026-E15+1))</x:f>
         <x:v>94.5</x:v>
       </x:c>
       <x:c r="R15" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S15" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Magma%3A%20A%20Foundation%20Model%20for%20Multimodal%20AI%20Agents</x:v>
       </x:c>
       <x:c r="T15" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
@@ -7553,10 +7571,10 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C16" s="64" t="str">
-        <x:v>P042</x:v>
+        <x:v>P014</x:v>
       </x:c>
       <x:c r="D16" s="47" t="str">
-        <x:v>iVideoGPT: Interactive VideoGPTs are Scalable World Models</x:v>
+        <x:v>Gen2Act: Human Video Generation in Novel Scenarios enables Generalizable Robot Manipulation</x:v>
       </x:c>
       <x:c r="E16" s="63" t="n">
         <x:v>2024</x:v>
@@ -7565,13 +7583,13 @@
         <x:v>Bridge</x:v>
       </x:c>
       <x:c r="G16" s="47" t="str">
-        <x:v>G2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="H16" s="47" t="str">
-        <x:v>Action-conditioned video, action, and reward tokens</x:v>
+        <x:v>Generated human video</x:v>
       </x:c>
       <x:c r="I16" s="47" t="str">
-        <x:v>Planning</x:v>
+        <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="J16" s="47" t="str">
         <x:v>Major</x:v>
@@ -7580,28 +7598,29 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="L16" s="47" t="str">
-        <x:v>Asia</x:v>
+        <x:v>US</x:v>
       </x:c>
       <x:c r="M16" s="47" t="str">
-        <x:v>Jialong Wu; Shaofeng Yin; Ningya Feng; Xu He; Dong Li; Jianye Hao; Mingsheng Long</x:v>
+        <x:v>Authors per paper</x:v>
       </x:c>
       <x:c r="N16" s="47" t="str">
-        <x:v>https://arxiv.org/abs/2405.15223</x:v>
+        <x:v>https://arxiv.org/abs/2409.16283</x:v>
       </x:c>
       <x:c r="O16" s="47" t="str">
-        <x:v>Pretrained on large-scale human and robot manipulation video, then adapted to visual planning and model-based RL</x:v>
+        <x:v>Generated videos supervise robot actions</x:v>
       </x:c>
       <x:c r="P16" s="51" t="n">
-        <x:v>181</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="Q16" s="51" t="n">
-        <x:v>60.333333333333336</x:v>
+        <x:f>IF(P16="","",P16/MAX(1,2026-E16+1))</x:f>
+        <x:v>61.333333333333336</x:v>
       </x:c>
       <x:c r="R16" s="47" t="str">
-        <x:v>Observed scholarly web index; added during G2 audit; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S16" s="47" t="str">
-        <x:v>https://openreview.net/forum?id=4TENzBftZR</x:v>
+        <x:v>https://www.semanticscholar.org/search?q=Gen2Act%3A%20Human%20Video%20Generation%20in%20Novel%20Scenarios%20enables%20Generalizable%20Robot%20Manipulation</x:v>
       </x:c>
       <x:c r="T16" s="52" t="str">
         <x:v>2026-09-02</x:v>
@@ -7615,10 +7634,10 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C17" s="64" t="str">
-        <x:v>P014</x:v>
+        <x:v>P042</x:v>
       </x:c>
       <x:c r="D17" s="47" t="str">
-        <x:v>Gen2Act: Human Video Generation in Novel Scenarios enables Generalizable Robot Manipulation</x:v>
+        <x:v>iVideoGPT: Interactive VideoGPTs are Scalable World Models</x:v>
       </x:c>
       <x:c r="E17" s="63" t="n">
         <x:v>2024</x:v>
@@ -7627,13 +7646,13 @@
         <x:v>Bridge</x:v>
       </x:c>
       <x:c r="G17" s="47" t="str">
-        <x:v>G1</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="H17" s="47" t="str">
-        <x:v>Generated human video</x:v>
+        <x:v>Action-conditioned video, action, and reward tokens</x:v>
       </x:c>
       <x:c r="I17" s="47" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>Planning</x:v>
       </x:c>
       <x:c r="J17" s="47" t="str">
         <x:v>Major</x:v>
@@ -7642,31 +7661,32 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="L17" s="47" t="str">
-        <x:v>US</x:v>
+        <x:v>Asia</x:v>
       </x:c>
       <x:c r="M17" s="47" t="str">
-        <x:v>Authors per paper</x:v>
+        <x:v>Jialong Wu; Shaofeng Yin; Ningya Feng; Xu He; Dong Li; Jianye Hao; Mingsheng Long</x:v>
       </x:c>
       <x:c r="N17" s="47" t="str">
-        <x:v>https://arxiv.org/abs/2409.16283</x:v>
+        <x:v>https://arxiv.org/abs/2405.15223</x:v>
       </x:c>
       <x:c r="O17" s="47" t="str">
-        <x:v>Generated videos supervise robot actions</x:v>
+        <x:v>Pretrained on large-scale human and robot manipulation video, then adapted to visual planning and model-based RL</x:v>
       </x:c>
       <x:c r="P17" s="51" t="n">
-        <x:v>161</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="Q17" s="51" t="n">
-        <x:v>53.666666666666664</x:v>
+        <x:f>IF(P17="","",P17/MAX(1,2026-E17+1))</x:f>
+        <x:v>60.333333333333336</x:v>
       </x:c>
       <x:c r="R17" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S17" s="47" t="str">
-        <x:v>https://www.semanticscholar.org/search?q=Gen2Act%3A%20Human%20Video%20Generation%20in%20Novel%20Scenarios%20enables%20Generalizable%20Robot%20Manipulation</x:v>
+        <x:v>https://openreview.net/forum?id=4TENzBftZR</x:v>
       </x:c>
       <x:c r="T17" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
@@ -7719,16 +7739,17 @@
         <x:v>161</x:v>
       </x:c>
       <x:c r="Q18" s="51" t="n">
+        <x:f>IF(P18="","",P18/MAX(1,2026-E18+1))</x:f>
         <x:v>40.25</x:v>
       </x:c>
       <x:c r="R18" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S18" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=RoboCat%3A%20A%20Self-Improving%20Generalist%20Agent%20for%20Robotic%20Manipulation</x:v>
       </x:c>
       <x:c r="T18" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
@@ -7781,16 +7802,17 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="Q19" s="51" t="n">
+        <x:f>IF(P19="","",P19/MAX(1,2026-E19+1))</x:f>
         <x:v>20.5</x:v>
       </x:c>
       <x:c r="R19" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S19" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=SuSIE%3A%20Subgoal%20Synthesis%20via%20Image%20Editing</x:v>
       </x:c>
       <x:c r="T19" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
@@ -7801,10 +7823,10 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="C20" s="64" t="str">
-        <x:v>P044</x:v>
+        <x:v>P043</x:v>
       </x:c>
       <x:c r="D20" s="47" t="str">
-        <x:v>Navigation World Models</x:v>
+        <x:v>IRASim: A Fine-Grained World Model for Robot Manipulation</x:v>
       </x:c>
       <x:c r="E20" s="63" t="n">
         <x:v>2024</x:v>
@@ -7816,10 +7838,10 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H20" s="47" t="str">
-        <x:v>Navigation-action-conditioned future video</x:v>
+        <x:v>Robot-action-conditioned future video</x:v>
       </x:c>
       <x:c r="I20" s="47" t="str">
-        <x:v>Planning</x:v>
+        <x:v>World simulation</x:v>
       </x:c>
       <x:c r="J20" s="47" t="str">
         <x:v>Major</x:v>
@@ -7828,28 +7850,29 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="L20" s="47" t="str">
-        <x:v>Mixed</x:v>
+        <x:v>Asia</x:v>
       </x:c>
       <x:c r="M20" s="47" t="str">
-        <x:v>Amir Bar; Gaoyue Zhou; Danny Tran; Trevor Darrell; Yann LeCun</x:v>
+        <x:v>Fangqi Zhu; Hongtao Wu; Song Guo; Yuxiao Liu; Chilam Cheang; Tao Kong</x:v>
       </x:c>
       <x:c r="N20" s="47" t="str">
-        <x:v>https://arxiv.org/abs/2412.03572</x:v>
+        <x:v>https://arxiv.org/abs/2406.14540</x:v>
       </x:c>
       <x:c r="O20" s="47" t="str">
-        <x:v>Controllable video generation used to simulate and rank navigation trajectories for embodied agents</x:v>
+        <x:v>Direct robot manipulation world model with frame-level action conditioning and policy-evaluation use</x:v>
       </x:c>
       <x:c r="P20" s="51" t="n">
         <x:v>70</x:v>
       </x:c>
       <x:c r="Q20" s="51" t="n">
+        <x:f>IF(P20="","",P20/MAX(1,2026-E20+1))</x:f>
         <x:v>23.333333333333332</x:v>
       </x:c>
       <x:c r="R20" s="47" t="str">
-        <x:v>Observed scholarly web index; added during G2 audit; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S20" s="47" t="str">
-        <x:v>https://scholargps.com/scholars/98004081812687/amir-bar</x:v>
+        <x:v>https://arxiv.org/abs/2406.14540</x:v>
       </x:c>
       <x:c r="T20" s="52" t="str">
         <x:v>2026-09-02</x:v>
@@ -7863,58 +7886,59 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C21" s="64" t="str">
-        <x:v>P038</x:v>
+        <x:v>P044</x:v>
       </x:c>
       <x:c r="D21" s="47" t="str">
-        <x:v>PointWorld: Scaling 3D World Models for In-the-Wild Robotic Manipulation</x:v>
+        <x:v>Navigation World Models</x:v>
       </x:c>
       <x:c r="E21" s="63" t="n">
-        <x:v>2026</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="F21" s="47" t="str">
         <x:v>Bridge</x:v>
       </x:c>
       <x:c r="G21" s="47" t="str">
-        <x:v>U2</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="H21" s="47" t="str">
-        <x:v>3D point flows</x:v>
+        <x:v>Navigation-action-conditioned future video</x:v>
       </x:c>
       <x:c r="I21" s="47" t="str">
-        <x:v>World simulation</x:v>
+        <x:v>Planning</x:v>
       </x:c>
       <x:c r="J21" s="47" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Major</x:v>
       </x:c>
       <x:c r="K21" s="47" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="L21" s="47" t="str">
-        <x:v>US</x:v>
+        <x:v>Mixed</x:v>
       </x:c>
       <x:c r="M21" s="47" t="str">
-        <x:v>Wenlong Huang; Yu-Wei Chao; Arsalan Mousavian; Ming-Yu Liu; Dieter Fox; Kaichun Mo; Fei-Fei Li</x:v>
+        <x:v>Amir Bar; Gaoyue Zhou; Danny Tran; Trevor Darrell; Yann LeCun</x:v>
       </x:c>
       <x:c r="N21" s="47" t="str">
-        <x:v>https://arxiv.org/abs/2601.03782</x:v>
+        <x:v>https://arxiv.org/abs/2412.03572</x:v>
       </x:c>
       <x:c r="O21" s="47" t="str">
-        <x:v>Non-pixel predictive world model, useful architecture contrast</x:v>
+        <x:v>Controllable video generation used to simulate and rank navigation trajectories for embodied agents</x:v>
       </x:c>
       <x:c r="P21" s="51" t="n">
-        <x:v>67</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="Q21" s="51" t="n">
-        <x:v>67</x:v>
+        <x:f>IF(P21="","",P21/MAX(1,2026-E21+1))</x:f>
+        <x:v>23.333333333333332</x:v>
       </x:c>
       <x:c r="R21" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S21" s="47" t="str">
-        <x:v>https://www.semanticscholar.org/search?q=PointWorld%3A%20Scaling%203D%20World%20Models%20for%20In-the-Wild%20Robotic%20Manipulation</x:v>
+        <x:v>https://scholargps.com/scholars/98004081812687/amir-bar</x:v>
       </x:c>
       <x:c r="T21" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
@@ -7925,13 +7949,13 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="C22" s="64" t="str">
-        <x:v>P021</x:v>
+        <x:v>P038</x:v>
       </x:c>
       <x:c r="D22" s="47" t="str">
-        <x:v>Vid2Robot: End-to-End Video-Conditioned Policy Learning with Cross-Attention Transformers</x:v>
+        <x:v>PointWorld: Scaling 3D World Models for In-the-Wild Robotic Manipulation</x:v>
       </x:c>
       <x:c r="E22" s="63" t="n">
-        <x:v>2024</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="F22" s="47" t="str">
         <x:v>Bridge</x:v>
@@ -7940,43 +7964,44 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H22" s="47" t="str">
-        <x:v>Video-conditioned action</x:v>
+        <x:v>3D point flows</x:v>
       </x:c>
       <x:c r="I22" s="47" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>World simulation</x:v>
       </x:c>
       <x:c r="J22" s="47" t="str">
-        <x:v>Major</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="K22" s="47" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="L22" s="47" t="str">
-        <x:v>Europe</x:v>
+        <x:v>US</x:v>
       </x:c>
       <x:c r="M22" s="47" t="str">
-        <x:v>Authors per paper; DeepMind Robotics</x:v>
+        <x:v>Wenlong Huang; Yu-Wei Chao; Arsalan Mousavian; Ming-Yu Liu; Dieter Fox; Kaichun Mo; Fei-Fei Li</x:v>
       </x:c>
       <x:c r="N22" s="47" t="str">
-        <x:v>https://arxiv.org/abs/2403.12943</x:v>
+        <x:v>https://arxiv.org/abs/2601.03782</x:v>
       </x:c>
       <x:c r="O22" s="47" t="str">
-        <x:v>Directly produces robot actions from human/robot video prompts</x:v>
+        <x:v>Non-pixel predictive world model, useful architecture contrast</x:v>
       </x:c>
       <x:c r="P22" s="51" t="n">
-        <x:v>65</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="Q22" s="51" t="n">
-        <x:v>21.666666666666668</x:v>
+        <x:f>IF(P22="","",P22/MAX(1,2026-E22+1))</x:f>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="R22" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S22" s="47" t="str">
-        <x:v>https://www.semanticscholar.org/search?q=Vid2Robot%3A%20End-to-End%20Video-Conditioned%20Policy%20Learning%20with%20Cross-Attention%20Transformers</x:v>
+        <x:v>https://www.semanticscholar.org/search?q=PointWorld%3A%20Scaling%203D%20World%20Models%20for%20In-the-Wild%20Robotic%20Manipulation</x:v>
       </x:c>
       <x:c r="T22" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -7987,10 +8012,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="C23" s="64" t="str">
-        <x:v>P043</x:v>
+        <x:v>P021</x:v>
       </x:c>
       <x:c r="D23" s="47" t="str">
-        <x:v>IRASim: A Fine-Grained World Model for Robot Manipulation</x:v>
+        <x:v>Vid2Robot: End-to-End Video-Conditioned Policy Learning with Cross-Attention Transformers</x:v>
       </x:c>
       <x:c r="E23" s="63" t="n">
         <x:v>2024</x:v>
@@ -7999,13 +8024,13 @@
         <x:v>Bridge</x:v>
       </x:c>
       <x:c r="G23" s="47" t="str">
-        <x:v>G2</x:v>
+        <x:v>U2</x:v>
       </x:c>
       <x:c r="H23" s="47" t="str">
-        <x:v>Robot-action-conditioned future video</x:v>
+        <x:v>Video-conditioned action</x:v>
       </x:c>
       <x:c r="I23" s="47" t="str">
-        <x:v>World simulation</x:v>
+        <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="J23" s="47" t="str">
         <x:v>Major</x:v>
@@ -8014,28 +8039,29 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="L23" s="47" t="str">
-        <x:v>Asia</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="M23" s="47" t="str">
-        <x:v>Fangqi Zhu; Hongtao Wu; Song Guo; Yuxiao Liu; Chilam Cheang; Tao Kong</x:v>
+        <x:v>Authors per paper; DeepMind Robotics</x:v>
       </x:c>
       <x:c r="N23" s="47" t="str">
-        <x:v>https://arxiv.org/abs/2406.14540</x:v>
+        <x:v>https://arxiv.org/abs/2403.12943</x:v>
       </x:c>
       <x:c r="O23" s="47" t="str">
-        <x:v>Direct robot manipulation world model with frame-level action conditioning and policy-evaluation use</x:v>
+        <x:v>Directly produces robot actions from human/robot video prompts</x:v>
       </x:c>
       <x:c r="P23" s="51" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="Q23" s="51" t="n">
+        <x:f>IF(P23="","",P23/MAX(1,2026-E23+1))</x:f>
         <x:v>21.666666666666668</x:v>
       </x:c>
       <x:c r="R23" s="47" t="str">
-        <x:v>Observed scholarly web index; added during G2 audit; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S23" s="47" t="str">
-        <x:v>https://arxiv.org/abs/2406.14540</x:v>
+        <x:v>https://www.semanticscholar.org/search?q=Vid2Robot%3A%20End-to-End%20Video-Conditioned%20Policy%20Learning%20with%20Cross-Attention%20Transformers</x:v>
       </x:c>
       <x:c r="T23" s="52" t="str">
         <x:v>2026-09-02</x:v>
@@ -8091,16 +8117,17 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="Q24" s="51" t="n">
+        <x:f>IF(P24="","",P24/MAX(1,2026-E24+1))</x:f>
         <x:v>20.666666666666668</x:v>
       </x:c>
       <x:c r="R24" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S24" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=ViViDex%3A%20Learning%20Vision-Based%20Dexterous%20Manipulation%20from%20Human%20Videos</x:v>
       </x:c>
       <x:c r="T24" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
@@ -8153,10 +8180,11 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="Q25" s="51" t="n">
+        <x:f>IF(P25="","",P25/MAX(1,2026-E25+1))</x:f>
         <x:v>28.5</x:v>
       </x:c>
       <x:c r="R25" s="47" t="str">
-        <x:v>Observed scholarly web index; added during G2 audit; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S25" s="47" t="str">
         <x:v>https://openreview.net/forum?id=pFyzqbUiF9</x:v>
@@ -8215,16 +8243,17 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="Q26" s="51" t="n">
+        <x:f>IF(P26="","",P26/MAX(1,2026-E26+1))</x:f>
         <x:v>27.5</x:v>
       </x:c>
       <x:c r="R26" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S26" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=GWM%3A%20Towards%20Scalable%20Gaussian%20World%20Models%20for%20Robotic%20Manipulation</x:v>
       </x:c>
       <x:c r="T26" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
@@ -8277,16 +8306,17 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="Q27" s="51" t="n">
+        <x:f>IF(P27="","",P27/MAX(1,2026-E27+1))</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="R27" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S27" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=RIGVid%3A%20Robots%20Imitating%20Generated%20Videos</x:v>
       </x:c>
       <x:c r="T27" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
@@ -8339,16 +8369,17 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="Q28" s="51" t="n">
+        <x:f>IF(P28="","",P28/MAX(1,2026-E28+1))</x:f>
         <x:v>9.25</x:v>
       </x:c>
       <x:c r="R28" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S28" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Learning%20Video-Conditioned%20Policies%20for%20Unseen%20Manipulation%20Tasks</x:v>
       </x:c>
       <x:c r="T28" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
@@ -8401,10 +8432,11 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="Q29" s="51" t="n">
+        <x:f>IF(P29="","",P29/MAX(1,2026-E29+1))</x:f>
         <x:v>11.666666666666666</x:v>
       </x:c>
       <x:c r="R29" s="47" t="str">
-        <x:v>Observed scholarly web index; added during G2 audit; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S29" s="47" t="str">
         <x:v>https://openreview.net/forum?id=15ASUbzg0N</x:v>
@@ -8421,58 +8453,59 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="C30" s="64" t="str">
-        <x:v>P027</x:v>
+        <x:v>P026</x:v>
       </x:c>
       <x:c r="D30" s="47" t="str">
-        <x:v>Gemini Robotics 1.5</x:v>
+        <x:v>Dream2Flow: Bridging Video Generation and Open-World Manipulation with 3D Object Flow</x:v>
       </x:c>
       <x:c r="E30" s="63" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="F30" s="47" t="str">
-        <x:v>Robotics</x:v>
+        <x:v>Bridge</x:v>
       </x:c>
       <x:c r="G30" s="47" t="str">
-        <x:v>VL</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="H30" s="47" t="str">
-        <x:v>Robot actions</x:v>
+        <x:v>3D object flow</x:v>
       </x:c>
       <x:c r="I30" s="47" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>Planning</x:v>
       </x:c>
       <x:c r="J30" s="47" t="str">
-        <x:v>Landmark</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="K30" s="47" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="L30" s="47" t="str">
-        <x:v>Europe</x:v>
+        <x:v>US</x:v>
       </x:c>
       <x:c r="M30" s="47" t="str">
-        <x:v>Google DeepMind robotics team incl. Agrim Gupta</x:v>
+        <x:v>Karthik Dharmarajan; Wenlong Huang; Jiajun Wu; Li Fei-Fei; Ruohan Zhang</x:v>
       </x:c>
       <x:c r="N30" s="47" t="str">
-        <x:v>https://arxiv.org/abs/2510.03342</x:v>
+        <x:v>https://jiajunwu.com/</x:v>
       </x:c>
       <x:c r="O30" s="47" t="str">
-        <x:v>Generalist VLA with embodied reasoning</x:v>
+        <x:v>Explicit video-generation-to-manipulation bridge</x:v>
       </x:c>
       <x:c r="P30" s="51" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="Q30" s="51" t="n">
-        <x:v>2</x:v>
+        <x:f>IF(P30="","",P30/MAX(1,2026-E30+1))</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="R30" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S30" s="47" t="str">
-        <x:v>https://www.semanticscholar.org/search?q=Gemini%20Robotics%201.5</x:v>
+        <x:v>https://www.semanticscholar.org/search?q=Dream2Flow%3A%20Bridging%20Video%20Generation%20and%20Open-World%20Manipulation%20with%203D%20Object%20Flow</x:v>
       </x:c>
       <x:c r="T30" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
@@ -8483,56 +8516,59 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="C31" s="64" t="str">
-        <x:v>P026</x:v>
+        <x:v>P027</x:v>
       </x:c>
       <x:c r="D31" s="47" t="str">
-        <x:v>Dream2Flow: Bridging Video Generation and Open-World Manipulation with 3D Object Flow</x:v>
+        <x:v>Gemini Robotics 1.5</x:v>
       </x:c>
       <x:c r="E31" s="63" t="n">
-        <x:v>2026</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="F31" s="47" t="str">
-        <x:v>Bridge</x:v>
+        <x:v>Robotics</x:v>
       </x:c>
       <x:c r="G31" s="47" t="str">
-        <x:v>G2</x:v>
+        <x:v>VL</x:v>
       </x:c>
       <x:c r="H31" s="47" t="str">
-        <x:v>3D object flow</x:v>
+        <x:v>Robot actions</x:v>
       </x:c>
       <x:c r="I31" s="47" t="str">
-        <x:v>Planning</x:v>
+        <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="J31" s="47" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Landmark</x:v>
       </x:c>
       <x:c r="K31" s="47" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="L31" s="47" t="str">
-        <x:v>US</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="M31" s="47" t="str">
-        <x:v>Karthik Dharmarajan; Wenlong Huang; Jiajun Wu; Li Fei-Fei; Ruohan Zhang</x:v>
+        <x:v>Google DeepMind robotics team incl. Agrim Gupta</x:v>
       </x:c>
       <x:c r="N31" s="47" t="str">
-        <x:v>https://jiajunwu.com/</x:v>
+        <x:v>https://arxiv.org/abs/2510.03342</x:v>
       </x:c>
       <x:c r="O31" s="47" t="str">
-        <x:v>Explicit video-generation-to-manipulation bridge</x:v>
+        <x:v>Generalist VLA with embodied reasoning</x:v>
       </x:c>
       <x:c r="P31" s="51" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q31" s="51" t="str"/>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="Q31" s="51" t="n">
+        <x:f>IF(P31="","",P31/MAX(1,2026-E31+1))</x:f>
+        <x:v>3.5</x:v>
+      </x:c>
       <x:c r="R31" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S31" s="47" t="str">
-        <x:v>https://www.semanticscholar.org/search?q=Dream2Flow%3A%20Bridging%20Video%20Generation%20and%20Open-World%20Manipulation%20with%203D%20Object%20Flow</x:v>
+        <x:v>https://www.semanticscholar.org/search?q=Gemini%20Robotics%201.5</x:v>
       </x:c>
       <x:c r="T31" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
@@ -8581,20 +8617,25 @@
       <x:c r="O32" s="47" t="str">
         <x:v>Robot video world model and self-learning system</x:v>
       </x:c>
-      <x:c r="P32" s="51"/>
-      <x:c r="Q32" s="51" t="str"/>
+      <x:c r="P32" s="51" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="Q32" s="51" t="n">
+        <x:f>IF(P32="","",P32/MAX(1,2026-E32+1))</x:f>
+        <x:v>2.5</x:v>
+      </x:c>
       <x:c r="R32" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S32" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=1X%20World%20Model</x:v>
       </x:c>
       <x:c r="T32" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
-      <x:c r="A33" s="63" t="str"/>
+      <x:c r="A33" s="63"/>
       <x:c r="B33" s="63" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -8641,20 +8682,21 @@
         <x:v>3936</x:v>
       </x:c>
       <x:c r="Q33" s="51" t="n">
+        <x:f>IF(P33="","",P33/MAX(1,2026-E33+1))</x:f>
         <x:v>984</x:v>
       </x:c>
       <x:c r="R33" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S33" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=RT-2%3A%20Vision-Language-Action%20Models%20Transfer%20Web%20Knowledge%20to%20Robotic%20Control</x:v>
       </x:c>
       <x:c r="T33" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
-      <x:c r="A34" s="63" t="str"/>
+      <x:c r="A34" s="63"/>
       <x:c r="B34" s="63" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -8701,20 +8743,21 @@
         <x:v>3896</x:v>
       </x:c>
       <x:c r="Q34" s="51" t="n">
+        <x:f>IF(P34="","",P34/MAX(1,2026-E34+1))</x:f>
         <x:v>974</x:v>
       </x:c>
       <x:c r="R34" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S34" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Diffusion%20Policy%3A%20Visuomotor%20Policy%20Learning%20via%20Action%20Diffusion</x:v>
       </x:c>
       <x:c r="T34" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
-      <x:c r="A35" s="63" t="str"/>
+      <x:c r="A35" s="63"/>
       <x:c r="B35" s="63" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -8761,20 +8804,21 @@
         <x:v>3125</x:v>
       </x:c>
       <x:c r="Q35" s="51" t="n">
+        <x:f>IF(P35="","",P35/MAX(1,2026-E35+1))</x:f>
         <x:v>1041.6666666666667</x:v>
       </x:c>
       <x:c r="R35" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S35" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=OpenVLA%3A%20An%20Open-Source%20Vision-Language-Action%20Model</x:v>
       </x:c>
       <x:c r="T35" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
-      <x:c r="A36" s="63" t="str"/>
+      <x:c r="A36" s="63"/>
       <x:c r="B36" s="63" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -8821,10 +8865,11 @@
         <x:v>1151</x:v>
       </x:c>
       <x:c r="Q36" s="51" t="n">
+        <x:f>IF(P36="","",P36/MAX(1,2026-E36+1))</x:f>
         <x:v>95.91666666666667</x:v>
       </x:c>
       <x:c r="R36" s="47" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S36" s="47" t="str">
         <x:v>https://dl.acm.org/doi/10.5555/2969442.2969560</x:v>
@@ -8834,7 +8879,7 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
-      <x:c r="A37" s="63" t="str"/>
+      <x:c r="A37" s="63"/>
       <x:c r="B37" s="63" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -8878,23 +8923,24 @@
         <x:v>Foundational stochastic future prediction with control relevance</x:v>
       </x:c>
       <x:c r="P37" s="51" t="n">
-        <x:v>758</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="Q37" s="51" t="n">
-        <x:v>75.8</x:v>
+        <x:f>IF(P37="","",P37/MAX(1,2026-E37+1))</x:f>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="R37" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S37" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Stochastic%20Variational%20Video%20Prediction%20(SV2P)</x:v>
       </x:c>
       <x:c r="T37" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
-      <x:c r="A38" s="63" t="str"/>
+      <x:c r="A38" s="63"/>
       <x:c r="B38" s="63" t="n">
         <x:v>12</x:v>
       </x:c>
@@ -8941,20 +8987,21 @@
         <x:v>735</x:v>
       </x:c>
       <x:c r="Q38" s="51" t="n">
+        <x:f>IF(P38="","",P38/MAX(1,2026-E38+1))</x:f>
         <x:v>122.5</x:v>
       </x:c>
       <x:c r="R38" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S38" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=CALVIN%3A%20A%20Benchmark%20for%20Language-Conditioned%20Policy%20Learning%20for%20Long-Horizon%20Robot%20Manipulation</x:v>
       </x:c>
       <x:c r="T38" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
-      <x:c r="A39" s="63" t="str"/>
+      <x:c r="A39" s="63"/>
       <x:c r="B39" s="63" t="n">
         <x:v>13</x:v>
       </x:c>
@@ -9001,10 +9048,11 @@
         <x:v>731</x:v>
       </x:c>
       <x:c r="Q39" s="51" t="n">
+        <x:f>IF(P39="","",P39/MAX(1,2026-E39+1))</x:f>
         <x:v>243.66666666666666</x:v>
       </x:c>
       <x:c r="R39" s="47" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S39" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Genie%3A%20Generative%20Interactive%20Environments</x:v>
@@ -9014,7 +9062,7 @@
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
-      <x:c r="A40" s="63" t="str"/>
+      <x:c r="A40" s="63"/>
       <x:c r="B40" s="63" t="n">
         <x:v>14</x:v>
       </x:c>
@@ -9058,23 +9106,24 @@
         <x:v>Strong motion representation feeding world-model research</x:v>
       </x:c>
       <x:c r="P40" s="51" t="n">
-        <x:v>716</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="Q40" s="51" t="n">
-        <x:v>179</x:v>
+        <x:f>IF(P40="","",P40/MAX(1,2026-E40+1))</x:f>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="R40" s="47" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S40" s="47" t="str">
         <x:v>https://www.semanticscholar.org/search?q=CoTracker%3A%20It%20is%20Better%20to%20Track%20Together</x:v>
       </x:c>
       <x:c r="T40" s="52" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
-      <x:c r="A41" s="63" t="str"/>
+      <x:c r="A41" s="63"/>
       <x:c r="B41" s="63" t="n">
         <x:v>23</x:v>
       </x:c>
@@ -9121,10 +9170,11 @@
         <x:v>363</x:v>
       </x:c>
       <x:c r="Q41" s="51" t="n">
+        <x:f>IF(P41="","",P41/MAX(1,2026-E41+1))</x:f>
         <x:v>121</x:v>
       </x:c>
       <x:c r="R41" s="47" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S41" s="47" t="str">
         <x:v>https://openreview.net/forum?id=NadTwTODgC</x:v>
@@ -9134,7 +9184,7 @@
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="66" t="str"/>
+      <x:c r="A42" s="66"/>
       <x:c r="B42" s="66" t="n">
         <x:v>24</x:v>
       </x:c>
@@ -9181,20 +9231,21 @@
         <x:v>332</x:v>
       </x:c>
       <x:c r="Q42" s="24" t="n">
+        <x:f>IF(P42="","",P42/MAX(1,2026-E42+1))</x:f>
         <x:v>66.4</x:v>
       </x:c>
       <x:c r="R42" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S42" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=TAP-Vid%3A%20A%20Benchmark%20for%20Tracking%20Any%20Point%20in%20a%20Video</x:v>
       </x:c>
       <x:c r="T42" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="66" t="str"/>
+      <x:c r="A43" s="66"/>
       <x:c r="B43" s="66" t="n">
         <x:v>25</x:v>
       </x:c>
@@ -9241,10 +9292,11 @@
         <x:v>301</x:v>
       </x:c>
       <x:c r="Q43" s="24" t="n">
+        <x:f>IF(P43="","",P43/MAX(1,2026-E43+1))</x:f>
         <x:v>100.33333333333333</x:v>
       </x:c>
       <x:c r="R43" s="15" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S43" s="15" t="str">
         <x:v>https://openreview.net/forum?id=P8pqeEkn1H</x:v>
@@ -9254,7 +9306,7 @@
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="66" t="str"/>
+      <x:c r="A44" s="66"/>
       <x:c r="B44" s="66" t="n">
         <x:v>31</x:v>
       </x:c>
@@ -9301,10 +9353,11 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="Q44" s="24" t="n">
+        <x:f>IF(P44="","",P44/MAX(1,2026-E44+1))</x:f>
         <x:v>26.857142857142858</x:v>
       </x:c>
       <x:c r="R44" s="15" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S44" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Learning%20to%20Simulate%20Dynamic%20Environments%20with%20GameGAN</x:v>
@@ -9314,7 +9367,7 @@
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="66" t="str"/>
+      <x:c r="A45" s="66"/>
       <x:c r="B45" s="66" t="n">
         <x:v>36</x:v>
       </x:c>
@@ -9361,20 +9414,21 @@
         <x:v>135</x:v>
       </x:c>
       <x:c r="Q45" s="24" t="n">
+        <x:f>IF(P45="","",P45/MAX(1,2026-E45+1))</x:f>
         <x:v>22.5</x:v>
       </x:c>
       <x:c r="R45" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S45" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=FitVid%3A%20Overfitting%20in%20Pixel-Level%20Video%20Prediction</x:v>
       </x:c>
       <x:c r="T45" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="66" t="str"/>
+      <x:c r="A46" s="66"/>
       <x:c r="B46" s="66" t="n">
         <x:v>37</x:v>
       </x:c>
@@ -9418,13 +9472,14 @@
         <x:v>Extends action-conditioned generation to open-world game video; included as later lineage, not robot evidence</x:v>
       </x:c>
       <x:c r="P46" s="24" t="n">
-        <x:v>129</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="Q46" s="24" t="n">
-        <x:v>43</x:v>
+        <x:f>IF(P46="","",P46/MAX(1,2026-E46+1))</x:f>
+        <x:v>43.666666666666664</x:v>
       </x:c>
       <x:c r="R46" s="15" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S46" s="15" t="str">
         <x:v>https://openreview.net/forum?id=8VG8tpPZhe</x:v>
@@ -9434,7 +9489,7 @@
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="66" t="str"/>
+      <x:c r="A47" s="66"/>
       <x:c r="B47" s="66" t="n">
         <x:v>38</x:v>
       </x:c>
@@ -9481,10 +9536,11 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="Q47" s="24" t="n">
+        <x:f>IF(P47="","",P47/MAX(1,2026-E47+1))</x:f>
         <x:v>14.833333333333334</x:v>
       </x:c>
       <x:c r="R47" s="15" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S47" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Playable%20Video%20Generation</x:v>
@@ -9494,7 +9550,7 @@
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="66" t="str"/>
+      <x:c r="A48" s="66"/>
       <x:c r="B48" s="66" t="n">
         <x:v>40</x:v>
       </x:c>
@@ -9541,10 +9597,11 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="Q48" s="24" t="n">
+        <x:f>IF(P48="","",P48/MAX(1,2026-E48+1))</x:f>
         <x:v>27.333333333333332</x:v>
       </x:c>
       <x:c r="R48" s="15" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S48" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Pandora%3A%20Towards%20General%20World%20Model%20with%20Natural%20Language%20Actions%20and%20Video%20States</x:v>
@@ -9554,7 +9611,7 @@
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="66" t="str"/>
+      <x:c r="A49" s="66"/>
       <x:c r="B49" s="66" t="n">
         <x:v>51</x:v>
       </x:c>
@@ -9598,13 +9655,14 @@
         <x:v>Extends playable video toward language and high-level action control; no direct robotics result</x:v>
       </x:c>
       <x:c r="P49" s="24" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="Q49" s="24" t="n">
-        <x:v>7</x:v>
+        <x:f>IF(P49="","",P49/MAX(1,2026-E49+1))</x:f>
+        <x:v>7.25</x:v>
       </x:c>
       <x:c r="R49" s="15" t="str">
-        <x:v>Observed scholarly web index; adjacent lineage row; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S49" s="15" t="str">
         <x:v>https://dl.acm.org/doi/10.1145/3635705</x:v>
@@ -9614,7 +9672,7 @@
       </x:c>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="66" t="str"/>
+      <x:c r="A50" s="66"/>
       <x:c r="B50" s="66" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -9661,20 +9719,21 @@
         <x:v>4328</x:v>
       </x:c>
       <x:c r="Q50" s="24" t="n">
+        <x:f>IF(P50="","",P50/MAX(1,2026-E50+1))</x:f>
         <x:v>541</x:v>
       </x:c>
       <x:c r="R50" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S50" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=SlowFast%20Networks%20for%20Video%20Recognition</x:v>
       </x:c>
       <x:c r="T50" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="66" t="str"/>
+      <x:c r="A51" s="66"/>
       <x:c r="B51" s="66" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -9721,20 +9780,21 @@
         <x:v>1508</x:v>
       </x:c>
       <x:c r="Q51" s="24" t="n">
+        <x:f>IF(P51="","",P51/MAX(1,2026-E51+1))</x:f>
         <x:v>502.6666666666667</x:v>
       </x:c>
       <x:c r="R51" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S51" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=%CF%800%3A%20A%20Vision-Language-Action%20Flow%20Model%20for%20General%20Robot%20Control</x:v>
       </x:c>
       <x:c r="T51" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="66" t="str"/>
+      <x:c r="A52" s="66"/>
       <x:c r="B52" s="66" t="n">
         <x:v>17</x:v>
       </x:c>
@@ -9781,20 +9841,21 @@
         <x:v>586</x:v>
       </x:c>
       <x:c r="Q52" s="24" t="n">
+        <x:f>IF(P52="","",P52/MAX(1,2026-E52+1))</x:f>
         <x:v>146.5</x:v>
       </x:c>
       <x:c r="R52" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S52" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=VideoPoet%3A%20A%20Large%20Language%20Model%20for%20Zero-Shot%20Video%20Generation</x:v>
       </x:c>
       <x:c r="T52" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="66" t="str"/>
+      <x:c r="A53" s="66"/>
       <x:c r="B53" s="66" t="n">
         <x:v>18</x:v>
       </x:c>
@@ -9838,23 +9899,24 @@
         <x:v>Masked latent prediction architecture</x:v>
       </x:c>
       <x:c r="P53" s="24" t="n">
-        <x:v>554</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="Q53" s="24" t="n">
-        <x:v>184.66666666666666</x:v>
+        <x:f>IF(P53="","",P53/MAX(1,2026-E53+1))</x:f>
+        <x:v>187.66666666666666</x:v>
       </x:c>
       <x:c r="R53" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S53" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Revisiting%20Feature%20Prediction%20for%20Learning%20Visual%20Representations%20from%20Video%20(V-JEPA)</x:v>
       </x:c>
       <x:c r="T53" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="66" t="str"/>
+      <x:c r="A54" s="66"/>
       <x:c r="B54" s="66" t="n">
         <x:v>22</x:v>
       </x:c>
@@ -9898,23 +9960,24 @@
         <x:v>Strong video-generation credential for later robotics bridges</x:v>
       </x:c>
       <x:c r="P54" s="24" t="n">
-        <x:v>388</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="Q54" s="24" t="n">
-        <x:v>97</x:v>
+        <x:f>IF(P54="","",P54/MAX(1,2026-E54+1))</x:f>
+        <x:v>97.75</x:v>
       </x:c>
       <x:c r="R54" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S54" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Photorealistic%20Video%20Generation%20with%20Diffusion%20Models%20(WALT)</x:v>
       </x:c>
       <x:c r="T54" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="66" t="str"/>
+      <x:c r="A55" s="66"/>
       <x:c r="B55" s="66" t="n">
         <x:v>35</x:v>
       </x:c>
@@ -9961,20 +10024,21 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="Q55" s="24" t="n">
+        <x:f>IF(P55="","",P55/MAX(1,2026-E55+1))</x:f>
         <x:v>39.25</x:v>
       </x:c>
       <x:c r="R55" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S55" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Siamese%20Masked%20Autoencoders</x:v>
       </x:c>
       <x:c r="T55" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="66" t="str"/>
+      <x:c r="A56" s="66"/>
       <x:c r="B56" s="66" t="n">
         <x:v>52</x:v>
       </x:c>
@@ -10018,25 +10082,26 @@
         <x:v>External survey for scope checking and future expansion</x:v>
       </x:c>
       <x:c r="P56" s="24" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="Q56" s="24" t="n">
-        <x:v>17</x:v>
+        <x:f>IF(P56="","",P56/MAX(1,2026-E56+1))</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="R56" s="15" t="str">
-        <x:v>Observed scholarly web index; versions may be split</x:v>
+        <x:v>Observed scholarly-web-index count; rechecked 2026-09-02; versions may be split</x:v>
       </x:c>
       <x:c r="S56" s="15" t="str">
         <x:v>https://www.semanticscholar.org/search?q=Video%20Generation%20Models%20in%20Robotics%3A%20Applications%2C%20Challenges%2C%20and%20Future%20Directions</x:v>
       </x:c>
       <x:c r="T56" s="15" t="str">
-        <x:v>2026-08-30</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61e2816769f14b96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ff05ce629ed4a5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10504,7 +10569,7 @@
     <x:mergeCell ref="A19:H19"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67b4e3f109df4657"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf64bf6312bfa4e5f"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Unify architecture mapping and tighten researcher scope
</commit_message>
<xml_diff>
--- a/notes/01-video-to-robotics-transition/video_to_robotics_architecture_pilot.xlsx
+++ b/notes/01-video-to-robotics-transition/video_to_robotics_architecture_pilot.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Method" sheetId="1" r:id="R836eb544cdcc47eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="Ra656c9939c7c423a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="3" r:id="Rb9a0d70abfa44fd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Researchers" sheetId="4" r:id="R17481e95c5c847f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Matrix" sheetId="5" r:id="R733f72f91a8842b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transition_Matrix" sheetId="6" r:id="R8db4a937c72a4893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="7" r:id="Rb0e3dd2974ef4de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_Log" sheetId="8" r:id="R26e4e6992f26465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Method" sheetId="1" r:id="R03443d765dbd4125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="Ra95937d9b828454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="3" r:id="Re806c23774eb47ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Researchers" sheetId="4" r:id="R002a0634677046c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Matrix" sheetId="5" r:id="R8f6491d6504c40cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transition_Matrix" sheetId="6" r:id="R65e40ab97d1e410f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="7" r:id="R765f756fbc334669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_Log" sheetId="8" r:id="R916f27f12b4a43f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -195,14 +195,14 @@
   <x:dxfs count="2">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E4"/>
         </x:patternFill>
       </x:fill>
@@ -243,7 +243,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResearchersTable" displayName="ResearchersTable" ref="A1:AE58" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResearchersTable" displayName="ResearchersTable" ref="A1:AE57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Impact_rank"/>
     <x:tableColumn id="2" name="Researcher_ID"/>
@@ -274,7 +274,7 @@
     <x:tableColumn id="27" name="Citation_coverage"/>
     <x:tableColumn id="28" name="Citation_as_of"/>
     <x:tableColumn id="29" name="Representative_video_mechanism"/>
-    <x:tableColumn id="30" name="Representative_robot_output"/>
+    <x:tableColumn id="30" name="Representative_robot_output_description"/>
     <x:tableColumn id="31" name="Audit_status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -515,15 +515,15 @@
         <x:v>Sample</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>57 researchers and 66 papers in separate, non-1:1 tables; 31 direct bridge, 22 adjacent/context, 13 one-side reference papers</x:v>
+        <x:v>56 researchers and 66 papers in separate, non-1:1 tables; 31 direct bridge, 22 adjacent/context, 13 one-side reference papers</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="6" t="str">
-        <x:v>Three classification axes</x:v>
+        <x:v>Unified chart axis</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>Video_bridge_mechanism records what came from video; Focal_output_code records what the focal model emits; Robot_role records downstream use</x:v>
+        <x:v>Video_bridge_mechanism is the only architecture code used in mappings; it records what came from video and maps directly to Robot_role. Model output is descriptive metadata only</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -547,7 +547,7 @@
         <x:v>Citation coverage</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>Scores require two distinct selected papers, both with citation counts. A single bridge paper can establish a connection but is not counted twice</x:v>
+        <x:v>Scores require two distinct selected papers, both with citation counts. Single-paper bridges remain documented but are not part of the distinct-paper ranking</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -579,7 +579,7 @@
         <x:v>Audit correction</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
-        <x:v>Dream2Flow is G1; PointWorld is G2; CALVIN is a benchmark; RoboCat and Gemini Robotics are not direct video-model bridges</x:v>
+        <x:v>Dream2Flow is G1; PointWorld is G2; CALVIN is a benchmark; Tim Rocktäschel is excluded from the researcher sample while Genie remains context</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -604,7 +604,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Video Mechanism, Output, and Transition Taxonomy</x:v>
+        <x:v>Unified Video-Origin Architecture and Transition Taxonomy</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -612,6 +612,22 @@
       <x:c r="E1" s="3"/>
       <x:c r="F1" s="3"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+    </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
         <x:v>Code</x:v>
@@ -637,7 +653,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>Video mechanism / output</x:v>
+        <x:v>Unified video-origin code</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str">
         <x:v>Generates image/video pixels or tokens without robot action as a central input</x:v>
@@ -649,7 +665,7 @@
         <x:v>visual plan, subgoal, synthetic data</x:v>
       </x:c>
       <x:c r="F5" s="6" t="str">
-        <x:v>Motion or language prompts do not by themselves make the model G2</x:v>
+        <x:v>Motion or language prompts alone do not make a model G2</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -657,10 +673,10 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
-        <x:v>Video mechanism / output</x:v>
+        <x:v>Unified video-origin code</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str">
-        <x:v>Predicts future video/state; robot or agent action may condition input but is not the output</x:v>
+        <x:v>Predicts future video/state; robot or agent action may condition the input but is not emitted</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
         <x:v>Visual Foresight, PointWorld, GameNGen</x:v>
@@ -669,7 +685,7 @@
         <x:v>world simulation, planning</x:v>
       </x:c>
       <x:c r="F6" s="6" t="str">
-        <x:v>Game papers remain Adjacent unless robotics transfer is shown</x:v>
+        <x:v>Game papers remain context unless robotics transfer is shown</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -677,10 +693,10 @@
         <x:v>G3</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>Video mechanism / output</x:v>
+        <x:v>Unified video-origin code</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
-        <x:v>Jointly emits future visual/state variables and actions</x:v>
+        <x:v>Jointly generates future visual/state variables and actions</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
         <x:v>GR-2, Cosmos Policy</x:v>
@@ -689,7 +705,7 @@
         <x:v>direct policy</x:v>
       </x:c>
       <x:c r="F7" s="6" t="str">
-        <x:v>Different from A by joint visual/state output</x:v>
+        <x:v>Action-only policies are not a separate video-origin code</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -697,10 +713,10 @@
         <x:v>U1</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>Video mechanism</x:v>
+        <x:v>Unified video-origin code</x:v>
       </x:c>
       <x:c r="C8" s="6" t="str">
-        <x:v>Semantic/action/event understanding</x:v>
+        <x:v>Learns semantic, action, or event understanding from video</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
         <x:v>SlowFast</x:v>
@@ -709,7 +725,7 @@
         <x:v>perception</x:v>
       </x:c>
       <x:c r="F8" s="6" t="str">
-        <x:v>Representation axis, not an action-output code</x:v>
+        <x:v>Understanding rather than generation</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -717,10 +733,10 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="B9" s="6" t="str">
-        <x:v>Video mechanism</x:v>
+        <x:v>Unified video-origin code</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
-        <x:v>Motion, tracking, interaction, affordance</x:v>
+        <x:v>Learns motion, tracking, interaction, or affordance from video</x:v>
       </x:c>
       <x:c r="D9" s="6" t="str">
         <x:v>CoTracker, FlowNet, Track2Act</x:v>
@@ -729,7 +745,7 @@
         <x:v>perception, reward, policy condition</x:v>
       </x:c>
       <x:c r="F9" s="6" t="str">
-        <x:v>Can feed an A output policy</x:v>
+        <x:v>The downstream robot may still output actions</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -737,10 +753,10 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>Video mechanism</x:v>
+        <x:v>Unified video-origin code</x:v>
       </x:c>
       <x:c r="C10" s="6" t="str">
-        <x:v>Future or masked latent representation prediction</x:v>
+        <x:v>Predicts future or masked latent representations</x:v>
       </x:c>
       <x:c r="D10" s="6" t="str">
         <x:v>V-JEPA 2</x:v>
@@ -757,10 +773,10 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>Video mechanism</x:v>
+        <x:v>Unified video-origin code</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
-        <x:v>Video-language alignment or temporal multimodal reasoning</x:v>
+        <x:v>Aligns temporal video information with language or reasons over both</x:v>
       </x:c>
       <x:c r="D11" s="6" t="str">
         <x:v>MineDojo, LIV, Magma</x:v>
@@ -774,171 +790,135 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>Focal output</x:v>
+        <x:v>Unified video-origin code</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str">
-        <x:v>Action trajectory or action tokens only</x:v>
+        <x:v>No verified video-specific research mechanism</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:v>Diffusion Policy, RT-2, OpenVLA</x:v>
+        <x:v>RoboCat, RT-2</x:v>
       </x:c>
       <x:c r="E12" s="6" t="str">
-        <x:v>direct policy</x:v>
+        <x:v>comparison</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str">
-        <x:v>A is an output code, not a video-origin code</x:v>
+        <x:v>Robotics evidence alone is not a video bridge</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="6" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="B13" s="6" t="str">
-        <x:v>Focal output</x:v>
-      </x:c>
-      <x:c r="C13" s="6" t="str">
-        <x:v>Representation, reward, value, or feature</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="str">
-        <x:v>TCN, LIV</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="str">
-        <x:v>perception, reward</x:v>
-      </x:c>
-      <x:c r="F13" s="6" t="str">
-        <x:v>May coexist with U or VL on the video mechanism axis</x:v>
-      </x:c>
+      <x:c r="A13" s="6"/>
+      <x:c r="B13" s="6"/>
+      <x:c r="C13" s="6"/>
+      <x:c r="D13" s="6"/>
+      <x:c r="E13" s="6"/>
+      <x:c r="F13" s="6"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>Transition type</x:v>
       </x:c>
       <x:c r="B14" s="6" t="str">
-        <x:v>Focal output</x:v>
+        <x:v>Rule</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str">
-        <x:v>Dataset or benchmark rather than a model output</x:v>
+        <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D14" s="6" t="str">
-        <x:v>RoboNet, CALVIN, TAP-Vid</x:v>
-      </x:c>
-      <x:c r="E14" s="6" t="str">
-        <x:v>data/evaluation</x:v>
-      </x:c>
-      <x:c r="F14" s="6" t="str">
-        <x:v>Do not force a benchmark into a model architecture</x:v>
-      </x:c>
+        <x:v>Use</x:v>
+      </x:c>
+      <x:c r="E14" s="6"/>
+      <x:c r="F14" s="6"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="11" t="str">
-        <x:v>None</x:v>
+        <x:v>Switcher</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>Video mechanism</x:v>
+        <x:v>Organization or primary topic clearly moved video → robotics/world models</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>No verified video-specific research mechanism</x:v>
+        <x:v>strong migration</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>RoboCat, RT-2</x:v>
-      </x:c>
-      <x:c r="E15" s="14" t="str">
-        <x:v>comparison</x:v>
-      </x:c>
-      <x:c r="F15" s="12" t="str">
-        <x:v>Robotics evidence alone is not a video bridge</x:v>
-      </x:c>
+        <x:v>strict transition count</x:v>
+      </x:c>
+      <x:c r="E15" s="14"/>
+      <x:c r="F15" s="12"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
-      <x:c r="C16" s="6"/>
-      <x:c r="D16" s="6"/>
+      <x:c r="A16" s="6" t="str">
+        <x:v>Bridger</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>Verified important work on both sides or explicit transfer across papers</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>core bridge</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>bridge-talent count</x:v>
+      </x:c>
       <x:c r="E16" s="6"/>
       <x:c r="F16" s="6"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="str">
-        <x:v>Transition type</x:v>
+        <x:v>Native hybrid</x:v>
       </x:c>
       <x:c r="B17" s="6" t="str">
-        <x:v>Rule</x:v>
+        <x:v>Video and robotics pursued together from an early stage</x:v>
       </x:c>
       <x:c r="C17" s="6" t="str">
-        <x:v>Meaning</x:v>
+        <x:v>fusion rather than migration</x:v>
       </x:c>
       <x:c r="D17" s="6" t="str">
-        <x:v>Use</x:v>
+        <x:v>ecosystem count</x:v>
       </x:c>
       <x:c r="E17" s="6"/>
       <x:c r="F17" s="6"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="str">
-        <x:v>Switcher</x:v>
+        <x:v>Robotics-first</x:v>
       </x:c>
       <x:c r="B18" s="6" t="str">
-        <x:v>Organization or primary topic clearly moved video → robotics/world models</x:v>
+        <x:v>Robotics-centered comparison with no verified video-origin paper</x:v>
       </x:c>
       <x:c r="C18" s="6" t="str">
-        <x:v>strong migration</x:v>
+        <x:v>control group</x:v>
       </x:c>
       <x:c r="D18" s="6" t="str">
-        <x:v>strict transition count</x:v>
+        <x:v>overclaim check</x:v>
       </x:c>
       <x:c r="E18" s="6"/>
       <x:c r="F18" s="6"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="6" t="str">
-        <x:v>Bridger</x:v>
-      </x:c>
-      <x:c r="B19" s="6" t="str">
-        <x:v>Verified important work on both sides or explicit transfer across papers</x:v>
-      </x:c>
-      <x:c r="C19" s="6" t="str">
-        <x:v>core bridge</x:v>
-      </x:c>
-      <x:c r="D19" s="6" t="str">
-        <x:v>bridge-talent count</x:v>
-      </x:c>
-      <x:c r="E19" s="6"/>
-      <x:c r="F19" s="6"/>
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="6" t="str">
-        <x:v>Native hybrid</x:v>
-      </x:c>
-      <x:c r="B20" s="6" t="str">
-        <x:v>Video and robotics pursued together from an early stage</x:v>
-      </x:c>
-      <x:c r="C20" s="6" t="str">
-        <x:v>fusion rather than migration</x:v>
-      </x:c>
-      <x:c r="D20" s="6" t="str">
-        <x:v>ecosystem count</x:v>
-      </x:c>
-      <x:c r="E20" s="6"/>
-      <x:c r="F20" s="6"/>
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="6" t="str">
-        <x:v>Robotics-first</x:v>
-      </x:c>
-      <x:c r="B21" s="6" t="str">
-        <x:v>Robotics-centered comparison with no verified video-origin paper</x:v>
-      </x:c>
-      <x:c r="C21" s="6" t="str">
-        <x:v>control group</x:v>
-      </x:c>
-      <x:c r="D21" s="6" t="str">
-        <x:v>overclaim check</x:v>
-      </x:c>
-      <x:c r="E21" s="6"/>
-      <x:c r="F21" s="6"/>
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1000,7 +980,7 @@
         <x:v>Video_bridge_mechanism</x:v>
       </x:c>
       <x:c r="H1" s="14" t="str">
-        <x:v>Focal_output_code</x:v>
+        <x:v>Model_output_description</x:v>
       </x:c>
       <x:c r="I1" s="14" t="str">
         <x:v>Artifact_type</x:v>
@@ -1073,7 +1053,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I2" s="6" t="str">
         <x:v>Model</x:v>
@@ -1145,7 +1125,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str">
         <x:v>Model</x:v>
@@ -1217,7 +1197,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I4" s="6" t="str">
         <x:v>Model</x:v>
@@ -1289,7 +1269,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H5" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
         <x:v>Model</x:v>
@@ -1361,7 +1341,7 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="H6" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I6" s="6" t="str">
         <x:v>Model</x:v>
@@ -1433,7 +1413,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I7" s="6" t="str">
         <x:v>Model</x:v>
@@ -1505,7 +1485,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H8" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I8" s="6" t="str">
         <x:v>Model</x:v>
@@ -1577,7 +1557,7 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I9" s="6" t="str">
         <x:v>Model</x:v>
@@ -1649,7 +1629,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H10" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I10" s="6" t="str">
         <x:v>Model</x:v>
@@ -1721,7 +1701,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H11" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I11" s="6" t="str">
         <x:v>Model</x:v>
@@ -1793,7 +1773,7 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="H12" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I12" s="6" t="str">
         <x:v>Model</x:v>
@@ -1865,7 +1845,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H13" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I13" s="6" t="str">
         <x:v>Model</x:v>
@@ -1937,7 +1917,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H14" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>Dataset/benchmark</x:v>
       </x:c>
       <x:c r="I14" s="6" t="str">
         <x:v>Dataset</x:v>
@@ -2011,7 +1991,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H15" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I15" s="6" t="str">
         <x:v>Model</x:v>
@@ -2083,7 +2063,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H16" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I16" s="6" t="str">
         <x:v>Platform / model</x:v>
@@ -2155,7 +2135,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H17" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I17" s="6" t="str">
         <x:v>Model</x:v>
@@ -2227,7 +2207,7 @@
         <x:v>G3</x:v>
       </x:c>
       <x:c r="H18" s="6" t="str">
-        <x:v>G3</x:v>
+        <x:v>Joint visual/state + action</x:v>
       </x:c>
       <x:c r="I18" s="6" t="str">
         <x:v>Model</x:v>
@@ -2299,7 +2279,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="H19" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I19" s="6" t="str">
         <x:v>Model</x:v>
@@ -2371,7 +2351,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H20" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I20" s="6" t="str">
         <x:v>Model</x:v>
@@ -2443,7 +2423,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H21" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I21" s="6" t="str">
         <x:v>Model</x:v>
@@ -2515,7 +2495,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H22" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I22" s="6" t="str">
         <x:v>Model</x:v>
@@ -2587,7 +2567,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H23" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I23" s="6" t="str">
         <x:v>Model</x:v>
@@ -2659,7 +2639,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H24" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I24" s="6" t="str">
         <x:v>Model</x:v>
@@ -2731,7 +2711,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H25" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I25" s="6" t="str">
         <x:v>Model</x:v>
@@ -2802,7 +2782,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H26" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I26" s="6" t="str">
         <x:v>Model</x:v>
@@ -2872,7 +2852,7 @@
         <x:v>G3</x:v>
       </x:c>
       <x:c r="H27" s="6" t="str">
-        <x:v>G3</x:v>
+        <x:v>Joint visual/state + action</x:v>
       </x:c>
       <x:c r="I27" s="6" t="str">
         <x:v>Model</x:v>
@@ -2942,7 +2922,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H28" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I28" s="6" t="str">
         <x:v>Model</x:v>
@@ -3014,7 +2994,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H29" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I29" s="6" t="str">
         <x:v>Model</x:v>
@@ -3084,7 +3064,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H30" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I30" s="6" t="str">
         <x:v>Model</x:v>
@@ -3156,7 +3136,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H31" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I31" s="6" t="str">
         <x:v>Model</x:v>
@@ -3226,7 +3206,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H32" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I32" s="6" t="str">
         <x:v>Model card</x:v>
@@ -3294,7 +3274,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H33" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I33" s="6" t="str">
         <x:v>Model</x:v>
@@ -3365,7 +3345,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H34" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I34" s="6" t="str">
         <x:v>Model</x:v>
@@ -3436,7 +3416,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H35" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I35" s="6" t="str">
         <x:v>Model</x:v>
@@ -3507,7 +3487,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H36" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I36" s="6" t="str">
         <x:v>Model</x:v>
@@ -3578,7 +3558,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H37" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I37" s="6" t="str">
         <x:v>Model</x:v>
@@ -3649,7 +3629,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H38" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I38" s="6" t="str">
         <x:v>Model</x:v>
@@ -3722,7 +3702,7 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="H39" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I39" s="6" t="str">
         <x:v>Benchmark / platform</x:v>
@@ -3795,7 +3775,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H40" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I40" s="6" t="str">
         <x:v>Model</x:v>
@@ -3866,7 +3846,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H41" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I41" s="6" t="str">
         <x:v>Model</x:v>
@@ -3937,7 +3917,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H42" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>Dataset/benchmark</x:v>
       </x:c>
       <x:c r="I42" s="6" t="str">
         <x:v>Benchmark</x:v>
@@ -4008,7 +3988,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H43" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I43" s="6" t="str">
         <x:v>Model</x:v>
@@ -4079,7 +4059,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H44" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I44" s="6" t="str">
         <x:v>Model</x:v>
@@ -4150,7 +4130,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H45" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I45" s="6" t="str">
         <x:v>Model</x:v>
@@ -4223,7 +4203,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H46" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I46" s="6" t="str">
         <x:v>Model</x:v>
@@ -4296,7 +4276,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H47" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>Dataset/benchmark</x:v>
       </x:c>
       <x:c r="I47" s="6" t="str">
         <x:v>Benchmark</x:v>
@@ -4369,7 +4349,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H48" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I48" s="6" t="str">
         <x:v>Model</x:v>
@@ -4440,7 +4420,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H49" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I49" s="6" t="str">
         <x:v>Model</x:v>
@@ -4511,7 +4491,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H50" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I50" s="6" t="str">
         <x:v>Model</x:v>
@@ -4582,7 +4562,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H51" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I51" s="6" t="str">
         <x:v>Model</x:v>
@@ -4653,7 +4633,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H52" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I52" s="6" t="str">
         <x:v>Model</x:v>
@@ -4726,7 +4706,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H53" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I53" s="6" t="str">
         <x:v>Model</x:v>
@@ -4797,7 +4777,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="H54" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="I54" s="6" t="str">
         <x:v>Model</x:v>
@@ -4868,7 +4848,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="H55" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I55" s="6" t="str">
         <x:v>Model</x:v>
@@ -4939,7 +4919,7 @@
         <x:v>U1</x:v>
       </x:c>
       <x:c r="H56" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I56" s="6" t="str">
         <x:v>Model</x:v>
@@ -5010,7 +4990,7 @@
         <x:v>U1</x:v>
       </x:c>
       <x:c r="H57" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I57" s="6" t="str">
         <x:v>Model</x:v>
@@ -5081,7 +5061,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H58" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I58" s="6" t="str">
         <x:v>Model</x:v>
@@ -5152,7 +5132,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H59" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I59" s="6" t="str">
         <x:v>Model</x:v>
@@ -5223,7 +5203,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H60" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I60" s="6" t="str">
         <x:v>Model</x:v>
@@ -5294,7 +5274,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="H61" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I61" s="6" t="str">
         <x:v>Model</x:v>
@@ -5365,7 +5345,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="H62" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="I62" s="6" t="str">
         <x:v>Model</x:v>
@@ -5436,7 +5416,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H63" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I63" s="6" t="str">
         <x:v>Model</x:v>
@@ -5507,7 +5487,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="H64" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="I64" s="6" t="str">
         <x:v>Model</x:v>
@@ -5578,7 +5558,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H65" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I65" s="6" t="str">
         <x:v>Model</x:v>
@@ -5649,7 +5629,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="H66" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="I66" s="6" t="str">
         <x:v>Model</x:v>
@@ -5773,7 +5753,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cfdf78738aa470d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58b6931ac03a4e17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5904,7 +5884,7 @@
         <x:v>Representative_video_mechanism</x:v>
       </x:c>
       <x:c r="AD1" s="14" t="str">
-        <x:v>Representative_robot_output</x:v>
+        <x:v>Representative_robot_output_description</x:v>
       </x:c>
       <x:c r="AE1" s="12" t="str">
         <x:v>Audit_status</x:v>
@@ -5912,7 +5892,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="n">
-        <x:f>IF(Z2="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z2))</x:f>
+        <x:f>IF(Z2="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z2))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
@@ -6002,7 +5982,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD2" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE2" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6010,7 +5990,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="6" t="n">
-        <x:f>IF(Z3="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z3))</x:f>
+        <x:f>IF(Z3="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z3))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
@@ -6100,7 +6080,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD3" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE3" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6108,7 +6088,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="6" t="n">
-        <x:f>IF(Z4="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z4))</x:f>
+        <x:f>IF(Z4="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z4))</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
@@ -6198,7 +6178,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD4" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE4" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6206,7 +6186,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="6" t="n">
-        <x:f>IF(Z5="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z5))</x:f>
+        <x:f>IF(Z5="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z5))</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
@@ -6296,7 +6276,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD5" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>Dataset/benchmark</x:v>
       </x:c>
       <x:c r="AE5" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6304,7 +6284,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="6" t="n">
-        <x:f>IF(Z6="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z6))</x:f>
+        <x:f>IF(Z6="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z6))</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
@@ -6394,7 +6374,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD6" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>Dataset/benchmark</x:v>
       </x:c>
       <x:c r="AE6" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6402,7 +6382,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="6" t="n">
-        <x:f>IF(Z7="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z7))</x:f>
+        <x:f>IF(Z7="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z7))</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
@@ -6492,7 +6472,7 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="AD7" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE7" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6500,7 +6480,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="6" t="n">
-        <x:f>IF(Z8="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z8))</x:f>
+        <x:f>IF(Z8="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z8))</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
@@ -6590,7 +6570,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD8" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE8" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6598,7 +6578,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6" t="n">
-        <x:f>IF(Z9="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z9))</x:f>
+        <x:f>IF(Z9="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z9))</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="6" t="str">
@@ -6688,7 +6668,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD9" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE9" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6696,7 +6676,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="6" t="n">
-        <x:f>IF(Z10="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z10))</x:f>
+        <x:f>IF(Z10="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z10))</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
@@ -6786,7 +6766,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD10" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE10" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6794,7 +6774,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="6" t="n">
-        <x:f>IF(Z11="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z11))</x:f>
+        <x:f>IF(Z11="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z11))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
@@ -6884,7 +6864,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD11" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE11" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6892,7 +6872,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6" t="n">
-        <x:f>IF(Z12="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z12))</x:f>
+        <x:f>IF(Z12="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z12))</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
@@ -6982,7 +6962,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD12" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE12" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -6990,7 +6970,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="6" t="n">
-        <x:f>IF(Z13="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z13))</x:f>
+        <x:f>IF(Z13="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z13))</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="6" t="str">
@@ -7080,7 +7060,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD13" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE13" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7088,7 +7068,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="6" t="n">
-        <x:f>IF(Z14="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z14))</x:f>
+        <x:f>IF(Z14="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z14))</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="6" t="str">
@@ -7178,7 +7158,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD14" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE14" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7186,7 +7166,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="6" t="n">
-        <x:f>IF(Z15="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z15))</x:f>
+        <x:f>IF(Z15="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z15))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
@@ -7276,7 +7256,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="AD15" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE15" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7284,7 +7264,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="n">
-        <x:f>IF(Z16="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z16))</x:f>
+        <x:f>IF(Z16="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z16))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B16" s="6" t="str">
@@ -7374,7 +7354,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="AD16" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE16" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7382,7 +7362,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="n">
-        <x:f>IF(Z17="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z17))</x:f>
+        <x:f>IF(Z17="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z17))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B17" s="6" t="str">
@@ -7472,7 +7452,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="AD17" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE17" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7480,7 +7460,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="n">
-        <x:f>IF(Z18="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z18))</x:f>
+        <x:f>IF(Z18="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z18))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B18" s="6" t="str">
@@ -7570,7 +7550,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="AD18" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE18" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7578,7 +7558,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="6" t="n">
-        <x:f>IF(Z19="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z19))</x:f>
+        <x:f>IF(Z19="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z19))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B19" s="6" t="str">
@@ -7668,7 +7648,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="AD19" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE19" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7676,7 +7656,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="6" t="n">
-        <x:f>IF(Z20="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z20))</x:f>
+        <x:f>IF(Z20="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z20))</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="6" t="str">
@@ -7766,7 +7746,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD20" s="6" t="str">
-        <x:v>G3</x:v>
+        <x:v>Joint visual/state + action</x:v>
       </x:c>
       <x:c r="AE20" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7774,7 +7754,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="6" t="n">
-        <x:f>IF(Z21="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z21))</x:f>
+        <x:f>IF(Z21="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z21))</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="B21" s="6" t="str">
@@ -7864,7 +7844,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD21" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE21" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -7872,7 +7852,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="6" t="str">
-        <x:f>IF(Z22="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z22))</x:f>
+        <x:f>IF(Z22="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z22))</x:f>
       </x:c>
       <x:c r="B22" s="6" t="str">
         <x:v>R048</x:v>
@@ -7962,7 +7942,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="6" t="str">
-        <x:f>IF(Z23="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z23))</x:f>
+        <x:f>IF(Z23="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z23))</x:f>
       </x:c>
       <x:c r="B23" s="6" t="str">
         <x:v>R006</x:v>
@@ -8050,7 +8030,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD23" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE23" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -8058,7 +8038,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="6" t="str">
-        <x:f>IF(Z24="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z24))</x:f>
+        <x:f>IF(Z24="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z24))</x:f>
       </x:c>
       <x:c r="B24" s="6" t="str">
         <x:v>R047</x:v>
@@ -8148,7 +8128,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="6" t="str">
-        <x:f>IF(Z25="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z25))</x:f>
+        <x:f>IF(Z25="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z25))</x:f>
       </x:c>
       <x:c r="B25" s="6" t="str">
         <x:v>R012</x:v>
@@ -8236,7 +8216,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="AD25" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE25" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -8244,7 +8224,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="6" t="str">
-        <x:f>IF(Z26="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z26))</x:f>
+        <x:f>IF(Z26="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z26))</x:f>
       </x:c>
       <x:c r="B26" s="6" t="str">
         <x:v>R028</x:v>
@@ -8332,7 +8312,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD26" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE26" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -8340,7 +8320,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="6" t="str">
-        <x:f>IF(Z27="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z27))</x:f>
+        <x:f>IF(Z27="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z27))</x:f>
       </x:c>
       <x:c r="B27" s="6" t="str">
         <x:v>R032</x:v>
@@ -8428,7 +8408,7 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="AD27" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE27" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -8436,7 +8416,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="6" t="str">
-        <x:f>IF(Z28="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z28))</x:f>
+        <x:f>IF(Z28="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z28))</x:f>
       </x:c>
       <x:c r="B28" s="6" t="str">
         <x:v>R044</x:v>
@@ -8524,7 +8504,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD28" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE28" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -8532,7 +8512,7 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="6" t="str">
-        <x:f>IF(Z29="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z29))</x:f>
+        <x:f>IF(Z29="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z29))</x:f>
       </x:c>
       <x:c r="B29" s="6" t="str">
         <x:v>R015</x:v>
@@ -8620,7 +8600,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="AD29" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE29" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -8628,7 +8608,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="6" t="str">
-        <x:f>IF(Z30="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z30))</x:f>
+        <x:f>IF(Z30="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z30))</x:f>
       </x:c>
       <x:c r="B30" s="6" t="str">
         <x:v>R035</x:v>
@@ -8716,7 +8696,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD30" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE30" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -8724,7 +8704,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="6" t="str">
-        <x:f>IF(Z31="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z31))</x:f>
+        <x:f>IF(Z31="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z31))</x:f>
       </x:c>
       <x:c r="B31" s="6" t="str">
         <x:v>R043</x:v>
@@ -8812,7 +8792,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD31" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE31" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -8820,7 +8800,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="6" t="str">
-        <x:f>IF(Z32="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z32))</x:f>
+        <x:f>IF(Z32="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z32))</x:f>
       </x:c>
       <x:c r="B32" s="6" t="str">
         <x:v>R004</x:v>
@@ -8908,7 +8888,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD32" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE32" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -8916,7 +8896,7 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="6" t="str">
-        <x:f>IF(Z33="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z33))</x:f>
+        <x:f>IF(Z33="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z33))</x:f>
       </x:c>
       <x:c r="B33" s="6" t="str">
         <x:v>R053</x:v>
@@ -9004,7 +8984,7 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="AD33" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE33" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -9012,7 +8992,7 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="6" t="str">
-        <x:f>IF(Z34="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z34))</x:f>
+        <x:f>IF(Z34="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z34))</x:f>
       </x:c>
       <x:c r="B34" s="6" t="str">
         <x:v>R007</x:v>
@@ -9100,7 +9080,7 @@
         <x:v>U1</x:v>
       </x:c>
       <x:c r="AD34" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>Dataset/benchmark</x:v>
       </x:c>
       <x:c r="AE34" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -9108,7 +9088,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="6" t="str">
-        <x:f>IF(Z35="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z35))</x:f>
+        <x:f>IF(Z35="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z35))</x:f>
       </x:c>
       <x:c r="B35" s="6" t="str">
         <x:v>R003</x:v>
@@ -9198,7 +9178,7 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="6" t="str">
-        <x:f>IF(Z36="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z36))</x:f>
+        <x:f>IF(Z36="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z36))</x:f>
       </x:c>
       <x:c r="B36" s="6" t="str">
         <x:v>R041</x:v>
@@ -9286,7 +9266,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD36" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE36" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -9294,7 +9274,7 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="6" t="str">
-        <x:f>IF(Z37="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z37))</x:f>
+        <x:f>IF(Z37="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z37))</x:f>
       </x:c>
       <x:c r="B37" s="6" t="str">
         <x:v>R038</x:v>
@@ -9376,7 +9356,7 @@
       </x:c>
       <x:c r="AC37" s="6"/>
       <x:c r="AD37" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE37" s="6" t="str">
         <x:v>Partial evidence</x:v>
@@ -9384,7 +9364,7 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="6" t="str">
-        <x:f>IF(Z38="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z38))</x:f>
+        <x:f>IF(Z38="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z38))</x:f>
       </x:c>
       <x:c r="B38" s="6" t="str">
         <x:v>R002</x:v>
@@ -9474,7 +9454,7 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="6" t="str">
-        <x:f>IF(Z39="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z39))</x:f>
+        <x:f>IF(Z39="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z39))</x:f>
       </x:c>
       <x:c r="B39" s="6" t="str">
         <x:v>R027</x:v>
@@ -9562,7 +9542,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD39" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE39" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -9570,7 +9550,7 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="6" t="str">
-        <x:f>IF(Z40="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z40))</x:f>
+        <x:f>IF(Z40="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z40))</x:f>
       </x:c>
       <x:c r="B40" s="6" t="str">
         <x:v>R021</x:v>
@@ -9658,7 +9638,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD40" s="6" t="str">
-        <x:v>G3</x:v>
+        <x:v>Joint visual/state + action</x:v>
       </x:c>
       <x:c r="AE40" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -9666,7 +9646,7 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="6" t="str">
-        <x:f>IF(Z41="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z41))</x:f>
+        <x:f>IF(Z41="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z41))</x:f>
       </x:c>
       <x:c r="B41" s="6" t="str">
         <x:v>R046</x:v>
@@ -9746,7 +9726,7 @@
       </x:c>
       <x:c r="AC41" s="6"/>
       <x:c r="AD41" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>Dataset/benchmark</x:v>
       </x:c>
       <x:c r="AE41" s="6" t="str">
         <x:v>Partial evidence</x:v>
@@ -9754,7 +9734,7 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="6" t="str">
-        <x:f>IF(Z42="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z42))</x:f>
+        <x:f>IF(Z42="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z42))</x:f>
       </x:c>
       <x:c r="B42" s="6" t="str">
         <x:v>R045</x:v>
@@ -9834,7 +9814,7 @@
       </x:c>
       <x:c r="AC42" s="6"/>
       <x:c r="AD42" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE42" s="6" t="str">
         <x:v>Partial evidence</x:v>
@@ -9842,7 +9822,7 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="6" t="str">
-        <x:f>IF(Z43="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z43))</x:f>
+        <x:f>IF(Z43="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z43))</x:f>
       </x:c>
       <x:c r="B43" s="6" t="str">
         <x:v>R039</x:v>
@@ -9930,7 +9910,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD43" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE43" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -9938,7 +9918,7 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="6" t="str">
-        <x:f>IF(Z44="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z44))</x:f>
+        <x:f>IF(Z44="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z44))</x:f>
       </x:c>
       <x:c r="B44" s="6" t="str">
         <x:v>R036</x:v>
@@ -10026,7 +10006,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD44" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE44" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10034,7 +10014,7 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="6" t="str">
-        <x:f>IF(Z45="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z45))</x:f>
+        <x:f>IF(Z45="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z45))</x:f>
       </x:c>
       <x:c r="B45" s="6" t="str">
         <x:v>R051</x:v>
@@ -10118,7 +10098,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD45" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE45" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -10126,7 +10106,7 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="6" t="str">
-        <x:f>IF(Z46="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z46))</x:f>
+        <x:f>IF(Z46="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z46))</x:f>
       </x:c>
       <x:c r="B46" s="6" t="str">
         <x:v>R016</x:v>
@@ -10214,7 +10194,7 @@
         <x:v>U3</x:v>
       </x:c>
       <x:c r="AD46" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE46" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10222,7 +10202,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="6" t="str">
-        <x:f>IF(Z47="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z47))</x:f>
+        <x:f>IF(Z47="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z47))</x:f>
       </x:c>
       <x:c r="B47" s="6" t="str">
         <x:v>R005</x:v>
@@ -10310,7 +10290,7 @@
         <x:v>G1</x:v>
       </x:c>
       <x:c r="AD47" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE47" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10318,7 +10298,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="6" t="str">
-        <x:f>IF(Z48="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z48))</x:f>
+        <x:f>IF(Z48="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z48))</x:f>
       </x:c>
       <x:c r="B48" s="6" t="str">
         <x:v>R031</x:v>
@@ -10406,7 +10386,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="AD48" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE48" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10414,7 +10394,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="6" t="str">
-        <x:f>IF(Z49="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z49))</x:f>
+        <x:f>IF(Z49="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z49))</x:f>
       </x:c>
       <x:c r="B49" s="6" t="str">
         <x:v>R037</x:v>
@@ -10502,7 +10482,7 @@
         <x:v>VL</x:v>
       </x:c>
       <x:c r="AD49" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE49" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10510,7 +10490,7 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="6" t="str">
-        <x:f>IF(Z50="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z50))</x:f>
+        <x:f>IF(Z50="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z50))</x:f>
       </x:c>
       <x:c r="B50" s="6" t="str">
         <x:v>R052</x:v>
@@ -10594,281 +10574,289 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="6" t="str">
-        <x:f>IF(Z51="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z51))</x:f>
+        <x:f>IF(Z51="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z51))</x:f>
       </x:c>
       <x:c r="B51" s="6" t="str">
-        <x:v>R009</x:v>
+        <x:v>R040</x:v>
       </x:c>
       <x:c r="C51" s="6" t="str">
-        <x:v>Tim Rocktäschel</x:v>
+        <x:v>Wenlong Huang</x:v>
       </x:c>
       <x:c r="D51" s="6" t="str">
-        <x:v>Europe</x:v>
+        <x:v>US</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:v>UCL / DeepMind</x:v>
+        <x:v>Stanford</x:v>
       </x:c>
       <x:c r="F51" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G51" s="6" t="str">
-        <x:v>No verified robot role</x:v>
+        <x:v>Planning</x:v>
       </x:c>
       <x:c r="H51" s="6" t="str">
-        <x:v>Video-first</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I51" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J51" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K51" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L51" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M51" s="6" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N51" s="6" t="str">
         <x:f>IF(AND(L51="Yes",M51="Yes"),"Yes","No")</x:f>
         <x:v>No</x:v>
       </x:c>
       <x:c r="O51" s="6" t="str">
-        <x:v>Genie</x:v>
+        <x:v>Generative planning</x:v>
       </x:c>
       <x:c r="P51" s="6" t="str">
-        <x:v>No verified robotics paper</x:v>
+        <x:v>Dream2Flow</x:v>
       </x:c>
       <x:c r="Q51" s="6" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="R51" s="6" t="str">
-        <x:v>Genie and open-ended embodied-agent work are relevant context, but no physical-robot paper was selected</x:v>
+        <x:v>Recent bridge; exact citation tracked via project page</x:v>
       </x:c>
       <x:c r="S51" s="6" t="str">
-        <x:v>https://rockt.ai/</x:v>
+        <x:v>https://wenlong.page/</x:v>
       </x:c>
       <x:c r="T51" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2402.15391</x:v>
-      </x:c>
-      <x:c r="U51" s="6"/>
+        <x:v>https://jiajunwu.com/</x:v>
+      </x:c>
+      <x:c r="U51" s="6" t="str">
+        <x:v>https://jiajunwu.com/</x:v>
+      </x:c>
       <x:c r="V51" s="6" t="str">
-        <x:v>P051</x:v>
+        <x:v>P026</x:v>
       </x:c>
       <x:c r="W51" s="6" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="X51" s="6"/>
-      <x:c r="Y51" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X51" s="6" t="str">
+        <x:v>P026</x:v>
+      </x:c>
+      <x:c r="Y51" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="Z51" s="15" t="str">
         <x:f>IF(AND(N51="Yes",AA51="Both distinct selected papers covered"),SQRT((W51+1)*(Y51+1))*IF(Q51="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA51" s="6" t="str">
-        <x:v>Partial / missing selected-paper coverage</x:v>
+        <x:v>Single bridge paper used on both sides</x:v>
       </x:c>
       <x:c r="AB51" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC51" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="AD51" s="6"/>
+        <x:v>G1</x:v>
+      </x:c>
+      <x:c r="AD51" s="6" t="str">
+        <x:v>Generated image/video</x:v>
+      </x:c>
       <x:c r="AE51" s="6" t="str">
-        <x:v>Partial evidence</x:v>
+        <x:v>Verified single-paper bridge; not ranked</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="6" t="str">
-        <x:f>IF(Z52="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z52))</x:f>
+        <x:f>IF(Z52="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z52))</x:f>
       </x:c>
       <x:c r="B52" s="6" t="str">
-        <x:v>R040</x:v>
+        <x:v>R030</x:v>
       </x:c>
       <x:c r="C52" s="6" t="str">
-        <x:v>Wenlong Huang</x:v>
+        <x:v>Xiaolong Wang</x:v>
       </x:c>
       <x:c r="D52" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>UC San Diego</x:v>
       </x:c>
       <x:c r="F52" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>U2</x:v>
       </x:c>
       <x:c r="G52" s="6" t="str">
-        <x:v>Planning</x:v>
+        <x:v>Reward / affordance</x:v>
       </x:c>
       <x:c r="H52" s="6" t="str">
-        <x:v>Bridger</x:v>
+        <x:v>Native hybrid</x:v>
       </x:c>
       <x:c r="I52" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J52" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K52" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L52" s="6" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M52" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N52" s="6" t="str">
         <x:f>IF(AND(L52="Yes",M52="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="O52" s="6" t="str">
-        <x:v>Generative planning</x:v>
+        <x:v>Unsupervised video representation</x:v>
       </x:c>
       <x:c r="P52" s="6" t="str">
-        <x:v>Dream2Flow</x:v>
+        <x:v>Robot learning from video</x:v>
       </x:c>
       <x:c r="Q52" s="6" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="R52" s="6" t="str">
-        <x:v>Recent bridge; exact citation tracked via project page</x:v>
+        <x:v>Motion/interaction understanding to robotics</x:v>
       </x:c>
       <x:c r="S52" s="6" t="str">
-        <x:v>https://wenlong.page/</x:v>
+        <x:v>https://xiaolonw.github.io/</x:v>
       </x:c>
       <x:c r="T52" s="6" t="str">
-        <x:v>https://jiajunwu.com/</x:v>
+        <x:v>https://arxiv.org/abs/1905.11993</x:v>
       </x:c>
       <x:c r="U52" s="6" t="str">
-        <x:v>https://jiajunwu.com/</x:v>
-      </x:c>
-      <x:c r="V52" s="6" t="str">
-        <x:v>P026</x:v>
-      </x:c>
-      <x:c r="W52" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="X52" s="6" t="str">
-        <x:v>P026</x:v>
-      </x:c>
-      <x:c r="Y52" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>https://arxiv.org/abs/2204.01691</x:v>
+      </x:c>
+      <x:c r="V52" s="6"/>
+      <x:c r="W52" s="6"/>
+      <x:c r="X52" s="6"/>
+      <x:c r="Y52" s="6"/>
       <x:c r="Z52" s="15" t="str">
         <x:f>IF(AND(N52="Yes",AA52="Both distinct selected papers covered"),SQRT((W52+1)*(Y52+1))*IF(Q52="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA52" s="6" t="str">
-        <x:v>Single bridge paper used on both sides</x:v>
+        <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB52" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC52" s="6" t="str">
-        <x:v>G1</x:v>
-      </x:c>
-      <x:c r="AD52" s="6" t="str">
-        <x:v>G1</x:v>
-      </x:c>
+      <x:c r="AC52" s="6"/>
+      <x:c r="AD52" s="6"/>
       <x:c r="AE52" s="6" t="str">
-        <x:v>Verified single-paper bridge; not ranked</x:v>
+        <x:v>Partial evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="6" t="str">
-        <x:f>IF(Z53="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z53))</x:f>
+        <x:f>IF(Z53="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z53))</x:f>
       </x:c>
       <x:c r="B53" s="6" t="str">
-        <x:v>R030</x:v>
+        <x:v>R019</x:v>
       </x:c>
       <x:c r="C53" s="6" t="str">
-        <x:v>Xiaolong Wang</x:v>
+        <x:v>Xun Huang</x:v>
       </x:c>
       <x:c r="D53" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E53" s="6" t="str">
-        <x:v>UC San Diego</x:v>
+        <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="F53" s="6" t="str">
-        <x:v>U2</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G53" s="6" t="str">
-        <x:v>Reward / affordance</x:v>
+        <x:v>World simulation</x:v>
       </x:c>
       <x:c r="H53" s="6" t="str">
-        <x:v>Native hybrid</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I53" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J53" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J53" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="K53" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L53" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="M53" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="N53" s="6" t="str">
         <x:f>IF(AND(L53="Yes",M53="Yes"),"Yes","No")</x:f>
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="O53" s="6" t="str">
-        <x:v>Unsupervised video representation</x:v>
+        <x:v>Video/image synthesis</x:v>
       </x:c>
       <x:c r="P53" s="6" t="str">
-        <x:v>Robot learning from video</x:v>
+        <x:v>Cosmos</x:v>
       </x:c>
       <x:c r="Q53" s="6" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="R53" s="6" t="str">
-        <x:v>Motion/interaction understanding to robotics</x:v>
+        <x:v>Generative backbone to physical-AI world models</x:v>
       </x:c>
       <x:c r="S53" s="6" t="str">
-        <x:v>https://xiaolonw.github.io/</x:v>
+        <x:v>https://xunhuang1995.github.io/</x:v>
       </x:c>
       <x:c r="T53" s="6" t="str">
-        <x:v>https://arxiv.org/abs/1905.11993</x:v>
+        <x:v>https://arxiv.org/abs/1808.06601</x:v>
       </x:c>
       <x:c r="U53" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2204.01691</x:v>
-      </x:c>
-      <x:c r="V53" s="6"/>
-      <x:c r="W53" s="6"/>
-      <x:c r="X53" s="6"/>
-      <x:c r="Y53" s="6"/>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
+      </x:c>
+      <x:c r="V53" s="6" t="str">
+        <x:v>P016</x:v>
+      </x:c>
+      <x:c r="W53" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="X53" s="6" t="str">
+        <x:v>P016</x:v>
+      </x:c>
+      <x:c r="Y53" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="Z53" s="15" t="str">
         <x:f>IF(AND(N53="Yes",AA53="Both distinct selected papers covered"),SQRT((W53+1)*(Y53+1))*IF(Q53="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA53" s="6" t="str">
-        <x:v>Partial / missing selected-paper coverage</x:v>
+        <x:v>Single bridge paper used on both sides</x:v>
       </x:c>
       <x:c r="AB53" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC53" s="6"/>
-      <x:c r="AD53" s="6"/>
+      <x:c r="AC53" s="6" t="str">
+        <x:v>G2</x:v>
+      </x:c>
+      <x:c r="AD53" s="6" t="str">
+        <x:v>Predicted future video/state</x:v>
+      </x:c>
       <x:c r="AE53" s="6" t="str">
-        <x:v>Partial evidence</x:v>
+        <x:v>Verified single-paper bridge; not ranked</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="6" t="str">
-        <x:f>IF(Z54="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z54))</x:f>
+        <x:f>IF(Z54="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z54))</x:f>
       </x:c>
       <x:c r="B54" s="6" t="str">
-        <x:v>R019</x:v>
+        <x:v>R023</x:v>
       </x:c>
       <x:c r="C54" s="6" t="str">
-        <x:v>Xun Huang</x:v>
+        <x:v>Yihuai Gao</x:v>
       </x:c>
       <x:c r="D54" s="6" t="str">
         <x:v>US</x:v>
@@ -10886,7 +10874,7 @@
         <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I54" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J54" s="6" t="n">
         <x:v>1</x:v>
@@ -10895,7 +10883,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="L54" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M54" s="6" t="str">
         <x:v>Emerging</x:v>
@@ -10905,22 +10893,22 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="O54" s="6" t="str">
-        <x:v>Video/image synthesis</x:v>
+        <x:v>Cosmos</x:v>
       </x:c>
       <x:c r="P54" s="6" t="str">
-        <x:v>Cosmos</x:v>
+        <x:v>Cosmos robotics applications</x:v>
       </x:c>
       <x:c r="Q54" s="6" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="R54" s="6" t="str">
-        <x:v>Generative backbone to physical-AI world models</x:v>
+        <x:v>Recent bridge; impact still maturing</x:v>
       </x:c>
       <x:c r="S54" s="6" t="str">
-        <x:v>https://xunhuang1995.github.io/</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="T54" s="6" t="str">
-        <x:v>https://arxiv.org/abs/1808.06601</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="U54" s="6" t="str">
         <x:v>https://arxiv.org/abs/2501.03575</x:v>
@@ -10950,7 +10938,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD54" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE54" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10958,80 +10946,80 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="6" t="str">
-        <x:f>IF(Z55="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z55))</x:f>
+        <x:f>IF(Z55="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z55))</x:f>
       </x:c>
       <x:c r="B55" s="6" t="str">
-        <x:v>R023</x:v>
+        <x:v>R056</x:v>
       </x:c>
       <x:c r="C55" s="6" t="str">
-        <x:v>Yihuai Gao</x:v>
+        <x:v>Yuke Zhu</x:v>
       </x:c>
       <x:c r="D55" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E55" s="6" t="str">
-        <x:v>NVIDIA</x:v>
+        <x:v>UT Austin / NVIDIA</x:v>
       </x:c>
       <x:c r="F55" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>VL</x:v>
       </x:c>
       <x:c r="G55" s="6" t="str">
-        <x:v>World simulation</x:v>
+        <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="H55" s="6" t="str">
-        <x:v>Bridger</x:v>
+        <x:v>Native hybrid</x:v>
       </x:c>
       <x:c r="I55" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J55" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="J55" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="K55" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L55" s="6" t="str">
         <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M55" s="6" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N55" s="6" t="str">
         <x:f>IF(AND(L55="Yes",M55="Yes"),"Yes","No")</x:f>
         <x:v>No</x:v>
       </x:c>
       <x:c r="O55" s="6" t="str">
-        <x:v>Cosmos</x:v>
+        <x:v>Multimodal representation</x:v>
       </x:c>
       <x:c r="P55" s="6" t="str">
-        <x:v>Cosmos robotics applications</x:v>
+        <x:v>VIMA; robot learning</x:v>
       </x:c>
       <x:c r="Q55" s="6" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="R55" s="6" t="str">
-        <x:v>Recent bridge; impact still maturing</x:v>
+        <x:v>Robotics-led hybrid/control case</x:v>
       </x:c>
       <x:c r="S55" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
+        <x:v>https://www.cs.utexas.edu/~yukez/</x:v>
       </x:c>
       <x:c r="T55" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
+        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
       </x:c>
       <x:c r="U55" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
+        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
       </x:c>
       <x:c r="V55" s="6" t="str">
-        <x:v>P016</x:v>
+        <x:v>P019</x:v>
       </x:c>
       <x:c r="W55" s="6" t="n">
-        <x:v>10</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="X55" s="6" t="str">
-        <x:v>P016</x:v>
+        <x:v>P019</x:v>
       </x:c>
       <x:c r="Y55" s="6" t="n">
-        <x:v>10</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="Z55" s="15" t="str">
         <x:f>IF(AND(N55="Yes",AA55="Both distinct selected papers covered"),SQRT((W55+1)*(Y55+1))*IF(Q55="High",1,0.8),"")</x:f>
@@ -11043,10 +11031,10 @@
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC55" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="AD55" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE55" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -11054,19 +11042,19 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="6" t="str">
-        <x:f>IF(Z56="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z56))</x:f>
+        <x:f>IF(Z56="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z56))</x:f>
       </x:c>
       <x:c r="B56" s="6" t="str">
-        <x:v>R056</x:v>
+        <x:v>R054</x:v>
       </x:c>
       <x:c r="C56" s="6" t="str">
-        <x:v>Yuke Zhu</x:v>
+        <x:v>Yunfan Jiang</x:v>
       </x:c>
       <x:c r="D56" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E56" s="6" t="str">
-        <x:v>UT Austin / NVIDIA</x:v>
+        <x:v>Stanford / NVIDIA</x:v>
       </x:c>
       <x:c r="F56" s="6" t="str">
         <x:v>VL</x:v>
@@ -11075,7 +11063,7 @@
         <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="H56" s="6" t="str">
-        <x:v>Native hybrid</x:v>
+        <x:v>Robotics-first</x:v>
       </x:c>
       <x:c r="I56" s="6" t="n">
         <x:v>0</x:v>
@@ -11097,19 +11085,19 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="O56" s="6" t="str">
-        <x:v>Multimodal representation</x:v>
+        <x:v>Multimodal prompts</x:v>
       </x:c>
       <x:c r="P56" s="6" t="str">
-        <x:v>VIMA; robot learning</x:v>
+        <x:v>VIMA</x:v>
       </x:c>
       <x:c r="Q56" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R56" s="6" t="str">
-        <x:v>Robotics-led hybrid/control case</x:v>
+        <x:v>Key VIMA author; not a clear video-first trajectory</x:v>
       </x:c>
       <x:c r="S56" s="6" t="str">
-        <x:v>https://www.cs.utexas.edu/~yukez/</x:v>
+        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
       </x:c>
       <x:c r="T56" s="6" t="str">
         <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
@@ -11142,7 +11130,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="AD56" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE56" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -11150,80 +11138,80 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="6" t="str">
-        <x:f>IF(Z57="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z57))</x:f>
+        <x:f>IF(Z57="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z57))</x:f>
       </x:c>
       <x:c r="B57" s="6" t="str">
-        <x:v>R054</x:v>
+        <x:v>R022</x:v>
       </x:c>
       <x:c r="C57" s="6" t="str">
-        <x:v>Yunfan Jiang</x:v>
+        <x:v>Yunhao Ge</x:v>
       </x:c>
       <x:c r="D57" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E57" s="6" t="str">
-        <x:v>Stanford / NVIDIA</x:v>
+        <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="F57" s="6" t="str">
-        <x:v>VL</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G57" s="6" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>World simulation</x:v>
       </x:c>
       <x:c r="H57" s="6" t="str">
-        <x:v>Robotics-first</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I57" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J57" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="K57" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L57" s="6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M57" s="6" t="str">
         <x:v>Emerging</x:v>
-      </x:c>
-      <x:c r="M57" s="6" t="str">
-        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N57" s="6" t="str">
         <x:f>IF(AND(L57="Yes",M57="Yes"),"Yes","No")</x:f>
         <x:v>No</x:v>
       </x:c>
       <x:c r="O57" s="6" t="str">
-        <x:v>Multimodal prompts</x:v>
+        <x:v>Generative visual models</x:v>
       </x:c>
       <x:c r="P57" s="6" t="str">
-        <x:v>VIMA</x:v>
+        <x:v>Cosmos</x:v>
       </x:c>
       <x:c r="Q57" s="6" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="R57" s="6" t="str">
-        <x:v>Key VIMA author; not a clear video-first trajectory</x:v>
+        <x:v>Physical-AI model development</x:v>
       </x:c>
       <x:c r="S57" s="6" t="str">
-        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
+        <x:v>https://scholar.google.com/scholar?q=Yunhao+Ge+NVIDIA+Cosmos</x:v>
       </x:c>
       <x:c r="T57" s="6" t="str">
-        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="U57" s="6" t="str">
-        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="V57" s="6" t="str">
-        <x:v>P019</x:v>
+        <x:v>P016</x:v>
       </x:c>
       <x:c r="W57" s="6" t="n">
-        <x:v>65</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X57" s="6" t="str">
-        <x:v>P019</x:v>
+        <x:v>P016</x:v>
       </x:c>
       <x:c r="Y57" s="6" t="n">
-        <x:v>65</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="Z57" s="15" t="str">
         <x:f>IF(AND(N57="Yes",AA57="Both distinct selected papers covered"),SQRT((W57+1)*(Y57+1))*IF(Q57="High",1,0.8),"")</x:f>
@@ -11235,110 +11223,47 @@
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC57" s="6" t="str">
-        <x:v>None</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="AD57" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE57" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="6" t="str">
-        <x:f>IF(Z58="","",1+COUNTIF($Z$2:$Z$58,"&gt;"&amp;Z58))</x:f>
-      </x:c>
-      <x:c r="B58" s="6" t="str">
-        <x:v>R022</x:v>
-      </x:c>
-      <x:c r="C58" s="6" t="str">
-        <x:v>Yunhao Ge</x:v>
-      </x:c>
-      <x:c r="D58" s="6" t="str">
-        <x:v>US</x:v>
-      </x:c>
-      <x:c r="E58" s="6" t="str">
-        <x:v>NVIDIA</x:v>
-      </x:c>
-      <x:c r="F58" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="G58" s="6" t="str">
-        <x:v>World simulation</x:v>
-      </x:c>
-      <x:c r="H58" s="6" t="str">
-        <x:v>Bridger</x:v>
-      </x:c>
-      <x:c r="I58" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J58" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K58" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="L58" s="6" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="M58" s="6" t="str">
-        <x:v>Emerging</x:v>
-      </x:c>
-      <x:c r="N58" s="6" t="str">
-        <x:f>IF(AND(L58="Yes",M58="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="O58" s="6" t="str">
-        <x:v>Generative visual models</x:v>
-      </x:c>
-      <x:c r="P58" s="6" t="str">
-        <x:v>Cosmos</x:v>
-      </x:c>
-      <x:c r="Q58" s="6" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="R58" s="6" t="str">
-        <x:v>Physical-AI model development</x:v>
-      </x:c>
-      <x:c r="S58" s="6" t="str">
-        <x:v>https://scholar.google.com/scholar?q=Yunhao+Ge+NVIDIA+Cosmos</x:v>
-      </x:c>
-      <x:c r="T58" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
-      </x:c>
-      <x:c r="U58" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
-      </x:c>
-      <x:c r="V58" s="6" t="str">
-        <x:v>P016</x:v>
-      </x:c>
-      <x:c r="W58" s="6" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="X58" s="6" t="str">
-        <x:v>P016</x:v>
-      </x:c>
-      <x:c r="Y58" s="6" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="Z58" s="15" t="str">
-        <x:f>IF(AND(N58="Yes",AA58="Both distinct selected papers covered"),SQRT((W58+1)*(Y58+1))*IF(Q58="High",1,0.8),"")</x:f>
-      </x:c>
-      <x:c r="AA58" s="6" t="str">
-        <x:v>Single bridge paper used on both sides</x:v>
-      </x:c>
-      <x:c r="AB58" s="6" t="str">
-        <x:v>2026-09-02</x:v>
-      </x:c>
-      <x:c r="AC58" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="AD58" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="AE58" s="6" t="str">
-        <x:v>Verified single-paper bridge; not ranked</x:v>
-      </x:c>
+      <x:c r="A58"/>
+      <x:c r="B58"/>
+      <x:c r="C58"/>
+      <x:c r="D58"/>
+      <x:c r="E58"/>
+      <x:c r="F58"/>
+      <x:c r="G58"/>
+      <x:c r="H58"/>
+      <x:c r="I58"/>
+      <x:c r="J58"/>
+      <x:c r="K58"/>
+      <x:c r="L58"/>
+      <x:c r="M58"/>
+      <x:c r="N58"/>
+      <x:c r="O58"/>
+      <x:c r="P58"/>
+      <x:c r="Q58"/>
+      <x:c r="R58"/>
+      <x:c r="S58"/>
+      <x:c r="T58"/>
+      <x:c r="U58"/>
+      <x:c r="V58"/>
+      <x:c r="W58"/>
+      <x:c r="X58"/>
+      <x:c r="Y58"/>
+      <x:c r="Z58"/>
+      <x:c r="AA58"/>
+      <x:c r="AB58"/>
+      <x:c r="AC58"/>
+      <x:c r="AD58"/>
+      <x:c r="AE58"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="N2:N58">
@@ -11346,7 +11271,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17b2e8125d48479e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb16bcf1f2b045f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11367,7 +11292,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Researcher origin mechanism × primary robot role</x:v>
+        <x:v>Researchers: unified video-origin code × primary robot role</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -11377,6 +11302,24 @@
       <x:c r="G1" s="3"/>
       <x:c r="H1" s="3"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+    </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
         <x:v>Origin</x:v>
@@ -11399,9 +11342,7 @@
       <x:c r="G4" s="14" t="str">
         <x:v>Direct policy</x:v>
       </x:c>
-      <x:c r="H4" s="12" t="str">
-        <x:v>No verified robot role</x:v>
-      </x:c>
+      <x:c r="H4" s="12"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="6" t="str">
@@ -11425,9 +11366,7 @@
       <x:c r="G5" s="17" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H5" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H5" s="17"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="6" t="str">
@@ -11451,9 +11390,7 @@
       <x:c r="G6" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H6" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H6" s="17"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="6" t="str">
@@ -11477,9 +11414,7 @@
       <x:c r="G7" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H7" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H7" s="17"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="6" t="str">
@@ -11503,9 +11438,7 @@
       <x:c r="G8" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H8" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H8" s="17"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6" t="str">
@@ -11529,9 +11462,7 @@
       <x:c r="G9" s="17" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H9" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H9" s="17"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="6" t="str">
@@ -11555,9 +11486,7 @@
       <x:c r="G10" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H10" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H10" s="17"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="6" t="str">
@@ -11581,9 +11510,7 @@
       <x:c r="G11" s="17" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H11" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H11" s="17"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6" t="str">
@@ -11607,11 +11534,10 @@
       <x:c r="G12" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H12" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H12" s="17"/>
     </x:row>
     <x:row r="13">
+      <x:c r="A13"/>
       <x:c r="B13" s="18"/>
       <x:c r="C13" s="18"/>
       <x:c r="D13" s="18"/>
@@ -11622,7 +11548,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="3" t="str">
-        <x:v>Direct bridge papers: video mechanism × robot role</x:v>
+        <x:v>Direct bridge papers: same video-origin code × robot role</x:v>
       </x:c>
       <x:c r="B14" s="19"/>
       <x:c r="C14" s="19"/>
@@ -11633,6 +11559,7 @@
       <x:c r="H14" s="18"/>
     </x:row>
     <x:row r="15">
+      <x:c r="A15"/>
       <x:c r="B15" s="18"/>
       <x:c r="C15" s="18"/>
       <x:c r="D15" s="18"/>
@@ -11643,7 +11570,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="11" t="str">
-        <x:v>Mechanism</x:v>
+        <x:v>Origin</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
         <x:v>Perception backbone</x:v>
@@ -11858,211 +11785,111 @@
       <x:c r="H24" s="18"/>
     </x:row>
     <x:row r="25">
-      <x:c r="B25" s="18"/>
-      <x:c r="C25" s="18"/>
-      <x:c r="D25" s="18"/>
-      <x:c r="E25" s="18"/>
-      <x:c r="F25" s="18"/>
-      <x:c r="G25" s="18"/>
-      <x:c r="H25" s="18"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
+      <x:c r="G25"/>
+      <x:c r="H25"/>
     </x:row>
     <x:row r="26">
-      <x:c r="B26" s="18"/>
-      <x:c r="C26" s="18"/>
-      <x:c r="D26" s="18"/>
-      <x:c r="E26" s="18"/>
-      <x:c r="F26" s="18"/>
-      <x:c r="G26" s="18"/>
-      <x:c r="H26" s="18"/>
+      <x:c r="B26"/>
+      <x:c r="C26"/>
+      <x:c r="D26"/>
+      <x:c r="E26"/>
+      <x:c r="F26"/>
+      <x:c r="G26"/>
+      <x:c r="H26"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="3" t="str">
-        <x:v>Direct bridge papers: focal output × robot role</x:v>
-      </x:c>
-      <x:c r="B27" s="19"/>
-      <x:c r="C27" s="19"/>
-      <x:c r="D27" s="19"/>
-      <x:c r="E27" s="19"/>
-      <x:c r="F27" s="19"/>
-      <x:c r="G27" s="19"/>
-      <x:c r="H27" s="18"/>
+      <x:c r="A27"/>
+      <x:c r="B27"/>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
+      <x:c r="G27"/>
+      <x:c r="H27"/>
     </x:row>
     <x:row r="28">
-      <x:c r="B28" s="18"/>
-      <x:c r="C28" s="18"/>
-      <x:c r="D28" s="18"/>
-      <x:c r="E28" s="18"/>
-      <x:c r="F28" s="18"/>
-      <x:c r="G28" s="18"/>
-      <x:c r="H28" s="18"/>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="11" t="str">
-        <x:v>Output</x:v>
-      </x:c>
-      <x:c r="B29" s="16" t="str">
-        <x:v>Perception backbone</x:v>
-      </x:c>
-      <x:c r="C29" s="16" t="str">
-        <x:v>Reward / affordance</x:v>
-      </x:c>
-      <x:c r="D29" s="16" t="str">
-        <x:v>Data generation</x:v>
-      </x:c>
-      <x:c r="E29" s="16" t="str">
-        <x:v>World simulation</x:v>
-      </x:c>
-      <x:c r="F29" s="16" t="str">
-        <x:v>Planning</x:v>
-      </x:c>
-      <x:c r="G29" s="20" t="str">
-        <x:v>Direct policy</x:v>
-      </x:c>
-      <x:c r="H29" s="18"/>
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="6" t="str">
-        <x:v>G1</x:v>
-      </x:c>
-      <x:c r="B30" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C30" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D30" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E30" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F30" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G30" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H30" s="18"/>
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="B31" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C31" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D31" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E31" s="17" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="F31" s="17" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G31" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H31" s="18"/>
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31"/>
+      <x:c r="F31"/>
+      <x:c r="G31"/>
+      <x:c r="H31"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="6" t="str">
-        <x:v>G3</x:v>
-      </x:c>
-      <x:c r="B32" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C32" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D32" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E32" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F32" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G32" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H32" s="18"/>
+      <x:c r="A32"/>
+      <x:c r="B32"/>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
+      <x:c r="E32"/>
+      <x:c r="F32"/>
+      <x:c r="G32"/>
+      <x:c r="H32"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="6" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="B33" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C33" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D33" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E33" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F33" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G33" s="17" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H33" s="18"/>
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33"/>
+      <x:c r="F33"/>
+      <x:c r="G33"/>
+      <x:c r="H33"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="6" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="B34" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C34" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D34" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E34" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F34" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G34" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H34" s="18"/>
+      <x:c r="A34"/>
+      <x:c r="B34"/>
+      <x:c r="C34"/>
+      <x:c r="D34"/>
+      <x:c r="E34"/>
+      <x:c r="F34"/>
+      <x:c r="G34"/>
+      <x:c r="H34"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="6" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="B35" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C35" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D35" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E35" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F35" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G35" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H35" s="18"/>
+      <x:c r="A35"/>
+      <x:c r="B35"/>
+      <x:c r="C35"/>
+      <x:c r="D35"/>
+      <x:c r="E35"/>
+      <x:c r="F35"/>
+      <x:c r="G35"/>
+      <x:c r="H35"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -12090,6 +11917,16 @@
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+    </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
         <x:v>Transition type</x:v>
@@ -12109,7 +11946,8 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C5" s="21" t="n">
-        <x:v>0.03508771929824561</x:v>
+        <x:f>B5/SUM($B$5:$B$8)</x:f>
+        <x:v>0.03571428571428571</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -12120,7 +11958,8 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="C6" s="21" t="n">
-        <x:v>0.6842105263157895</x:v>
+        <x:f>B6/SUM($B$5:$B$8)</x:f>
+        <x:v>0.6964285714285714</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -12131,7 +11970,8 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="C7" s="21" t="n">
-        <x:v>0.19298245614035087</x:v>
+        <x:f>B7/SUM($B$5:$B$8)</x:f>
+        <x:v>0.19642857142857142</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -12142,19 +11982,14 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C8" s="21" t="n">
-        <x:v>0.07017543859649122</x:v>
+        <x:f>B8/SUM($B$5:$B$8)</x:f>
+        <x:v>0.07142857142857142</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="6" t="str">
-        <x:v>Video-first</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C9" s="21" t="n">
-        <x:v>0.017543859649122806</x:v>
-      </x:c>
+      <x:c r="A9"/>
+      <x:c r="B9"/>
+      <x:c r="C9"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -12200,20 +12035,23 @@
       <x:c r="B4" s="12" t="str">
         <x:v>Value</x:v>
       </x:c>
+      <x:c r="C4"/>
       <x:c r="D4" s="11" t="str">
-        <x:v>Origin mechanism</x:v>
+        <x:v>Origin code</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
         <x:v>Researchers</x:v>
       </x:c>
+      <x:c r="F4"/>
       <x:c r="G4" s="11" t="str">
         <x:v>Transition type</x:v>
       </x:c>
       <x:c r="H4" s="12" t="str">
         <x:v>Researchers</x:v>
       </x:c>
+      <x:c r="I4"/>
       <x:c r="J4" s="11" t="str">
-        <x:v>Direct bridge output</x:v>
+        <x:v>Direct paper origin</x:v>
       </x:c>
       <x:c r="K4" s="12" t="str">
         <x:v>Papers</x:v>
@@ -12224,20 +12062,23 @@
         <x:v>Researchers</x:v>
       </x:c>
       <x:c r="B5" s="6" t="n">
-        <x:v>57</x:v>
-      </x:c>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C5"/>
       <x:c r="D5" s="6" t="str">
         <x:v>G1</x:v>
       </x:c>
       <x:c r="E5" s="6" t="n">
         <x:v>13</x:v>
       </x:c>
+      <x:c r="F5"/>
       <x:c r="G5" s="6" t="str">
         <x:v>Switcher</x:v>
       </x:c>
       <x:c r="H5" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="I5"/>
       <x:c r="J5" s="6" t="str">
         <x:v>G1</x:v>
       </x:c>
@@ -12252,23 +12093,26 @@
       <x:c r="B6" s="6" t="n">
         <x:v>66</x:v>
       </x:c>
+      <x:c r="C6"/>
       <x:c r="D6" s="6" t="str">
         <x:v>G2</x:v>
       </x:c>
       <x:c r="E6" s="6" t="n">
-        <x:v>13</x:v>
-      </x:c>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F6"/>
       <x:c r="G6" s="6" t="str">
         <x:v>Bridger</x:v>
       </x:c>
       <x:c r="H6" s="6" t="n">
         <x:v>39</x:v>
       </x:c>
+      <x:c r="I6"/>
       <x:c r="J6" s="6" t="str">
         <x:v>G2</x:v>
       </x:c>
       <x:c r="K6" s="6" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -12278,18 +12122,21 @@
       <x:c r="B7" s="6" t="n">
         <x:v>31</x:v>
       </x:c>
+      <x:c r="C7"/>
       <x:c r="D7" s="6" t="str">
         <x:v>G3</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F7"/>
       <x:c r="G7" s="6" t="str">
         <x:v>Native hybrid</x:v>
       </x:c>
       <x:c r="H7" s="6" t="n">
         <x:v>11</x:v>
       </x:c>
+      <x:c r="I7"/>
       <x:c r="J7" s="6" t="str">
         <x:v>G3</x:v>
       </x:c>
@@ -12304,23 +12151,26 @@
       <x:c r="B8" s="6" t="n">
         <x:v>22</x:v>
       </x:c>
+      <x:c r="C8"/>
       <x:c r="D8" s="6" t="str">
         <x:v>U1</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="F8"/>
       <x:c r="G8" s="6" t="str">
         <x:v>Robotics-first</x:v>
       </x:c>
       <x:c r="H8" s="6" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="I8"/>
       <x:c r="J8" s="6" t="str">
-        <x:v>A</x:v>
+        <x:v>U1</x:v>
       </x:c>
       <x:c r="K8" s="6" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -12330,23 +12180,22 @@
       <x:c r="B9" s="6" t="n">
         <x:v>13</x:v>
       </x:c>
+      <x:c r="C9"/>
       <x:c r="D9" s="6" t="str">
         <x:v>U2</x:v>
       </x:c>
       <x:c r="E9" s="6" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="G9" s="6" t="str">
-        <x:v>Video-first</x:v>
-      </x:c>
-      <x:c r="H9" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="F9"/>
+      <x:c r="G9" s="6"/>
+      <x:c r="H9" s="6"/>
+      <x:c r="I9"/>
       <x:c r="J9" s="6" t="str">
-        <x:v>R</x:v>
+        <x:v>U2</x:v>
       </x:c>
       <x:c r="K9" s="6" t="n">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -12356,14 +12205,19 @@
       <x:c r="B10" s="6" t="n">
         <x:v>20</x:v>
       </x:c>
+      <x:c r="C10"/>
       <x:c r="D10" s="6" t="str">
         <x:v>U3</x:v>
       </x:c>
       <x:c r="E10" s="6" t="n">
         <x:v>8</x:v>
       </x:c>
+      <x:c r="F10"/>
+      <x:c r="G10"/>
+      <x:c r="H10"/>
+      <x:c r="I10"/>
       <x:c r="J10" s="6" t="str">
-        <x:v>D</x:v>
+        <x:v>U3</x:v>
       </x:c>
       <x:c r="K10" s="6" t="n">
         <x:v>1</x:v>
@@ -12376,11 +12230,22 @@
       <x:c r="B11" s="6" t="n">
         <x:v>22</x:v>
       </x:c>
+      <x:c r="C11"/>
       <x:c r="D11" s="6" t="str">
         <x:v>VL</x:v>
       </x:c>
       <x:c r="E11" s="6" t="n">
         <x:v>6</x:v>
+      </x:c>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11"/>
+      <x:c r="I11"/>
+      <x:c r="J11" t="str">
+        <x:v>VL</x:v>
+      </x:c>
+      <x:c r="K11" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -12388,14 +12253,51 @@
         <x:v>Partial evidence rows</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n">
-        <x:v>11</x:v>
-      </x:c>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C12"/>
       <x:c r="D12" s="6" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="E12" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
+      <x:c r="I12"/>
+      <x:c r="J12" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="K12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
+      <x:c r="K13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
+      <x:c r="K14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="30" t="str">
@@ -12414,7 +12316,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="str">
-        <x:v>• Architecture is no longer a single mixed column: video mechanism, focal output, and robot role are separate.</x:v>
+        <x:v>• One code axis maps video-origin architecture directly to robot role; model output is descriptive metadata, not a second code system.</x:v>
       </x:c>
       <x:c r="B16" s="6"/>
       <x:c r="C16" s="6"/>
@@ -12429,7 +12331,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="str">
-        <x:v>• Bridge Impact requires two distinct authored papers; a single bridge paper is useful evidence but is not counted twice.</x:v>
+        <x:v>• G1 researchers map mainly to planning (6), direct policy (4), and world simulation (3).</x:v>
       </x:c>
       <x:c r="B17" s="6"/>
       <x:c r="C17" s="6"/>
@@ -12444,7 +12346,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="str">
-        <x:v>• Dream2Flow is G1 and PointWorld is G2 under the output/action-position rule.</x:v>
+        <x:v>• Bridge Impact requires two distinct authored papers; single-paper bridges remain documented but are not ranked.</x:v>
       </x:c>
       <x:c r="B18" s="6"/>
       <x:c r="C18" s="6"/>
@@ -12459,7 +12361,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="6" t="str">
-        <x:v>• RoboCat, Gemini Robotics, VIMA, and image-only SuSIE are adjacent context rather than direct video-model bridge papers.</x:v>
+        <x:v>• Tim Rocktäschel is excluded from the researcher sample because no physical-robot paper was verified; Genie remains a context paper.</x:v>
       </x:c>
       <x:c r="B19" s="6"/>
       <x:c r="C19" s="6"/>
@@ -12633,16 +12535,16 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6" t="str">
-        <x:v>Citation source</x:v>
+        <x:v>Tim Rocktäschel</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>Mixed scholarly-web snapshot</x:v>
+        <x:v>Video-first comparison inside researcher sample</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str">
-        <x:v>OpenAlex cited_by_count</x:v>
+        <x:v>Excluded from researcher sample; Genie retained as context</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:v>One explicit source and one snapshot date; values remain source-specific</x:v>
+        <x:v>No physical-robot paper was verified; virtual world-model and agent work alone does not meet the researcher inclusion rule</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Remove robotics-only controls from the transition sample
</commit_message>
<xml_diff>
--- a/notes/01-video-to-robotics-transition/video_to_robotics_architecture_pilot.xlsx
+++ b/notes/01-video-to-robotics-transition/video_to_robotics_architecture_pilot.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Method" sheetId="1" r:id="R03443d765dbd4125"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="Ra95937d9b828454a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="3" r:id="Re806c23774eb47ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Researchers" sheetId="4" r:id="R002a0634677046c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Matrix" sheetId="5" r:id="R8f6491d6504c40cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transition_Matrix" sheetId="6" r:id="R65e40ab97d1e410f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="7" r:id="R765f756fbc334669"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_Log" sheetId="8" r:id="R916f27f12b4a43f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Method" sheetId="1" r:id="Rfafdc1d82d9a4115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="R3f4e1ade273d4524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="3" r:id="R48968dc1a6cf4bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Researchers" sheetId="4" r:id="R5f30fdb061604d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Matrix" sheetId="5" r:id="Ree4cfeae9316496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transition_Matrix" sheetId="6" r:id="R97161d55068749d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="7" r:id="Rf732c25c2b484e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_Log" sheetId="8" r:id="R7cfe380a4be24bc0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -53,8 +53,24 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF19324D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF19324D"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -69,6 +85,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF2D6F9F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF19324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3378A8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF19324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3378A8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -108,7 +154,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="65">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -188,6 +234,78 @@
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -243,7 +361,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResearchersTable" displayName="ResearchersTable" ref="A1:AE57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResearchersTable" displayName="ResearchersTable" ref="A1:AE53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="31">
     <x:tableColumn id="1" name="Impact_rank"/>
     <x:tableColumn id="2" name="Researcher_ID"/>
@@ -515,7 +633,7 @@
         <x:v>Sample</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>56 researchers and 66 papers in separate, non-1:1 tables; 31 direct bridge, 22 adjacent/context, 13 one-side reference papers</x:v>
+        <x:v>52 researchers and 66 papers in separate, non-1:1 tables; 31 direct bridge, 22 adjacent/context, 13 one-side reference papers</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -579,7 +697,7 @@
         <x:v>Audit correction</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
-        <x:v>Dream2Flow is G1; PointWorld is G2; CALVIN is a benchmark; Tim Rocktäschel is excluded from the researcher sample while Genie remains context</x:v>
+        <x:v>Dream2Flow is G1; PointWorld is G2; CALVIN is a benchmark; four robotics-centered comparison cases were excluded from the core researcher sample; Genie remains context</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -789,112 +907,92 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
-      <x:c r="B12" s="6" t="str">
-        <x:v>Unified video-origin code</x:v>
-      </x:c>
-      <x:c r="C12" s="6" t="str">
-        <x:v>No verified video-specific research mechanism</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="str">
-        <x:v>RoboCat, RT-2</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="str">
-        <x:v>comparison</x:v>
-      </x:c>
-      <x:c r="F12" s="6" t="str">
-        <x:v>Robotics evidence alone is not a video bridge</x:v>
-      </x:c>
+      <x:c r="A12" s="6"/>
+      <x:c r="B12" s="6"/>
+      <x:c r="C12" s="6"/>
+      <x:c r="D12" s="6"/>
+      <x:c r="E12" s="6"/>
+      <x:c r="F12" s="6"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="6"/>
-      <x:c r="B13" s="6"/>
-      <x:c r="C13" s="6"/>
-      <x:c r="D13" s="6"/>
+      <x:c r="A13" s="6" t="str">
+        <x:v>Transition type</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>Meaning</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>Use</x:v>
+      </x:c>
       <x:c r="E13" s="6"/>
       <x:c r="F13" s="6"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="6" t="str">
-        <x:v>Transition type</x:v>
+        <x:v>Switcher</x:v>
       </x:c>
       <x:c r="B14" s="6" t="str">
-        <x:v>Rule</x:v>
+        <x:v>Organization or primary topic clearly moved video → robotics/world models</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str">
-        <x:v>Meaning</x:v>
+        <x:v>strong migration</x:v>
       </x:c>
       <x:c r="D14" s="6" t="str">
-        <x:v>Use</x:v>
+        <x:v>strict transition count</x:v>
       </x:c>
       <x:c r="E14" s="6"/>
       <x:c r="F14" s="6"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="11" t="str">
-        <x:v>Switcher</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>Organization or primary topic clearly moved video → robotics/world models</x:v>
+        <x:v>Verified important work on both sides or explicit transfer across papers</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>strong migration</x:v>
+        <x:v>core bridge</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>strict transition count</x:v>
+        <x:v>bridge-talent count</x:v>
       </x:c>
       <x:c r="E15" s="14"/>
       <x:c r="F15" s="12"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="str">
-        <x:v>Bridger</x:v>
+        <x:v>Native hybrid</x:v>
       </x:c>
       <x:c r="B16" s="6" t="str">
-        <x:v>Verified important work on both sides or explicit transfer across papers</x:v>
+        <x:v>Video and robotics pursued together from an early stage</x:v>
       </x:c>
       <x:c r="C16" s="6" t="str">
-        <x:v>core bridge</x:v>
+        <x:v>fusion rather than migration</x:v>
       </x:c>
       <x:c r="D16" s="6" t="str">
-        <x:v>bridge-talent count</x:v>
+        <x:v>ecosystem count</x:v>
       </x:c>
       <x:c r="E16" s="6"/>
       <x:c r="F16" s="6"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="6" t="str">
-        <x:v>Native hybrid</x:v>
-      </x:c>
-      <x:c r="B17" s="6" t="str">
-        <x:v>Video and robotics pursued together from an early stage</x:v>
-      </x:c>
-      <x:c r="C17" s="6" t="str">
-        <x:v>fusion rather than migration</x:v>
-      </x:c>
-      <x:c r="D17" s="6" t="str">
-        <x:v>ecosystem count</x:v>
-      </x:c>
-      <x:c r="E17" s="6"/>
-      <x:c r="F17" s="6"/>
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="6" t="str">
-        <x:v>Robotics-first</x:v>
-      </x:c>
-      <x:c r="B18" s="6" t="str">
-        <x:v>Robotics-centered comparison with no verified video-origin paper</x:v>
-      </x:c>
-      <x:c r="C18" s="6" t="str">
-        <x:v>control group</x:v>
-      </x:c>
-      <x:c r="D18" s="6" t="str">
-        <x:v>overclaim check</x:v>
-      </x:c>
-      <x:c r="E18" s="6"/>
-      <x:c r="F18" s="6"/>
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19"/>
@@ -3270,9 +3368,7 @@
       <x:c r="F33" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G33" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G33" s="6"/>
       <x:c r="H33" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -3412,9 +3508,7 @@
       <x:c r="F35" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G35" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G35" s="6"/>
       <x:c r="H35" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -3625,9 +3719,7 @@
       <x:c r="F38" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G38" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G38" s="6"/>
       <x:c r="H38" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -3771,9 +3863,7 @@
       <x:c r="F40" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G40" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G40" s="6"/>
       <x:c r="H40" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -4199,9 +4289,7 @@
       <x:c r="F46" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G46" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G46" s="6"/>
       <x:c r="H46" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -4272,9 +4360,7 @@
       <x:c r="F47" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G47" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G47" s="6"/>
       <x:c r="H47" s="6" t="str">
         <x:v>Dataset/benchmark</x:v>
       </x:c>
@@ -4629,9 +4715,7 @@
       <x:c r="F52" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G52" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G52" s="6"/>
       <x:c r="H52" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -4856,9 +4940,7 @@
       <x:c r="J55" s="6" t="str">
         <x:v>Optical flow</x:v>
       </x:c>
-      <x:c r="K55" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K55" s="6"/>
       <x:c r="L55" s="6" t="str">
         <x:v>Landmark</x:v>
       </x:c>
@@ -4927,9 +5009,7 @@
       <x:c r="J56" s="6" t="str">
         <x:v>Semantic features</x:v>
       </x:c>
-      <x:c r="K56" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K56" s="6"/>
       <x:c r="L56" s="6" t="str">
         <x:v>Landmark</x:v>
       </x:c>
@@ -4998,9 +5078,7 @@
       <x:c r="J57" s="6" t="str">
         <x:v>Spatiotemporal action-recognition features</x:v>
       </x:c>
-      <x:c r="K57" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K57" s="6"/>
       <x:c r="L57" s="6" t="str">
         <x:v>Landmark</x:v>
       </x:c>
@@ -5069,9 +5147,7 @@
       <x:c r="J58" s="6" t="str">
         <x:v>Motion-conditioned generated video</x:v>
       </x:c>
-      <x:c r="K58" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K58" s="6"/>
       <x:c r="L58" s="6" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -5140,9 +5216,7 @@
       <x:c r="J59" s="6" t="str">
         <x:v>Generated scenes and video</x:v>
       </x:c>
-      <x:c r="K59" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K59" s="6"/>
       <x:c r="L59" s="6" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -5211,9 +5285,7 @@
       <x:c r="J60" s="6" t="str">
         <x:v>Video/audio tokens</x:v>
       </x:c>
-      <x:c r="K60" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K60" s="6"/>
       <x:c r="L60" s="6" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -5282,9 +5354,7 @@
       <x:c r="J61" s="6" t="str">
         <x:v>Latent representation</x:v>
       </x:c>
-      <x:c r="K61" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K61" s="6"/>
       <x:c r="L61" s="6" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -5353,9 +5423,7 @@
       <x:c r="J62" s="6" t="str">
         <x:v>Latent representation</x:v>
       </x:c>
-      <x:c r="K62" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K62" s="6"/>
       <x:c r="L62" s="6" t="str">
         <x:v>Landmark</x:v>
       </x:c>
@@ -5412,9 +5480,7 @@
       <x:c r="F63" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G63" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G63" s="6"/>
       <x:c r="H63" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -5495,9 +5561,7 @@
       <x:c r="J64" s="6" t="str">
         <x:v>Pixels / latent video tokens</x:v>
       </x:c>
-      <x:c r="K64" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K64" s="6"/>
       <x:c r="L64" s="6" t="str">
         <x:v>Landmark</x:v>
       </x:c>
@@ -5554,9 +5618,7 @@
       <x:c r="F65" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G65" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G65" s="6"/>
       <x:c r="H65" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -5625,9 +5687,7 @@
       <x:c r="F66" s="6" t="str">
         <x:v>Robotics</x:v>
       </x:c>
-      <x:c r="G66" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="G66" s="6"/>
       <x:c r="H66" s="6" t="str">
         <x:v>Action trajectory/tokens</x:v>
       </x:c>
@@ -5656,7 +5716,7 @@
         <x:v>https://www.physicalintelligence.company/blog/pi0</x:v>
       </x:c>
       <x:c r="Q66" s="6" t="str">
-        <x:v>Robotics-first control case for denominator/comparison</x:v>
+        <x:v>Robotics-side reference paper; excluded from the researcher transition denominator</x:v>
       </x:c>
       <x:c r="R66" s="15" t="n">
         <x:v>1</x:v>
@@ -5707,9 +5767,7 @@
       <x:c r="J67" s="6" t="str">
         <x:v>Taxonomy</x:v>
       </x:c>
-      <x:c r="K67" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
+      <x:c r="K67" s="6"/>
       <x:c r="L67" s="6" t="str">
         <x:v>Reference</x:v>
       </x:c>
@@ -5753,7 +5811,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58b6931ac03a4e17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R427aca364b2e48bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5892,7 +5950,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="n">
-        <x:f>IF(Z2="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z2))</x:f>
+        <x:f>IF(Z2="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z2))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
@@ -5990,7 +6048,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="6" t="n">
-        <x:f>IF(Z3="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z3))</x:f>
+        <x:f>IF(Z3="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z3))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
@@ -6088,7 +6146,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="6" t="n">
-        <x:f>IF(Z4="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z4))</x:f>
+        <x:f>IF(Z4="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z4))</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
@@ -6186,7 +6244,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="6" t="n">
-        <x:f>IF(Z5="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z5))</x:f>
+        <x:f>IF(Z5="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z5))</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
@@ -6284,7 +6342,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="6" t="n">
-        <x:f>IF(Z6="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z6))</x:f>
+        <x:f>IF(Z6="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z6))</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
@@ -6382,7 +6440,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="6" t="n">
-        <x:f>IF(Z7="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z7))</x:f>
+        <x:f>IF(Z7="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z7))</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
@@ -6480,7 +6538,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="6" t="n">
-        <x:f>IF(Z8="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z8))</x:f>
+        <x:f>IF(Z8="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z8))</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
@@ -6578,7 +6636,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6" t="n">
-        <x:f>IF(Z9="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z9))</x:f>
+        <x:f>IF(Z9="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z9))</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="6" t="str">
@@ -6676,7 +6734,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="6" t="n">
-        <x:f>IF(Z10="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z10))</x:f>
+        <x:f>IF(Z10="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z10))</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
@@ -6774,7 +6832,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="6" t="n">
-        <x:f>IF(Z11="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z11))</x:f>
+        <x:f>IF(Z11="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z11))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
@@ -6872,7 +6930,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="6" t="n">
-        <x:f>IF(Z12="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z12))</x:f>
+        <x:f>IF(Z12="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z12))</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
@@ -6970,7 +7028,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="6" t="n">
-        <x:f>IF(Z13="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z13))</x:f>
+        <x:f>IF(Z13="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z13))</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="6" t="str">
@@ -7068,7 +7126,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="6" t="n">
-        <x:f>IF(Z14="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z14))</x:f>
+        <x:f>IF(Z14="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z14))</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="6" t="str">
@@ -7166,7 +7224,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="6" t="n">
-        <x:f>IF(Z15="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z15))</x:f>
+        <x:f>IF(Z15="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z15))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
@@ -7264,7 +7322,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="n">
-        <x:f>IF(Z16="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z16))</x:f>
+        <x:f>IF(Z16="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z16))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B16" s="6" t="str">
@@ -7362,7 +7420,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="n">
-        <x:f>IF(Z17="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z17))</x:f>
+        <x:f>IF(Z17="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z17))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B17" s="6" t="str">
@@ -7460,7 +7518,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="n">
-        <x:f>IF(Z18="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z18))</x:f>
+        <x:f>IF(Z18="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z18))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B18" s="6" t="str">
@@ -7558,7 +7616,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="6" t="n">
-        <x:f>IF(Z19="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z19))</x:f>
+        <x:f>IF(Z19="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z19))</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="B19" s="6" t="str">
@@ -7656,7 +7714,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="6" t="n">
-        <x:f>IF(Z20="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z20))</x:f>
+        <x:f>IF(Z20="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z20))</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="6" t="str">
@@ -7754,7 +7812,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="6" t="n">
-        <x:f>IF(Z21="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z21))</x:f>
+        <x:f>IF(Z21="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z21))</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="B21" s="6" t="str">
@@ -7852,7 +7910,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="6" t="str">
-        <x:f>IF(Z22="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z22))</x:f>
+        <x:f>IF(Z22="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z22))</x:f>
       </x:c>
       <x:c r="B22" s="6" t="str">
         <x:v>R048</x:v>
@@ -7942,7 +8000,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="6" t="str">
-        <x:f>IF(Z23="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z23))</x:f>
+        <x:f>IF(Z23="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z23))</x:f>
       </x:c>
       <x:c r="B23" s="6" t="str">
         <x:v>R006</x:v>
@@ -8038,7 +8096,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="6" t="str">
-        <x:f>IF(Z24="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z24))</x:f>
+        <x:f>IF(Z24="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z24))</x:f>
       </x:c>
       <x:c r="B24" s="6" t="str">
         <x:v>R047</x:v>
@@ -8128,7 +8186,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="6" t="str">
-        <x:f>IF(Z25="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z25))</x:f>
+        <x:f>IF(Z25="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z25))</x:f>
       </x:c>
       <x:c r="B25" s="6" t="str">
         <x:v>R012</x:v>
@@ -8224,7 +8282,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="6" t="str">
-        <x:f>IF(Z26="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z26))</x:f>
+        <x:f>IF(Z26="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z26))</x:f>
       </x:c>
       <x:c r="B26" s="6" t="str">
         <x:v>R028</x:v>
@@ -8320,7 +8378,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="6" t="str">
-        <x:f>IF(Z27="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z27))</x:f>
+        <x:f>IF(Z27="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z27))</x:f>
       </x:c>
       <x:c r="B27" s="6" t="str">
         <x:v>R032</x:v>
@@ -8416,7 +8474,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="6" t="str">
-        <x:f>IF(Z28="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z28))</x:f>
+        <x:f>IF(Z28="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z28))</x:f>
       </x:c>
       <x:c r="B28" s="6" t="str">
         <x:v>R044</x:v>
@@ -8512,7 +8570,7 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="6" t="str">
-        <x:f>IF(Z29="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z29))</x:f>
+        <x:f>IF(Z29="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z29))</x:f>
       </x:c>
       <x:c r="B29" s="6" t="str">
         <x:v>R015</x:v>
@@ -8608,7 +8666,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="6" t="str">
-        <x:f>IF(Z30="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z30))</x:f>
+        <x:f>IF(Z30="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z30))</x:f>
       </x:c>
       <x:c r="B30" s="6" t="str">
         <x:v>R035</x:v>
@@ -8704,7 +8762,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="6" t="str">
-        <x:f>IF(Z31="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z31))</x:f>
+        <x:f>IF(Z31="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z31))</x:f>
       </x:c>
       <x:c r="B31" s="6" t="str">
         <x:v>R043</x:v>
@@ -8800,7 +8858,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="6" t="str">
-        <x:f>IF(Z32="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z32))</x:f>
+        <x:f>IF(Z32="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z32))</x:f>
       </x:c>
       <x:c r="B32" s="6" t="str">
         <x:v>R004</x:v>
@@ -8896,7 +8954,7 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="6" t="str">
-        <x:f>IF(Z33="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z33))</x:f>
+        <x:f>IF(Z33="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z33))</x:f>
       </x:c>
       <x:c r="B33" s="6" t="str">
         <x:v>R053</x:v>
@@ -8992,7 +9050,7 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="6" t="str">
-        <x:f>IF(Z34="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z34))</x:f>
+        <x:f>IF(Z34="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z34))</x:f>
       </x:c>
       <x:c r="B34" s="6" t="str">
         <x:v>R007</x:v>
@@ -9088,7 +9146,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="6" t="str">
-        <x:f>IF(Z35="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z35))</x:f>
+        <x:f>IF(Z35="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z35))</x:f>
       </x:c>
       <x:c r="B35" s="6" t="str">
         <x:v>R003</x:v>
@@ -9178,7 +9236,7 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="6" t="str">
-        <x:f>IF(Z36="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z36))</x:f>
+        <x:f>IF(Z36="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z36))</x:f>
       </x:c>
       <x:c r="B36" s="6" t="str">
         <x:v>R041</x:v>
@@ -9274,77 +9332,77 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="6" t="str">
-        <x:f>IF(Z37="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z37))</x:f>
+        <x:f>IF(Z37="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z37))</x:f>
       </x:c>
       <x:c r="B37" s="6" t="str">
-        <x:v>R038</x:v>
+        <x:v>R002</x:v>
       </x:c>
       <x:c r="C37" s="6" t="str">
-        <x:v>Kevin Black</x:v>
+        <x:v>Lijun Yu</x:v>
       </x:c>
       <x:c r="D37" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
-        <x:v>Physical Intelligence</x:v>
+        <x:v>Google Research / DeepMind</x:v>
       </x:c>
       <x:c r="F37" s="6" t="str">
-        <x:v>U2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G37" s="6" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>World simulation</x:v>
       </x:c>
       <x:c r="H37" s="6" t="str">
-        <x:v>Robotics-first</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I37" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J37" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K37" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K37" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="L37" s="6" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M37" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="N37" s="6" t="str">
         <x:f>IF(AND(L37="Yes",M37="Yes"),"Yes","No")</x:f>
         <x:v>No</x:v>
       </x:c>
       <x:c r="O37" s="6" t="str">
-        <x:v>Visual representation use</x:v>
+        <x:v>WALT; MAGVIT-v2</x:v>
       </x:c>
       <x:c r="P37" s="6" t="str">
-        <x:v>π0</x:v>
+        <x:v>Genie / interactive world modeling</x:v>
       </x:c>
       <x:c r="Q37" s="6" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="R37" s="6" t="str">
-        <x:v>Control case: important robotics author without video-origin evidence</x:v>
+        <x:v>Pixel/token video generation to interactive worlds</x:v>
       </x:c>
       <x:c r="S37" s="6" t="str">
-        <x:v>https://www.physicalintelligence.company/blog/pi0</x:v>
+        <x:v>https://me.lj-y.com/</x:v>
       </x:c>
       <x:c r="T37" s="6" t="str">
-        <x:v>https://www.physicalintelligence.company/blog/pi0</x:v>
+        <x:v>https://arxiv.org/abs/2312.06662</x:v>
       </x:c>
       <x:c r="U37" s="6" t="str">
-        <x:v>https://www.physicalintelligence.company/blog/pi0</x:v>
-      </x:c>
-      <x:c r="V37" s="6"/>
-      <x:c r="W37" s="6"/>
-      <x:c r="X37" s="6" t="str">
-        <x:v>P030</x:v>
-      </x:c>
-      <x:c r="Y37" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>https://deepmind.google/discover/blog/genie-2-a-large-scale-foundation-world-model/</x:v>
+      </x:c>
+      <x:c r="V37" s="6" t="str">
+        <x:v>P001</x:v>
+      </x:c>
+      <x:c r="W37" s="6" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="X37" s="6"/>
+      <x:c r="Y37" s="6"/>
       <x:c r="Z37" s="15" t="str">
         <x:f>IF(AND(N37="Yes",AA37="Both distinct selected papers covered"),SQRT((W37+1)*(Y37+1))*IF(Q37="High",1,0.8),"")</x:f>
       </x:c>
@@ -9354,32 +9412,32 @@
       <x:c r="AB37" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC37" s="6"/>
-      <x:c r="AD37" s="6" t="str">
-        <x:v>Action trajectory/tokens</x:v>
-      </x:c>
+      <x:c r="AC37" s="6" t="str">
+        <x:v>G1</x:v>
+      </x:c>
+      <x:c r="AD37" s="6"/>
       <x:c r="AE37" s="6" t="str">
         <x:v>Partial evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="6" t="str">
-        <x:f>IF(Z38="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z38))</x:f>
+        <x:f>IF(Z38="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z38))</x:f>
       </x:c>
       <x:c r="B38" s="6" t="str">
-        <x:v>R002</x:v>
+        <x:v>R027</x:v>
       </x:c>
       <x:c r="C38" s="6" t="str">
-        <x:v>Lijun Yu</x:v>
+        <x:v>Mohammad Babaeizadeh</x:v>
       </x:c>
       <x:c r="D38" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
-        <x:v>Google Research / DeepMind</x:v>
+        <x:v>Google / NVIDIA</x:v>
       </x:c>
       <x:c r="F38" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G38" s="6" t="str">
         <x:v>World simulation</x:v>
@@ -9407,127 +9465,133 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="O38" s="6" t="str">
-        <x:v>WALT; MAGVIT-v2</x:v>
+        <x:v>SV2P; FitVid</x:v>
       </x:c>
       <x:c r="P38" s="6" t="str">
-        <x:v>Genie / interactive world modeling</x:v>
+        <x:v>Robot/world simulation</x:v>
       </x:c>
       <x:c r="Q38" s="6" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="R38" s="6" t="str">
-        <x:v>Pixel/token video generation to interactive worlds</x:v>
+        <x:v>Important stochastic video prediction lineage</x:v>
       </x:c>
       <x:c r="S38" s="6" t="str">
-        <x:v>https://me.lj-y.com/</x:v>
+        <x:v>https://scholar.google.com/scholar?q=Mohammad+Babaeizadeh+video+prediction</x:v>
       </x:c>
       <x:c r="T38" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2312.06662</x:v>
+        <x:v>https://arxiv.org/abs/1710.11252</x:v>
       </x:c>
       <x:c r="U38" s="6" t="str">
-        <x:v>https://deepmind.google/discover/blog/genie-2-a-large-scale-foundation-world-model/</x:v>
+        <x:v>https://arxiv.org/abs/2106.13195</x:v>
       </x:c>
       <x:c r="V38" s="6" t="str">
-        <x:v>P001</x:v>
+        <x:v>P008</x:v>
       </x:c>
       <x:c r="W38" s="6" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="X38" s="6"/>
-      <x:c r="Y38" s="6"/>
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="X38" s="6" t="str">
+        <x:v>P010</x:v>
+      </x:c>
+      <x:c r="Y38" s="6" t="n">
+        <x:v>29</x:v>
+      </x:c>
       <x:c r="Z38" s="15" t="str">
         <x:f>IF(AND(N38="Yes",AA38="Both distinct selected papers covered"),SQRT((W38+1)*(Y38+1))*IF(Q38="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA38" s="6" t="str">
-        <x:v>Partial / missing selected-paper coverage</x:v>
+        <x:v>Both distinct selected papers covered</x:v>
       </x:c>
       <x:c r="AB38" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC38" s="6" t="str">
-        <x:v>G1</x:v>
-      </x:c>
-      <x:c r="AD38" s="6"/>
+        <x:v>G2</x:v>
+      </x:c>
+      <x:c r="AD38" s="6" t="str">
+        <x:v>Predicted future video/state</x:v>
+      </x:c>
       <x:c r="AE38" s="6" t="str">
-        <x:v>Partial evidence</x:v>
+        <x:v>Verified distinct paper pair</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="6" t="str">
-        <x:f>IF(Z39="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z39))</x:f>
+        <x:f>IF(Z39="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z39))</x:f>
       </x:c>
       <x:c r="B39" s="6" t="str">
-        <x:v>R027</x:v>
+        <x:v>R021</x:v>
       </x:c>
       <x:c r="C39" s="6" t="str">
-        <x:v>Mohammad Babaeizadeh</x:v>
+        <x:v>Moo Jin Kim</x:v>
       </x:c>
       <x:c r="D39" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:v>Google / NVIDIA</x:v>
+        <x:v>NVIDIA / Stanford</x:v>
       </x:c>
       <x:c r="F39" s="6" t="str">
         <x:v>G2</x:v>
       </x:c>
       <x:c r="G39" s="6" t="str">
-        <x:v>World simulation</x:v>
+        <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="H39" s="6" t="str">
         <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I39" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J39" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K39" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L39" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M39" s="6" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N39" s="6" t="str">
         <x:f>IF(AND(L39="Yes",M39="Yes"),"Yes","No")</x:f>
         <x:v>No</x:v>
       </x:c>
       <x:c r="O39" s="6" t="str">
-        <x:v>SV2P; FitVid</x:v>
+        <x:v>Cosmos-Predict lineage</x:v>
       </x:c>
       <x:c r="P39" s="6" t="str">
-        <x:v>Robot/world simulation</x:v>
+        <x:v>Cosmos Policy</x:v>
       </x:c>
       <x:c r="Q39" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R39" s="6" t="str">
-        <x:v>Important stochastic video prediction lineage</x:v>
+        <x:v>Lead robotics transfer of generative video foundation model</x:v>
       </x:c>
       <x:c r="S39" s="6" t="str">
-        <x:v>https://scholar.google.com/scholar?q=Mohammad+Babaeizadeh+video+prediction</x:v>
+        <x:v>https://research.nvidia.com/labs/cosmos-lab/cosmos-policy/</x:v>
       </x:c>
       <x:c r="T39" s="6" t="str">
-        <x:v>https://arxiv.org/abs/1710.11252</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="U39" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2106.13195</x:v>
+        <x:v>https://arxiv.org/abs/2601.16163</x:v>
       </x:c>
       <x:c r="V39" s="6" t="str">
-        <x:v>P008</x:v>
+        <x:v>P016</x:v>
       </x:c>
       <x:c r="W39" s="6" t="n">
-        <x:v>73</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X39" s="6" t="str">
-        <x:v>P010</x:v>
+        <x:v>P017</x:v>
       </x:c>
       <x:c r="Y39" s="6" t="n">
-        <x:v>29</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Z39" s="15" t="str">
         <x:f>IF(AND(N39="Yes",AA39="Both distinct selected papers covered"),SQRT((W39+1)*(Y39+1))*IF(Q39="High",1,0.8),"")</x:f>
@@ -9542,7 +9606,7 @@
         <x:v>G2</x:v>
       </x:c>
       <x:c r="AD39" s="6" t="str">
-        <x:v>Predicted future video/state</x:v>
+        <x:v>Joint visual/state + action</x:v>
       </x:c>
       <x:c r="AE39" s="6" t="str">
         <x:v>Verified distinct paper pair</x:v>
@@ -9550,34 +9614,34 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="6" t="str">
-        <x:f>IF(Z40="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z40))</x:f>
+        <x:f>IF(Z40="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z40))</x:f>
       </x:c>
       <x:c r="B40" s="6" t="str">
-        <x:v>R021</x:v>
+        <x:v>R039</x:v>
       </x:c>
       <x:c r="C40" s="6" t="str">
-        <x:v>Moo Jin Kim</x:v>
+        <x:v>Ruohan Zhang</x:v>
       </x:c>
       <x:c r="D40" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
-        <x:v>NVIDIA / Stanford</x:v>
+        <x:v>Stanford</x:v>
       </x:c>
       <x:c r="F40" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G40" s="6" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>Planning</x:v>
       </x:c>
       <x:c r="H40" s="6" t="str">
-        <x:v>Bridger</x:v>
+        <x:v>Native hybrid</x:v>
       </x:c>
       <x:c r="I40" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="J40" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K40" s="6" t="n">
         <x:v>3</x:v>
@@ -9593,34 +9657,34 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="O40" s="6" t="str">
-        <x:v>Cosmos-Predict lineage</x:v>
+        <x:v>Generative/embodied visual work</x:v>
       </x:c>
       <x:c r="P40" s="6" t="str">
-        <x:v>Cosmos Policy</x:v>
+        <x:v>Dream2Flow</x:v>
       </x:c>
       <x:c r="Q40" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R40" s="6" t="str">
-        <x:v>Lead robotics transfer of generative video foundation model</x:v>
+        <x:v>Embodied generation and manipulation bridge</x:v>
       </x:c>
       <x:c r="S40" s="6" t="str">
-        <x:v>https://research.nvidia.com/labs/cosmos-lab/cosmos-policy/</x:v>
+        <x:v>https://ruohanzhang.com/</x:v>
       </x:c>
       <x:c r="T40" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
+        <x:v>https://jiajunwu.com/</x:v>
       </x:c>
       <x:c r="U40" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2601.16163</x:v>
+        <x:v>https://jiajunwu.com/</x:v>
       </x:c>
       <x:c r="V40" s="6" t="str">
-        <x:v>P016</x:v>
+        <x:v>P026</x:v>
       </x:c>
       <x:c r="W40" s="6" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="X40" s="6" t="str">
-        <x:v>P017</x:v>
+        <x:v>P026</x:v>
       </x:c>
       <x:c r="Y40" s="6" t="n">
         <x:v>0</x:v>
@@ -9629,45 +9693,45 @@
         <x:f>IF(AND(N40="Yes",AA40="Both distinct selected papers covered"),SQRT((W40+1)*(Y40+1))*IF(Q40="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA40" s="6" t="str">
-        <x:v>Both distinct selected papers covered</x:v>
+        <x:v>Single bridge paper used on both sides</x:v>
       </x:c>
       <x:c r="AB40" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC40" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="AD40" s="6" t="str">
-        <x:v>Joint visual/state + action</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE40" s="6" t="str">
-        <x:v>Verified distinct paper pair</x:v>
+        <x:v>Verified single-paper bridge; not ranked</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="6" t="str">
-        <x:f>IF(Z41="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z41))</x:f>
+        <x:f>IF(Z41="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z41))</x:f>
       </x:c>
       <x:c r="B41" s="6" t="str">
-        <x:v>R046</x:v>
+        <x:v>R036</x:v>
       </x:c>
       <x:c r="C41" s="6" t="str">
-        <x:v>Oier Mees</x:v>
+        <x:v>Russell Mendonca</x:v>
       </x:c>
       <x:c r="D41" s="6" t="str">
-        <x:v>Europe</x:v>
+        <x:v>US</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
-        <x:v>University of Freiburg</x:v>
+        <x:v>Carnegie Mellon</x:v>
       </x:c>
       <x:c r="F41" s="6" t="str">
-        <x:v>None</x:v>
+        <x:v>U2</x:v>
       </x:c>
       <x:c r="G41" s="6" t="str">
         <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="H41" s="6" t="str">
-        <x:v>Robotics-first</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I41" s="6" t="n">
         <x:v>1</x:v>
@@ -9679,130 +9743,140 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="L41" s="6" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M41" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N41" s="6" t="str">
         <x:f>IF(AND(L41="Yes",M41="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="O41" s="6" t="str">
-        <x:v>Language-conditioned video/representation learning</x:v>
+        <x:v>Learning from videos</x:v>
       </x:c>
       <x:c r="P41" s="6" t="str">
-        <x:v>CALVIN; generalist robot policies</x:v>
+        <x:v>WHIRL; robot learning</x:v>
       </x:c>
       <x:c r="Q41" s="6" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="R41" s="6" t="str">
-        <x:v>Robotics benchmark and policy researcher retained as a comparison case; no verified video-origin paper selected</x:v>
+        <x:v>Human-video imitation to real robots</x:v>
       </x:c>
       <x:c r="S41" s="6" t="str">
-        <x:v>https://www.oiermees.com/</x:v>
-      </x:c>
-      <x:c r="T41" s="6"/>
+        <x:v>https://russellmendonca.github.io/</x:v>
+      </x:c>
+      <x:c r="T41" s="6" t="str">
+        <x:v>https://arxiv.org/abs/2207.09450</x:v>
+      </x:c>
       <x:c r="U41" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2112.03227</x:v>
-      </x:c>
-      <x:c r="V41" s="6"/>
-      <x:c r="W41" s="6"/>
+        <x:v>https://arxiv.org/abs/2207.09450</x:v>
+      </x:c>
+      <x:c r="V41" s="6" t="str">
+        <x:v>P036</x:v>
+      </x:c>
+      <x:c r="W41" s="6" t="n">
+        <x:v>83</x:v>
+      </x:c>
       <x:c r="X41" s="6" t="str">
-        <x:v>P034</x:v>
+        <x:v>P036</x:v>
       </x:c>
       <x:c r="Y41" s="6" t="n">
-        <x:v>6</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="Z41" s="15" t="str">
         <x:f>IF(AND(N41="Yes",AA41="Both distinct selected papers covered"),SQRT((W41+1)*(Y41+1))*IF(Q41="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA41" s="6" t="str">
-        <x:v>Partial / missing selected-paper coverage</x:v>
+        <x:v>Single bridge paper used on both sides</x:v>
       </x:c>
       <x:c r="AB41" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC41" s="6"/>
+      <x:c r="AC41" s="6" t="str">
+        <x:v>U2</x:v>
+      </x:c>
       <x:c r="AD41" s="6" t="str">
-        <x:v>Dataset/benchmark</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE41" s="6" t="str">
-        <x:v>Partial evidence</x:v>
+        <x:v>Verified single-paper bridge; not ranked</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="6" t="str">
-        <x:f>IF(Z42="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z42))</x:f>
+        <x:f>IF(Z42="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z42))</x:f>
       </x:c>
       <x:c r="B42" s="6" t="str">
-        <x:v>R045</x:v>
+        <x:v>R051</x:v>
       </x:c>
       <x:c r="C42" s="6" t="str">
-        <x:v>Pierre-Louis Guhur</x:v>
+        <x:v>Samarth Sinha</x:v>
       </x:c>
       <x:c r="D42" s="6" t="str">
-        <x:v>Europe</x:v>
+        <x:v>US</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
-        <x:v>Inria / ENS Paris</x:v>
+        <x:v>Luma AI → 1X World Model Lab</x:v>
       </x:c>
       <x:c r="F42" s="6" t="str">
-        <x:v>None</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G42" s="6" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>World simulation</x:v>
       </x:c>
       <x:c r="H42" s="6" t="str">
-        <x:v>Robotics-first</x:v>
+        <x:v>Switcher</x:v>
       </x:c>
       <x:c r="I42" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J42" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K42" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L42" s="6" t="str">
-        <x:v>No</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M42" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="N42" s="6" t="str">
         <x:f>IF(AND(L42="Yes",M42="Yes"),"Yes","No")</x:f>
         <x:v>No</x:v>
       </x:c>
       <x:c r="O42" s="6" t="str">
-        <x:v>No verified video-origin paper</x:v>
+        <x:v>Video generation</x:v>
       </x:c>
       <x:c r="P42" s="6" t="str">
-        <x:v>Hiveformer</x:v>
+        <x:v>1X World Model</x:v>
       </x:c>
       <x:c r="Q42" s="6" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="R42" s="6" t="str">
-        <x:v>Video-language understanding to manipulation</x:v>
+        <x:v>Clear organizational move from video generation to robot world models</x:v>
       </x:c>
       <x:c r="S42" s="6" t="str">
-        <x:v>https://scholar.google.com/scholar?q=Pierre-Louis+Guhur</x:v>
-      </x:c>
-      <x:c r="T42" s="6"/>
+        <x:v>https://www.samsinha.me/</x:v>
+      </x:c>
+      <x:c r="T42" s="6" t="str">
+        <x:v>https://www.samsinha.me/</x:v>
+      </x:c>
       <x:c r="U42" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2209.04899</x:v>
-      </x:c>
-      <x:c r="V42" s="6"/>
+        <x:v>https://www.1x.tech/discover/1x-world-model-lab</x:v>
+      </x:c>
+      <x:c r="V42" s="6" t="str">
+        <x:v>P032</x:v>
+      </x:c>
       <x:c r="W42" s="6"/>
       <x:c r="X42" s="6" t="str">
-        <x:v>P058</x:v>
-      </x:c>
-      <x:c r="Y42" s="6" t="n">
-        <x:v>7</x:v>
-      </x:c>
+        <x:v>P032</x:v>
+      </x:c>
+      <x:c r="Y42" s="6"/>
       <x:c r="Z42" s="15" t="str">
         <x:f>IF(AND(N42="Yes",AA42="Both distinct selected papers covered"),SQRT((W42+1)*(Y42+1))*IF(Q42="High",1,0.8),"")</x:f>
       </x:c>
@@ -9812,90 +9886,92 @@
       <x:c r="AB42" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC42" s="6"/>
+      <x:c r="AC42" s="6" t="str">
+        <x:v>G2</x:v>
+      </x:c>
       <x:c r="AD42" s="6" t="str">
-        <x:v>Action trajectory/tokens</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE42" s="6" t="str">
-        <x:v>Partial evidence</x:v>
+        <x:v>Verified distinct paper pair</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="6" t="str">
-        <x:f>IF(Z43="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z43))</x:f>
+        <x:f>IF(Z43="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z43))</x:f>
       </x:c>
       <x:c r="B43" s="6" t="str">
-        <x:v>R039</x:v>
+        <x:v>R016</x:v>
       </x:c>
       <x:c r="C43" s="6" t="str">
-        <x:v>Ruohan Zhang</x:v>
+        <x:v>Sergio Arnaud</x:v>
       </x:c>
       <x:c r="D43" s="6" t="str">
-        <x:v>US</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>Meta FAIR Paris</x:v>
       </x:c>
       <x:c r="F43" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>U3</x:v>
       </x:c>
       <x:c r="G43" s="6" t="str">
         <x:v>Planning</x:v>
       </x:c>
       <x:c r="H43" s="6" t="str">
-        <x:v>Native hybrid</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I43" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J43" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K43" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L43" s="6" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M43" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N43" s="6" t="str">
         <x:f>IF(AND(L43="Yes",M43="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="O43" s="6" t="str">
-        <x:v>Generative/embodied visual work</x:v>
+        <x:v>V-JEPA 2</x:v>
       </x:c>
       <x:c r="P43" s="6" t="str">
-        <x:v>Dream2Flow</x:v>
+        <x:v>V-JEPA 2-AC</x:v>
       </x:c>
       <x:c r="Q43" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R43" s="6" t="str">
-        <x:v>Embodied generation and manipulation bridge</x:v>
+        <x:v>Core team on robotics post-training</x:v>
       </x:c>
       <x:c r="S43" s="6" t="str">
-        <x:v>https://ruohanzhang.com/</x:v>
+        <x:v>https://arxiv.org/abs/2506.09985</x:v>
       </x:c>
       <x:c r="T43" s="6" t="str">
-        <x:v>https://jiajunwu.com/</x:v>
+        <x:v>https://arxiv.org/abs/2506.09985</x:v>
       </x:c>
       <x:c r="U43" s="6" t="str">
-        <x:v>https://jiajunwu.com/</x:v>
+        <x:v>https://arxiv.org/abs/2506.09985</x:v>
       </x:c>
       <x:c r="V43" s="6" t="str">
-        <x:v>P026</x:v>
+        <x:v>P004</x:v>
       </x:c>
       <x:c r="W43" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X43" s="6" t="str">
-        <x:v>P026</x:v>
+        <x:v>P004</x:v>
       </x:c>
       <x:c r="Y43" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z43" s="15" t="str">
         <x:f>IF(AND(N43="Yes",AA43="Both distinct selected papers covered"),SQRT((W43+1)*(Y43+1))*IF(Q43="High",1,0.8),"")</x:f>
@@ -9907,10 +9983,10 @@
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC43" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>U3</x:v>
       </x:c>
       <x:c r="AD43" s="6" t="str">
-        <x:v>Generated image/video</x:v>
+        <x:v>Representation/reward/value</x:v>
       </x:c>
       <x:c r="AE43" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -9918,34 +9994,34 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="6" t="str">
-        <x:f>IF(Z44="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z44))</x:f>
+        <x:f>IF(Z44="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z44))</x:f>
       </x:c>
       <x:c r="B44" s="6" t="str">
-        <x:v>R036</x:v>
+        <x:v>R005</x:v>
       </x:c>
       <x:c r="C44" s="6" t="str">
-        <x:v>Russell Mendonca</x:v>
+        <x:v>Sherry Yang</x:v>
       </x:c>
       <x:c r="D44" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
-        <x:v>Carnegie Mellon</x:v>
+        <x:v>Google DeepMind</x:v>
       </x:c>
       <x:c r="F44" s="6" t="str">
-        <x:v>U2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G44" s="6" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>Planning</x:v>
       </x:c>
       <x:c r="H44" s="6" t="str">
         <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I44" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J44" s="6" t="n">
         <x:v>1</x:v>
-      </x:c>
-      <x:c r="J44" s="6" t="n">
-        <x:v>3</x:v>
       </x:c>
       <x:c r="K44" s="6" t="n">
         <x:v>3</x:v>
@@ -9961,37 +10037,37 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="O44" s="6" t="str">
-        <x:v>Learning from videos</x:v>
+        <x:v>Video generation research</x:v>
       </x:c>
       <x:c r="P44" s="6" t="str">
-        <x:v>WHIRL; robot learning</x:v>
+        <x:v>UniPi</x:v>
       </x:c>
       <x:c r="Q44" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R44" s="6" t="str">
-        <x:v>Human-video imitation to real robots</x:v>
+        <x:v>Text-guided video generation used as policy/planner</x:v>
       </x:c>
       <x:c r="S44" s="6" t="str">
-        <x:v>https://russellmendonca.github.io/</x:v>
+        <x:v>https://sherryy.github.io/</x:v>
       </x:c>
       <x:c r="T44" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2207.09450</x:v>
+        <x:v>https://arxiv.org/abs/2302.00111</x:v>
       </x:c>
       <x:c r="U44" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2207.09450</x:v>
+        <x:v>https://research.google/blog/unipi-learning-universal-policies-via-text-guided-video-generation/</x:v>
       </x:c>
       <x:c r="V44" s="6" t="str">
-        <x:v>P036</x:v>
+        <x:v>P011</x:v>
       </x:c>
       <x:c r="W44" s="6" t="n">
-        <x:v>83</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="X44" s="6" t="str">
-        <x:v>P036</x:v>
+        <x:v>P011</x:v>
       </x:c>
       <x:c r="Y44" s="6" t="n">
-        <x:v>83</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="Z44" s="15" t="str">
         <x:f>IF(AND(N44="Yes",AA44="Both distinct selected papers covered"),SQRT((W44+1)*(Y44+1))*IF(Q44="High",1,0.8),"")</x:f>
@@ -10003,10 +10079,10 @@
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC44" s="6" t="str">
-        <x:v>U2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="AD44" s="6" t="str">
-        <x:v>Action trajectory/tokens</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE44" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10014,172 +10090,176 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="6" t="str">
-        <x:f>IF(Z45="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z45))</x:f>
+        <x:f>IF(Z45="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z45))</x:f>
       </x:c>
       <x:c r="B45" s="6" t="str">
-        <x:v>R051</x:v>
+        <x:v>R031</x:v>
       </x:c>
       <x:c r="C45" s="6" t="str">
-        <x:v>Samarth Sinha</x:v>
+        <x:v>Shikhar Bahl</x:v>
       </x:c>
       <x:c r="D45" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
-        <x:v>Luma AI → 1X World Model Lab</x:v>
+        <x:v>Carnegie Mellon</x:v>
       </x:c>
       <x:c r="F45" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>U2</x:v>
       </x:c>
       <x:c r="G45" s="6" t="str">
-        <x:v>World simulation</x:v>
+        <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="H45" s="6" t="str">
-        <x:v>Switcher</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I45" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J45" s="6" t="n">
         <x:v>3</x:v>
-      </x:c>
-      <x:c r="J45" s="6" t="n">
-        <x:v>1</x:v>
       </x:c>
       <x:c r="K45" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L45" s="6" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M45" s="6" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N45" s="6" t="str">
         <x:f>IF(AND(L45="Yes",M45="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="O45" s="6" t="str">
-        <x:v>Video generation</x:v>
+        <x:v>Learning from video / interaction</x:v>
       </x:c>
       <x:c r="P45" s="6" t="str">
-        <x:v>1X World Model</x:v>
+        <x:v>WHIRL; robot learning</x:v>
       </x:c>
       <x:c r="Q45" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R45" s="6" t="str">
-        <x:v>Clear organizational move from video generation to robot world models</x:v>
+        <x:v>Human-video to robot policy bridge</x:v>
       </x:c>
       <x:c r="S45" s="6" t="str">
-        <x:v>https://www.samsinha.me/</x:v>
+        <x:v>https://shikharbahl.github.io/</x:v>
       </x:c>
       <x:c r="T45" s="6" t="str">
-        <x:v>https://www.samsinha.me/</x:v>
+        <x:v>https://arxiv.org/abs/2207.09450</x:v>
       </x:c>
       <x:c r="U45" s="6" t="str">
-        <x:v>https://www.1x.tech/discover/1x-world-model-lab</x:v>
+        <x:v>https://arxiv.org/abs/2207.09450</x:v>
       </x:c>
       <x:c r="V45" s="6" t="str">
-        <x:v>P032</x:v>
-      </x:c>
-      <x:c r="W45" s="6"/>
+        <x:v>P036</x:v>
+      </x:c>
+      <x:c r="W45" s="6" t="n">
+        <x:v>83</x:v>
+      </x:c>
       <x:c r="X45" s="6" t="str">
-        <x:v>P032</x:v>
-      </x:c>
-      <x:c r="Y45" s="6"/>
+        <x:v>P036</x:v>
+      </x:c>
+      <x:c r="Y45" s="6" t="n">
+        <x:v>83</x:v>
+      </x:c>
       <x:c r="Z45" s="15" t="str">
         <x:f>IF(AND(N45="Yes",AA45="Both distinct selected papers covered"),SQRT((W45+1)*(Y45+1))*IF(Q45="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA45" s="6" t="str">
-        <x:v>Partial / missing selected-paper coverage</x:v>
+        <x:v>Single bridge paper used on both sides</x:v>
       </x:c>
       <x:c r="AB45" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC45" s="6" t="str">
-        <x:v>G2</x:v>
+        <x:v>U2</x:v>
       </x:c>
       <x:c r="AD45" s="6" t="str">
-        <x:v>Predicted future video/state</x:v>
+        <x:v>Action trajectory/tokens</x:v>
       </x:c>
       <x:c r="AE45" s="6" t="str">
-        <x:v>Verified distinct paper pair</x:v>
+        <x:v>Verified single-paper bridge; not ranked</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="6" t="str">
-        <x:f>IF(Z46="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z46))</x:f>
+        <x:f>IF(Z46="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z46))</x:f>
       </x:c>
       <x:c r="B46" s="6" t="str">
-        <x:v>R016</x:v>
+        <x:v>R037</x:v>
       </x:c>
       <x:c r="C46" s="6" t="str">
-        <x:v>Sergio Arnaud</x:v>
+        <x:v>Suraj Nair</x:v>
       </x:c>
       <x:c r="D46" s="6" t="str">
-        <x:v>Europe</x:v>
+        <x:v>US</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
-        <x:v>Meta FAIR Paris</x:v>
+        <x:v>Stanford</x:v>
       </x:c>
       <x:c r="F46" s="6" t="str">
-        <x:v>U3</x:v>
+        <x:v>VL</x:v>
       </x:c>
       <x:c r="G46" s="6" t="str">
-        <x:v>Planning</x:v>
+        <x:v>Perception backbone</x:v>
       </x:c>
       <x:c r="H46" s="6" t="str">
         <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I46" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J46" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K46" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N46" s="6" t="str">
         <x:f>IF(AND(L46="Yes",M46="Yes"),"Yes","No")</x:f>
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="O46" s="6" t="str">
-        <x:v>V-JEPA 2</x:v>
+        <x:v>R3M</x:v>
       </x:c>
       <x:c r="P46" s="6" t="str">
-        <x:v>V-JEPA 2-AC</x:v>
+        <x:v>R3M</x:v>
       </x:c>
       <x:c r="Q46" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R46" s="6" t="str">
-        <x:v>Core team on robotics post-training</x:v>
+        <x:v>Human-video temporal and language alignment transferred as a frozen robot perception backbone</x:v>
       </x:c>
       <x:c r="S46" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2506.09985</x:v>
+        <x:v>https://suraj-nair-1.github.io/</x:v>
       </x:c>
       <x:c r="T46" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2506.09985</x:v>
+        <x:v>https://arxiv.org/abs/2203.12601</x:v>
       </x:c>
       <x:c r="U46" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2506.09985</x:v>
+        <x:v>https://arxiv.org/abs/2203.12601</x:v>
       </x:c>
       <x:c r="V46" s="6" t="str">
-        <x:v>P004</x:v>
+        <x:v>P066</x:v>
       </x:c>
       <x:c r="W46" s="6" t="n">
-        <x:v>5</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="X46" s="6" t="str">
-        <x:v>P004</x:v>
+        <x:v>P066</x:v>
       </x:c>
       <x:c r="Y46" s="6" t="n">
-        <x:v>5</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="Z46" s="15" t="str">
         <x:f>IF(AND(N46="Yes",AA46="Both distinct selected papers covered"),SQRT((W46+1)*(Y46+1))*IF(Q46="High",1,0.8),"")</x:f>
@@ -10191,7 +10271,7 @@
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC46" s="6" t="str">
-        <x:v>U3</x:v>
+        <x:v>VL</x:v>
       </x:c>
       <x:c r="AD46" s="6" t="str">
         <x:v>Representation/reward/value</x:v>
@@ -10202,28 +10282,28 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="6" t="str">
-        <x:f>IF(Z47="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z47))</x:f>
+        <x:f>IF(Z47="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z47))</x:f>
       </x:c>
       <x:c r="B47" s="6" t="str">
-        <x:v>R005</x:v>
+        <x:v>R052</x:v>
       </x:c>
       <x:c r="C47" s="6" t="str">
-        <x:v>Sherry Yang</x:v>
+        <x:v>Tim Brooks</x:v>
       </x:c>
       <x:c r="D47" s="6" t="str">
-        <x:v>US</x:v>
+        <x:v>Europe</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
-        <x:v>Google DeepMind</x:v>
+        <x:v>OpenAI → Google DeepMind London</x:v>
       </x:c>
       <x:c r="F47" s="6" t="str">
         <x:v>G1</x:v>
       </x:c>
       <x:c r="G47" s="6" t="str">
-        <x:v>Planning</x:v>
+        <x:v>World simulation</x:v>
       </x:c>
       <x:c r="H47" s="6" t="str">
-        <x:v>Bridger</x:v>
+        <x:v>Switcher</x:v>
       </x:c>
       <x:c r="I47" s="6" t="n">
         <x:v>3</x:v>
@@ -10232,146 +10312,134 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="K47" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L47" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="M47" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="N47" s="6" t="str">
         <x:f>IF(AND(L47="Yes",M47="Yes"),"Yes","No")</x:f>
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="O47" s="6" t="str">
-        <x:v>Video generation research</x:v>
+        <x:v>Sora / video generation</x:v>
       </x:c>
       <x:c r="P47" s="6" t="str">
-        <x:v>UniPi</x:v>
+        <x:v>Interactive world models</x:v>
       </x:c>
       <x:c r="Q47" s="6" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="R47" s="6" t="str">
-        <x:v>Text-guided video generation used as policy/planner</x:v>
+        <x:v>Clear video→world-model move; physical-robot evidence still limited</x:v>
       </x:c>
       <x:c r="S47" s="6" t="str">
-        <x:v>https://sherryy.github.io/</x:v>
+        <x:v>https://scholar.google.com/scholar?q=Tim+Brooks+video+generation</x:v>
       </x:c>
       <x:c r="T47" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2302.00111</x:v>
+        <x:v>https://openai.com/index/video-generation-models-as-world-simulators/</x:v>
       </x:c>
       <x:c r="U47" s="6" t="str">
-        <x:v>https://research.google/blog/unipi-learning-universal-policies-via-text-guided-video-generation/</x:v>
-      </x:c>
-      <x:c r="V47" s="6" t="str">
-        <x:v>P011</x:v>
-      </x:c>
-      <x:c r="W47" s="6" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="X47" s="6" t="str">
-        <x:v>P011</x:v>
-      </x:c>
-      <x:c r="Y47" s="6" t="n">
-        <x:v>29</x:v>
-      </x:c>
+        <x:v>https://deepmind.google/discover/blog/genie-2-a-large-scale-foundation-world-model/</x:v>
+      </x:c>
+      <x:c r="V47" s="6"/>
+      <x:c r="W47" s="6"/>
+      <x:c r="X47" s="6"/>
+      <x:c r="Y47" s="6"/>
       <x:c r="Z47" s="15" t="str">
         <x:f>IF(AND(N47="Yes",AA47="Both distinct selected papers covered"),SQRT((W47+1)*(Y47+1))*IF(Q47="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA47" s="6" t="str">
-        <x:v>Single bridge paper used on both sides</x:v>
+        <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB47" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC47" s="6" t="str">
-        <x:v>G1</x:v>
-      </x:c>
-      <x:c r="AD47" s="6" t="str">
-        <x:v>Generated image/video</x:v>
-      </x:c>
+      <x:c r="AC47" s="6"/>
+      <x:c r="AD47" s="6"/>
       <x:c r="AE47" s="6" t="str">
-        <x:v>Verified single-paper bridge; not ranked</x:v>
+        <x:v>Partial evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="6" t="str">
-        <x:f>IF(Z48="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z48))</x:f>
+        <x:f>IF(Z48="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z48))</x:f>
       </x:c>
       <x:c r="B48" s="6" t="str">
-        <x:v>R031</x:v>
+        <x:v>R040</x:v>
       </x:c>
       <x:c r="C48" s="6" t="str">
-        <x:v>Shikhar Bahl</x:v>
+        <x:v>Wenlong Huang</x:v>
       </x:c>
       <x:c r="D48" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E48" s="6" t="str">
-        <x:v>Carnegie Mellon</x:v>
+        <x:v>Stanford</x:v>
       </x:c>
       <x:c r="F48" s="6" t="str">
-        <x:v>U2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G48" s="6" t="str">
-        <x:v>Direct policy</x:v>
+        <x:v>Planning</x:v>
       </x:c>
       <x:c r="H48" s="6" t="str">
         <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I48" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J48" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K48" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L48" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M48" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N48" s="6" t="str">
         <x:f>IF(AND(L48="Yes",M48="Yes"),"Yes","No")</x:f>
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="O48" s="6" t="str">
-        <x:v>Learning from video / interaction</x:v>
+        <x:v>Generative planning</x:v>
       </x:c>
       <x:c r="P48" s="6" t="str">
-        <x:v>WHIRL; robot learning</x:v>
+        <x:v>Dream2Flow</x:v>
       </x:c>
       <x:c r="Q48" s="6" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="R48" s="6" t="str">
-        <x:v>Human-video to robot policy bridge</x:v>
+        <x:v>Recent bridge; exact citation tracked via project page</x:v>
       </x:c>
       <x:c r="S48" s="6" t="str">
-        <x:v>https://shikharbahl.github.io/</x:v>
+        <x:v>https://wenlong.page/</x:v>
       </x:c>
       <x:c r="T48" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2207.09450</x:v>
+        <x:v>https://jiajunwu.com/</x:v>
       </x:c>
       <x:c r="U48" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2207.09450</x:v>
+        <x:v>https://jiajunwu.com/</x:v>
       </x:c>
       <x:c r="V48" s="6" t="str">
-        <x:v>P036</x:v>
+        <x:v>P026</x:v>
       </x:c>
       <x:c r="W48" s="6" t="n">
-        <x:v>83</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="X48" s="6" t="str">
-        <x:v>P036</x:v>
+        <x:v>P026</x:v>
       </x:c>
       <x:c r="Y48" s="6" t="n">
-        <x:v>83</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Z48" s="15" t="str">
         <x:f>IF(AND(N48="Yes",AA48="Both distinct selected papers covered"),SQRT((W48+1)*(Y48+1))*IF(Q48="High",1,0.8),"")</x:f>
@@ -10383,10 +10451,10 @@
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC48" s="6" t="str">
-        <x:v>U2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="AD48" s="6" t="str">
-        <x:v>Action trajectory/tokens</x:v>
+        <x:v>Generated image/video</x:v>
       </x:c>
       <x:c r="AE48" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10394,124 +10462,112 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="6" t="str">
-        <x:f>IF(Z49="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z49))</x:f>
+        <x:f>IF(Z49="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z49))</x:f>
       </x:c>
       <x:c r="B49" s="6" t="str">
-        <x:v>R037</x:v>
+        <x:v>R030</x:v>
       </x:c>
       <x:c r="C49" s="6" t="str">
-        <x:v>Suraj Nair</x:v>
+        <x:v>Xiaolong Wang</x:v>
       </x:c>
       <x:c r="D49" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E49" s="6" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>UC San Diego</x:v>
       </x:c>
       <x:c r="F49" s="6" t="str">
-        <x:v>VL</x:v>
+        <x:v>U2</x:v>
       </x:c>
       <x:c r="G49" s="6" t="str">
-        <x:v>Perception backbone</x:v>
+        <x:v>Reward / affordance</x:v>
       </x:c>
       <x:c r="H49" s="6" t="str">
-        <x:v>Bridger</x:v>
+        <x:v>Native hybrid</x:v>
       </x:c>
       <x:c r="I49" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J49" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K49" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L49" s="6" t="str">
-        <x:v>Emerging</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M49" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N49" s="6" t="str">
         <x:f>IF(AND(L49="Yes",M49="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="O49" s="6" t="str">
-        <x:v>R3M</x:v>
+        <x:v>Unsupervised video representation</x:v>
       </x:c>
       <x:c r="P49" s="6" t="str">
-        <x:v>R3M</x:v>
+        <x:v>Robot learning from video</x:v>
       </x:c>
       <x:c r="Q49" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R49" s="6" t="str">
-        <x:v>Human-video temporal and language alignment transferred as a frozen robot perception backbone</x:v>
+        <x:v>Motion/interaction understanding to robotics</x:v>
       </x:c>
       <x:c r="S49" s="6" t="str">
-        <x:v>https://suraj-nair-1.github.io/</x:v>
+        <x:v>https://xiaolonw.github.io/</x:v>
       </x:c>
       <x:c r="T49" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2203.12601</x:v>
+        <x:v>https://arxiv.org/abs/1905.11993</x:v>
       </x:c>
       <x:c r="U49" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2203.12601</x:v>
-      </x:c>
-      <x:c r="V49" s="6" t="str">
-        <x:v>P066</x:v>
-      </x:c>
-      <x:c r="W49" s="6" t="n">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="X49" s="6" t="str">
-        <x:v>P066</x:v>
-      </x:c>
-      <x:c r="Y49" s="6" t="n">
-        <x:v>82</x:v>
-      </x:c>
+        <x:v>https://arxiv.org/abs/2204.01691</x:v>
+      </x:c>
+      <x:c r="V49" s="6"/>
+      <x:c r="W49" s="6"/>
+      <x:c r="X49" s="6"/>
+      <x:c r="Y49" s="6"/>
       <x:c r="Z49" s="15" t="str">
         <x:f>IF(AND(N49="Yes",AA49="Both distinct selected papers covered"),SQRT((W49+1)*(Y49+1))*IF(Q49="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA49" s="6" t="str">
-        <x:v>Single bridge paper used on both sides</x:v>
+        <x:v>Partial / missing selected-paper coverage</x:v>
       </x:c>
       <x:c r="AB49" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC49" s="6" t="str">
-        <x:v>VL</x:v>
-      </x:c>
-      <x:c r="AD49" s="6" t="str">
-        <x:v>Representation/reward/value</x:v>
-      </x:c>
+      <x:c r="AC49" s="6"/>
+      <x:c r="AD49" s="6"/>
       <x:c r="AE49" s="6" t="str">
-        <x:v>Verified single-paper bridge; not ranked</x:v>
+        <x:v>Partial evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="6" t="str">
-        <x:f>IF(Z50="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z50))</x:f>
+        <x:f>IF(Z50="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z50))</x:f>
       </x:c>
       <x:c r="B50" s="6" t="str">
-        <x:v>R052</x:v>
+        <x:v>R019</x:v>
       </x:c>
       <x:c r="C50" s="6" t="str">
-        <x:v>Tim Brooks</x:v>
+        <x:v>Xun Huang</x:v>
       </x:c>
       <x:c r="D50" s="6" t="str">
-        <x:v>Europe</x:v>
+        <x:v>US</x:v>
       </x:c>
       <x:c r="E50" s="6" t="str">
-        <x:v>OpenAI → Google DeepMind London</x:v>
+        <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="F50" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G50" s="6" t="str">
         <x:v>World simulation</x:v>
       </x:c>
       <x:c r="H50" s="6" t="str">
-        <x:v>Switcher</x:v>
+        <x:v>Bridger</x:v>
       </x:c>
       <x:c r="I50" s="6" t="n">
         <x:v>3</x:v>
@@ -10533,66 +10589,78 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="O50" s="6" t="str">
-        <x:v>Sora / video generation</x:v>
+        <x:v>Video/image synthesis</x:v>
       </x:c>
       <x:c r="P50" s="6" t="str">
-        <x:v>Interactive world models</x:v>
+        <x:v>Cosmos</x:v>
       </x:c>
       <x:c r="Q50" s="6" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="R50" s="6" t="str">
-        <x:v>Clear video→world-model move; physical-robot evidence still limited</x:v>
+        <x:v>Generative backbone to physical-AI world models</x:v>
       </x:c>
       <x:c r="S50" s="6" t="str">
-        <x:v>https://scholar.google.com/scholar?q=Tim+Brooks+video+generation</x:v>
+        <x:v>https://xunhuang1995.github.io/</x:v>
       </x:c>
       <x:c r="T50" s="6" t="str">
-        <x:v>https://openai.com/index/video-generation-models-as-world-simulators/</x:v>
+        <x:v>https://arxiv.org/abs/1808.06601</x:v>
       </x:c>
       <x:c r="U50" s="6" t="str">
-        <x:v>https://deepmind.google/discover/blog/genie-2-a-large-scale-foundation-world-model/</x:v>
-      </x:c>
-      <x:c r="V50" s="6"/>
-      <x:c r="W50" s="6"/>
-      <x:c r="X50" s="6"/>
-      <x:c r="Y50" s="6"/>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
+      </x:c>
+      <x:c r="V50" s="6" t="str">
+        <x:v>P016</x:v>
+      </x:c>
+      <x:c r="W50" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="X50" s="6" t="str">
+        <x:v>P016</x:v>
+      </x:c>
+      <x:c r="Y50" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="Z50" s="15" t="str">
         <x:f>IF(AND(N50="Yes",AA50="Both distinct selected papers covered"),SQRT((W50+1)*(Y50+1))*IF(Q50="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA50" s="6" t="str">
-        <x:v>Partial / missing selected-paper coverage</x:v>
+        <x:v>Single bridge paper used on both sides</x:v>
       </x:c>
       <x:c r="AB50" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC50" s="6"/>
-      <x:c r="AD50" s="6"/>
+      <x:c r="AC50" s="6" t="str">
+        <x:v>G2</x:v>
+      </x:c>
+      <x:c r="AD50" s="6" t="str">
+        <x:v>Predicted future video/state</x:v>
+      </x:c>
       <x:c r="AE50" s="6" t="str">
-        <x:v>Partial evidence</x:v>
+        <x:v>Verified single-paper bridge; not ranked</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="6" t="str">
-        <x:f>IF(Z51="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z51))</x:f>
+        <x:f>IF(Z51="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z51))</x:f>
       </x:c>
       <x:c r="B51" s="6" t="str">
-        <x:v>R040</x:v>
+        <x:v>R023</x:v>
       </x:c>
       <x:c r="C51" s="6" t="str">
-        <x:v>Wenlong Huang</x:v>
+        <x:v>Yihuai Gao</x:v>
       </x:c>
       <x:c r="D51" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E51" s="6" t="str">
-        <x:v>Stanford</x:v>
+        <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="F51" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G51" s="6" t="str">
-        <x:v>Planning</x:v>
+        <x:v>World simulation</x:v>
       </x:c>
       <x:c r="H51" s="6" t="str">
         <x:v>Bridger</x:v>
@@ -10601,53 +10669,53 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J51" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K51" s="6" t="n">
         <x:v>2</x:v>
-      </x:c>
-      <x:c r="K51" s="6" t="n">
-        <x:v>3</x:v>
       </x:c>
       <x:c r="L51" s="6" t="str">
         <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M51" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="N51" s="6" t="str">
         <x:f>IF(AND(L51="Yes",M51="Yes"),"Yes","No")</x:f>
         <x:v>No</x:v>
       </x:c>
       <x:c r="O51" s="6" t="str">
-        <x:v>Generative planning</x:v>
+        <x:v>Cosmos</x:v>
       </x:c>
       <x:c r="P51" s="6" t="str">
-        <x:v>Dream2Flow</x:v>
+        <x:v>Cosmos robotics applications</x:v>
       </x:c>
       <x:c r="Q51" s="6" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="R51" s="6" t="str">
-        <x:v>Recent bridge; exact citation tracked via project page</x:v>
+        <x:v>Recent bridge; impact still maturing</x:v>
       </x:c>
       <x:c r="S51" s="6" t="str">
-        <x:v>https://wenlong.page/</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="T51" s="6" t="str">
-        <x:v>https://jiajunwu.com/</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="U51" s="6" t="str">
-        <x:v>https://jiajunwu.com/</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="V51" s="6" t="str">
-        <x:v>P026</x:v>
+        <x:v>P016</x:v>
       </x:c>
       <x:c r="W51" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X51" s="6" t="str">
-        <x:v>P026</x:v>
+        <x:v>P016</x:v>
       </x:c>
       <x:c r="Y51" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="Z51" s="15" t="str">
         <x:f>IF(AND(N51="Yes",AA51="Both distinct selected papers covered"),SQRT((W51+1)*(Y51+1))*IF(Q51="High",1,0.8),"")</x:f>
@@ -10659,10 +10727,10 @@
         <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="AC51" s="6" t="str">
-        <x:v>G1</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="AD51" s="6" t="str">
-        <x:v>Generated image/video</x:v>
+        <x:v>Predicted future video/state</x:v>
       </x:c>
       <x:c r="AE51" s="6" t="str">
         <x:v>Verified single-paper bridge; not ranked</x:v>
@@ -10670,97 +10738,109 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="6" t="str">
-        <x:f>IF(Z52="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z52))</x:f>
+        <x:f>IF(Z52="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z52))</x:f>
       </x:c>
       <x:c r="B52" s="6" t="str">
-        <x:v>R030</x:v>
+        <x:v>R056</x:v>
       </x:c>
       <x:c r="C52" s="6" t="str">
-        <x:v>Xiaolong Wang</x:v>
+        <x:v>Yuke Zhu</x:v>
       </x:c>
       <x:c r="D52" s="6" t="str">
         <x:v>US</x:v>
       </x:c>
       <x:c r="E52" s="6" t="str">
-        <x:v>UC San Diego</x:v>
+        <x:v>UT Austin / NVIDIA</x:v>
       </x:c>
       <x:c r="F52" s="6" t="str">
-        <x:v>U2</x:v>
+        <x:v>VL</x:v>
       </x:c>
       <x:c r="G52" s="6" t="str">
-        <x:v>Reward / affordance</x:v>
+        <x:v>Direct policy</x:v>
       </x:c>
       <x:c r="H52" s="6" t="str">
         <x:v>Native hybrid</x:v>
       </x:c>
       <x:c r="I52" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J52" s="6" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K52" s="6" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="L52" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Emerging</x:v>
       </x:c>
       <x:c r="M52" s="6" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N52" s="6" t="str">
         <x:f>IF(AND(L52="Yes",M52="Yes"),"Yes","No")</x:f>
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="O52" s="6" t="str">
-        <x:v>Unsupervised video representation</x:v>
+        <x:v>Multimodal representation</x:v>
       </x:c>
       <x:c r="P52" s="6" t="str">
-        <x:v>Robot learning from video</x:v>
+        <x:v>VIMA; robot learning</x:v>
       </x:c>
       <x:c r="Q52" s="6" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="R52" s="6" t="str">
-        <x:v>Motion/interaction understanding to robotics</x:v>
+        <x:v>Robotics-led hybrid/control case</x:v>
       </x:c>
       <x:c r="S52" s="6" t="str">
-        <x:v>https://xiaolonw.github.io/</x:v>
+        <x:v>https://www.cs.utexas.edu/~yukez/</x:v>
       </x:c>
       <x:c r="T52" s="6" t="str">
-        <x:v>https://arxiv.org/abs/1905.11993</x:v>
+        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
       </x:c>
       <x:c r="U52" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2204.01691</x:v>
-      </x:c>
-      <x:c r="V52" s="6"/>
-      <x:c r="W52" s="6"/>
-      <x:c r="X52" s="6"/>
-      <x:c r="Y52" s="6"/>
+        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
+      </x:c>
+      <x:c r="V52" s="6" t="str">
+        <x:v>P019</x:v>
+      </x:c>
+      <x:c r="W52" s="6" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="X52" s="6" t="str">
+        <x:v>P019</x:v>
+      </x:c>
+      <x:c r="Y52" s="6" t="n">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="Z52" s="15" t="str">
         <x:f>IF(AND(N52="Yes",AA52="Both distinct selected papers covered"),SQRT((W52+1)*(Y52+1))*IF(Q52="High",1,0.8),"")</x:f>
       </x:c>
       <x:c r="AA52" s="6" t="str">
-        <x:v>Partial / missing selected-paper coverage</x:v>
+        <x:v>Single bridge paper used on both sides</x:v>
       </x:c>
       <x:c r="AB52" s="6" t="str">
         <x:v>2026-09-02</x:v>
       </x:c>
-      <x:c r="AC52" s="6"/>
-      <x:c r="AD52" s="6"/>
+      <x:c r="AC52" s="6" t="str">
+        <x:v>VL</x:v>
+      </x:c>
+      <x:c r="AD52" s="6" t="str">
+        <x:v>Action trajectory/tokens</x:v>
+      </x:c>
       <x:c r="AE52" s="6" t="str">
-        <x:v>Partial evidence</x:v>
+        <x:v>Verified single-paper bridge; not ranked</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="6" t="str">
-        <x:f>IF(Z53="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z53))</x:f>
+        <x:f>IF(Z53="","",1+COUNTIF($Z$2:$Z$53,"&gt;"&amp;Z53))</x:f>
       </x:c>
       <x:c r="B53" s="6" t="str">
-        <x:v>R019</x:v>
+        <x:v>R022</x:v>
       </x:c>
       <x:c r="C53" s="6" t="str">
-        <x:v>Xun Huang</x:v>
+        <x:v>Yunhao Ge</x:v>
       </x:c>
       <x:c r="D53" s="6" t="str">
         <x:v>US</x:v>
@@ -10781,7 +10861,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J53" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K53" s="6" t="n">
         <x:v>2</x:v>
@@ -10797,7 +10877,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="O53" s="6" t="str">
-        <x:v>Video/image synthesis</x:v>
+        <x:v>Generative visual models</x:v>
       </x:c>
       <x:c r="P53" s="6" t="str">
         <x:v>Cosmos</x:v>
@@ -10806,13 +10886,13 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="R53" s="6" t="str">
-        <x:v>Generative backbone to physical-AI world models</x:v>
+        <x:v>Physical-AI model development</x:v>
       </x:c>
       <x:c r="S53" s="6" t="str">
-        <x:v>https://xunhuang1995.github.io/</x:v>
+        <x:v>https://scholar.google.com/scholar?q=Yunhao+Ge+NVIDIA+Cosmos</x:v>
       </x:c>
       <x:c r="T53" s="6" t="str">
-        <x:v>https://arxiv.org/abs/1808.06601</x:v>
+        <x:v>https://arxiv.org/abs/2501.03575</x:v>
       </x:c>
       <x:c r="U53" s="6" t="str">
         <x:v>https://arxiv.org/abs/2501.03575</x:v>
@@ -10849,388 +10929,136 @@
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="6" t="str">
-        <x:f>IF(Z54="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z54))</x:f>
-      </x:c>
-      <x:c r="B54" s="6" t="str">
-        <x:v>R023</x:v>
-      </x:c>
-      <x:c r="C54" s="6" t="str">
-        <x:v>Yihuai Gao</x:v>
-      </x:c>
-      <x:c r="D54" s="6" t="str">
-        <x:v>US</x:v>
-      </x:c>
-      <x:c r="E54" s="6" t="str">
-        <x:v>NVIDIA</x:v>
-      </x:c>
-      <x:c r="F54" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="G54" s="6" t="str">
-        <x:v>World simulation</x:v>
-      </x:c>
-      <x:c r="H54" s="6" t="str">
-        <x:v>Bridger</x:v>
-      </x:c>
-      <x:c r="I54" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J54" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K54" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="L54" s="6" t="str">
-        <x:v>Emerging</x:v>
-      </x:c>
-      <x:c r="M54" s="6" t="str">
-        <x:v>Emerging</x:v>
-      </x:c>
-      <x:c r="N54" s="6" t="str">
-        <x:f>IF(AND(L54="Yes",M54="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="O54" s="6" t="str">
-        <x:v>Cosmos</x:v>
-      </x:c>
-      <x:c r="P54" s="6" t="str">
-        <x:v>Cosmos robotics applications</x:v>
-      </x:c>
-      <x:c r="Q54" s="6" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="R54" s="6" t="str">
-        <x:v>Recent bridge; impact still maturing</x:v>
-      </x:c>
-      <x:c r="S54" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
-      </x:c>
-      <x:c r="T54" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
-      </x:c>
-      <x:c r="U54" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
-      </x:c>
-      <x:c r="V54" s="6" t="str">
-        <x:v>P016</x:v>
-      </x:c>
-      <x:c r="W54" s="6" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="X54" s="6" t="str">
-        <x:v>P016</x:v>
-      </x:c>
-      <x:c r="Y54" s="6" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="Z54" s="15" t="str">
-        <x:f>IF(AND(N54="Yes",AA54="Both distinct selected papers covered"),SQRT((W54+1)*(Y54+1))*IF(Q54="High",1,0.8),"")</x:f>
-      </x:c>
-      <x:c r="AA54" s="6" t="str">
-        <x:v>Single bridge paper used on both sides</x:v>
-      </x:c>
-      <x:c r="AB54" s="6" t="str">
-        <x:v>2026-09-02</x:v>
-      </x:c>
-      <x:c r="AC54" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="AD54" s="6" t="str">
-        <x:v>Predicted future video/state</x:v>
-      </x:c>
-      <x:c r="AE54" s="6" t="str">
-        <x:v>Verified single-paper bridge; not ranked</x:v>
-      </x:c>
+      <x:c r="A54"/>
+      <x:c r="B54"/>
+      <x:c r="C54"/>
+      <x:c r="D54"/>
+      <x:c r="E54"/>
+      <x:c r="F54"/>
+      <x:c r="G54"/>
+      <x:c r="H54"/>
+      <x:c r="I54"/>
+      <x:c r="J54"/>
+      <x:c r="K54"/>
+      <x:c r="L54"/>
+      <x:c r="M54"/>
+      <x:c r="N54"/>
+      <x:c r="O54"/>
+      <x:c r="P54"/>
+      <x:c r="Q54"/>
+      <x:c r="R54"/>
+      <x:c r="S54"/>
+      <x:c r="T54"/>
+      <x:c r="U54"/>
+      <x:c r="V54"/>
+      <x:c r="W54"/>
+      <x:c r="X54"/>
+      <x:c r="Y54"/>
+      <x:c r="Z54"/>
+      <x:c r="AA54"/>
+      <x:c r="AB54"/>
+      <x:c r="AC54"/>
+      <x:c r="AD54"/>
+      <x:c r="AE54"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="6" t="str">
-        <x:f>IF(Z55="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z55))</x:f>
-      </x:c>
-      <x:c r="B55" s="6" t="str">
-        <x:v>R056</x:v>
-      </x:c>
-      <x:c r="C55" s="6" t="str">
-        <x:v>Yuke Zhu</x:v>
-      </x:c>
-      <x:c r="D55" s="6" t="str">
-        <x:v>US</x:v>
-      </x:c>
-      <x:c r="E55" s="6" t="str">
-        <x:v>UT Austin / NVIDIA</x:v>
-      </x:c>
-      <x:c r="F55" s="6" t="str">
-        <x:v>VL</x:v>
-      </x:c>
-      <x:c r="G55" s="6" t="str">
-        <x:v>Direct policy</x:v>
-      </x:c>
-      <x:c r="H55" s="6" t="str">
-        <x:v>Native hybrid</x:v>
-      </x:c>
-      <x:c r="I55" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J55" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K55" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L55" s="6" t="str">
-        <x:v>Emerging</x:v>
-      </x:c>
-      <x:c r="M55" s="6" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="N55" s="6" t="str">
-        <x:f>IF(AND(L55="Yes",M55="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="O55" s="6" t="str">
-        <x:v>Multimodal representation</x:v>
-      </x:c>
-      <x:c r="P55" s="6" t="str">
-        <x:v>VIMA; robot learning</x:v>
-      </x:c>
-      <x:c r="Q55" s="6" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="R55" s="6" t="str">
-        <x:v>Robotics-led hybrid/control case</x:v>
-      </x:c>
-      <x:c r="S55" s="6" t="str">
-        <x:v>https://www.cs.utexas.edu/~yukez/</x:v>
-      </x:c>
-      <x:c r="T55" s="6" t="str">
-        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
-      </x:c>
-      <x:c r="U55" s="6" t="str">
-        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
-      </x:c>
-      <x:c r="V55" s="6" t="str">
-        <x:v>P019</x:v>
-      </x:c>
-      <x:c r="W55" s="6" t="n">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="X55" s="6" t="str">
-        <x:v>P019</x:v>
-      </x:c>
-      <x:c r="Y55" s="6" t="n">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="Z55" s="15" t="str">
-        <x:f>IF(AND(N55="Yes",AA55="Both distinct selected papers covered"),SQRT((W55+1)*(Y55+1))*IF(Q55="High",1,0.8),"")</x:f>
-      </x:c>
-      <x:c r="AA55" s="6" t="str">
-        <x:v>Single bridge paper used on both sides</x:v>
-      </x:c>
-      <x:c r="AB55" s="6" t="str">
-        <x:v>2026-09-02</x:v>
-      </x:c>
-      <x:c r="AC55" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
-      <x:c r="AD55" s="6" t="str">
-        <x:v>Action trajectory/tokens</x:v>
-      </x:c>
-      <x:c r="AE55" s="6" t="str">
-        <x:v>Verified single-paper bridge; not ranked</x:v>
-      </x:c>
+      <x:c r="A55"/>
+      <x:c r="B55"/>
+      <x:c r="C55"/>
+      <x:c r="D55"/>
+      <x:c r="E55"/>
+      <x:c r="F55"/>
+      <x:c r="G55"/>
+      <x:c r="H55"/>
+      <x:c r="I55"/>
+      <x:c r="J55"/>
+      <x:c r="K55"/>
+      <x:c r="L55"/>
+      <x:c r="M55"/>
+      <x:c r="N55"/>
+      <x:c r="O55"/>
+      <x:c r="P55"/>
+      <x:c r="Q55"/>
+      <x:c r="R55"/>
+      <x:c r="S55"/>
+      <x:c r="T55"/>
+      <x:c r="U55"/>
+      <x:c r="V55"/>
+      <x:c r="W55"/>
+      <x:c r="X55"/>
+      <x:c r="Y55"/>
+      <x:c r="Z55"/>
+      <x:c r="AA55"/>
+      <x:c r="AB55"/>
+      <x:c r="AC55"/>
+      <x:c r="AD55"/>
+      <x:c r="AE55"/>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="6" t="str">
-        <x:f>IF(Z56="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z56))</x:f>
-      </x:c>
-      <x:c r="B56" s="6" t="str">
-        <x:v>R054</x:v>
-      </x:c>
-      <x:c r="C56" s="6" t="str">
-        <x:v>Yunfan Jiang</x:v>
-      </x:c>
-      <x:c r="D56" s="6" t="str">
-        <x:v>US</x:v>
-      </x:c>
-      <x:c r="E56" s="6" t="str">
-        <x:v>Stanford / NVIDIA</x:v>
-      </x:c>
-      <x:c r="F56" s="6" t="str">
-        <x:v>VL</x:v>
-      </x:c>
-      <x:c r="G56" s="6" t="str">
-        <x:v>Direct policy</x:v>
-      </x:c>
-      <x:c r="H56" s="6" t="str">
-        <x:v>Robotics-first</x:v>
-      </x:c>
-      <x:c r="I56" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J56" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K56" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="L56" s="6" t="str">
-        <x:v>Emerging</x:v>
-      </x:c>
-      <x:c r="M56" s="6" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="N56" s="6" t="str">
-        <x:f>IF(AND(L56="Yes",M56="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="O56" s="6" t="str">
-        <x:v>Multimodal prompts</x:v>
-      </x:c>
-      <x:c r="P56" s="6" t="str">
-        <x:v>VIMA</x:v>
-      </x:c>
-      <x:c r="Q56" s="6" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="R56" s="6" t="str">
-        <x:v>Key VIMA author; not a clear video-first trajectory</x:v>
-      </x:c>
-      <x:c r="S56" s="6" t="str">
-        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
-      </x:c>
-      <x:c r="T56" s="6" t="str">
-        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
-      </x:c>
-      <x:c r="U56" s="6" t="str">
-        <x:v>https://openreview.net/forum?id=oU2DzdTI94</x:v>
-      </x:c>
-      <x:c r="V56" s="6" t="str">
-        <x:v>P019</x:v>
-      </x:c>
-      <x:c r="W56" s="6" t="n">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="X56" s="6" t="str">
-        <x:v>P019</x:v>
-      </x:c>
-      <x:c r="Y56" s="6" t="n">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="Z56" s="15" t="str">
-        <x:f>IF(AND(N56="Yes",AA56="Both distinct selected papers covered"),SQRT((W56+1)*(Y56+1))*IF(Q56="High",1,0.8),"")</x:f>
-      </x:c>
-      <x:c r="AA56" s="6" t="str">
-        <x:v>Single bridge paper used on both sides</x:v>
-      </x:c>
-      <x:c r="AB56" s="6" t="str">
-        <x:v>2026-09-02</x:v>
-      </x:c>
-      <x:c r="AC56" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
-      <x:c r="AD56" s="6" t="str">
-        <x:v>Action trajectory/tokens</x:v>
-      </x:c>
-      <x:c r="AE56" s="6" t="str">
-        <x:v>Verified single-paper bridge; not ranked</x:v>
-      </x:c>
+      <x:c r="A56"/>
+      <x:c r="B56"/>
+      <x:c r="C56"/>
+      <x:c r="D56"/>
+      <x:c r="E56"/>
+      <x:c r="F56"/>
+      <x:c r="G56"/>
+      <x:c r="H56"/>
+      <x:c r="I56"/>
+      <x:c r="J56"/>
+      <x:c r="K56"/>
+      <x:c r="L56"/>
+      <x:c r="M56"/>
+      <x:c r="N56"/>
+      <x:c r="O56"/>
+      <x:c r="P56"/>
+      <x:c r="Q56"/>
+      <x:c r="R56"/>
+      <x:c r="S56"/>
+      <x:c r="T56"/>
+      <x:c r="U56"/>
+      <x:c r="V56"/>
+      <x:c r="W56"/>
+      <x:c r="X56"/>
+      <x:c r="Y56"/>
+      <x:c r="Z56"/>
+      <x:c r="AA56"/>
+      <x:c r="AB56"/>
+      <x:c r="AC56"/>
+      <x:c r="AD56"/>
+      <x:c r="AE56"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="6" t="str">
-        <x:f>IF(Z57="","",1+COUNTIF($Z$2:$Z$57,"&gt;"&amp;Z57))</x:f>
-      </x:c>
-      <x:c r="B57" s="6" t="str">
-        <x:v>R022</x:v>
-      </x:c>
-      <x:c r="C57" s="6" t="str">
-        <x:v>Yunhao Ge</x:v>
-      </x:c>
-      <x:c r="D57" s="6" t="str">
-        <x:v>US</x:v>
-      </x:c>
-      <x:c r="E57" s="6" t="str">
-        <x:v>NVIDIA</x:v>
-      </x:c>
-      <x:c r="F57" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="G57" s="6" t="str">
-        <x:v>World simulation</x:v>
-      </x:c>
-      <x:c r="H57" s="6" t="str">
-        <x:v>Bridger</x:v>
-      </x:c>
-      <x:c r="I57" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J57" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K57" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="L57" s="6" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="M57" s="6" t="str">
-        <x:v>Emerging</x:v>
-      </x:c>
-      <x:c r="N57" s="6" t="str">
-        <x:f>IF(AND(L57="Yes",M57="Yes"),"Yes","No")</x:f>
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="O57" s="6" t="str">
-        <x:v>Generative visual models</x:v>
-      </x:c>
-      <x:c r="P57" s="6" t="str">
-        <x:v>Cosmos</x:v>
-      </x:c>
-      <x:c r="Q57" s="6" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="R57" s="6" t="str">
-        <x:v>Physical-AI model development</x:v>
-      </x:c>
-      <x:c r="S57" s="6" t="str">
-        <x:v>https://scholar.google.com/scholar?q=Yunhao+Ge+NVIDIA+Cosmos</x:v>
-      </x:c>
-      <x:c r="T57" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
-      </x:c>
-      <x:c r="U57" s="6" t="str">
-        <x:v>https://arxiv.org/abs/2501.03575</x:v>
-      </x:c>
-      <x:c r="V57" s="6" t="str">
-        <x:v>P016</x:v>
-      </x:c>
-      <x:c r="W57" s="6" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="X57" s="6" t="str">
-        <x:v>P016</x:v>
-      </x:c>
-      <x:c r="Y57" s="6" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="Z57" s="15" t="str">
-        <x:f>IF(AND(N57="Yes",AA57="Both distinct selected papers covered"),SQRT((W57+1)*(Y57+1))*IF(Q57="High",1,0.8),"")</x:f>
-      </x:c>
-      <x:c r="AA57" s="6" t="str">
-        <x:v>Single bridge paper used on both sides</x:v>
-      </x:c>
-      <x:c r="AB57" s="6" t="str">
-        <x:v>2026-09-02</x:v>
-      </x:c>
-      <x:c r="AC57" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="AD57" s="6" t="str">
-        <x:v>Predicted future video/state</x:v>
-      </x:c>
-      <x:c r="AE57" s="6" t="str">
-        <x:v>Verified single-paper bridge; not ranked</x:v>
-      </x:c>
+      <x:c r="A57"/>
+      <x:c r="B57"/>
+      <x:c r="C57"/>
+      <x:c r="D57"/>
+      <x:c r="E57"/>
+      <x:c r="F57"/>
+      <x:c r="G57"/>
+      <x:c r="H57"/>
+      <x:c r="I57"/>
+      <x:c r="J57"/>
+      <x:c r="K57"/>
+      <x:c r="L57"/>
+      <x:c r="M57"/>
+      <x:c r="N57"/>
+      <x:c r="O57"/>
+      <x:c r="P57"/>
+      <x:c r="Q57"/>
+      <x:c r="R57"/>
+      <x:c r="S57"/>
+      <x:c r="T57"/>
+      <x:c r="U57"/>
+      <x:c r="V57"/>
+      <x:c r="W57"/>
+      <x:c r="X57"/>
+      <x:c r="Y57"/>
+      <x:c r="Z57"/>
+      <x:c r="AA57"/>
+      <x:c r="AB57"/>
+      <x:c r="AC57"/>
+      <x:c r="AD57"/>
+      <x:c r="AE57"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58"/>
@@ -11271,7 +11099,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb16bcf1f2b045f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95436ef363d64c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11300,7 +11128,7 @@
       <x:c r="E1" s="3"/>
       <x:c r="F1" s="3"/>
       <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
+      <x:c r="H1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2"/>
@@ -11342,7 +11170,7 @@
       <x:c r="G4" s="14" t="str">
         <x:v>Direct policy</x:v>
       </x:c>
-      <x:c r="H4" s="12"/>
+      <x:c r="H4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="6" t="str">
@@ -11366,7 +11194,7 @@
       <x:c r="G5" s="17" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H5" s="17"/>
+      <x:c r="H5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="6" t="str">
@@ -11390,7 +11218,7 @@
       <x:c r="G6" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H6" s="17"/>
+      <x:c r="H6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="6" t="str">
@@ -11414,7 +11242,7 @@
       <x:c r="G7" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H7" s="17"/>
+      <x:c r="H7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="6" t="str">
@@ -11438,7 +11266,7 @@
       <x:c r="G8" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H8" s="17"/>
+      <x:c r="H8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6" t="str">
@@ -11460,9 +11288,9 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="17" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="H9" s="17"/>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="6" t="str">
@@ -11486,7 +11314,7 @@
       <x:c r="G10" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H10" s="17"/>
+      <x:c r="H10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="6" t="str">
@@ -11508,281 +11336,253 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="17" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H11" s="17"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H11"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
-      <x:c r="B12" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C12" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D12" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E12" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F12" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G12" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H12" s="17"/>
+      <x:c r="A12" s="6"/>
+      <x:c r="B12" s="17"/>
+      <x:c r="C12" s="17"/>
+      <x:c r="D12" s="17"/>
+      <x:c r="E12" s="17"/>
+      <x:c r="F12" s="17"/>
+      <x:c r="G12" s="17"/>
+      <x:c r="H12"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13"/>
-      <x:c r="B13" s="18"/>
-      <x:c r="C13" s="18"/>
-      <x:c r="D13" s="18"/>
-      <x:c r="E13" s="18"/>
-      <x:c r="F13" s="18"/>
-      <x:c r="G13" s="18"/>
-      <x:c r="H13" s="18"/>
+      <x:c r="A13" s="51" t="str">
+        <x:v>Direct bridge papers: same video-origin code × robot role</x:v>
+      </x:c>
+      <x:c r="B13" s="52"/>
+      <x:c r="C13" s="52"/>
+      <x:c r="D13" s="52"/>
+      <x:c r="E13" s="52"/>
+      <x:c r="F13" s="52"/>
+      <x:c r="G13" s="52"/>
+      <x:c r="H13"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="3" t="str">
-        <x:v>Direct bridge papers: same video-origin code × robot role</x:v>
-      </x:c>
+      <x:c r="A14" s="3"/>
       <x:c r="B14" s="19"/>
       <x:c r="C14" s="19"/>
       <x:c r="D14" s="19"/>
       <x:c r="E14" s="19"/>
       <x:c r="F14" s="19"/>
       <x:c r="G14" s="19"/>
-      <x:c r="H14" s="18"/>
+      <x:c r="H14"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15"/>
-      <x:c r="B15" s="18"/>
-      <x:c r="C15" s="18"/>
-      <x:c r="D15" s="18"/>
-      <x:c r="E15" s="18"/>
-      <x:c r="F15" s="18"/>
-      <x:c r="G15" s="18"/>
-      <x:c r="H15" s="18"/>
+      <x:c r="A15" s="53" t="str">
+        <x:v>Origin</x:v>
+      </x:c>
+      <x:c r="B15" s="54" t="str">
+        <x:v>Perception backbone</x:v>
+      </x:c>
+      <x:c r="C15" s="54" t="str">
+        <x:v>Reward / affordance</x:v>
+      </x:c>
+      <x:c r="D15" s="54" t="str">
+        <x:v>Data generation</x:v>
+      </x:c>
+      <x:c r="E15" s="54" t="str">
+        <x:v>World simulation</x:v>
+      </x:c>
+      <x:c r="F15" s="54" t="str">
+        <x:v>Planning</x:v>
+      </x:c>
+      <x:c r="G15" s="54" t="str">
+        <x:v>Direct policy</x:v>
+      </x:c>
+      <x:c r="H15"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="11" t="str">
-        <x:v>Origin</x:v>
-      </x:c>
-      <x:c r="B16" s="16" t="str">
-        <x:v>Perception backbone</x:v>
-      </x:c>
-      <x:c r="C16" s="16" t="str">
-        <x:v>Reward / affordance</x:v>
-      </x:c>
-      <x:c r="D16" s="16" t="str">
-        <x:v>Data generation</x:v>
-      </x:c>
-      <x:c r="E16" s="16" t="str">
-        <x:v>World simulation</x:v>
-      </x:c>
-      <x:c r="F16" s="16" t="str">
-        <x:v>Planning</x:v>
-      </x:c>
-      <x:c r="G16" s="20" t="str">
-        <x:v>Direct policy</x:v>
-      </x:c>
-      <x:c r="H16" s="18"/>
+      <x:c r="A16" s="60" t="str">
+        <x:v>G1</x:v>
+      </x:c>
+      <x:c r="B16" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C16" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D16" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="61" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G16" s="62" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H16"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="6" t="str">
-        <x:v>G1</x:v>
-      </x:c>
-      <x:c r="B17" s="17" t="n">
+      <x:c r="A17" s="63" t="str">
+        <x:v>G2</x:v>
+      </x:c>
+      <x:c r="B17" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C17" s="17" t="n">
+      <x:c r="C17" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D17" s="17" t="n">
+      <x:c r="D17" s="64" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E17" s="17" t="n">
+      <x:c r="E17" s="64" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F17" s="64" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G17" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F17" s="17" t="n">
+      <x:c r="H17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="63" t="str">
+        <x:v>G3</x:v>
+      </x:c>
+      <x:c r="B18" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C18" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" s="64" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G17" s="17" t="n">
+      <x:c r="H18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="63" t="str">
+        <x:v>U1</x:v>
+      </x:c>
+      <x:c r="B19" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D19" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="63" t="str">
+        <x:v>U2</x:v>
+      </x:c>
+      <x:c r="B20" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C20" s="64" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H17" s="18"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="6" t="str">
-        <x:v>G2</x:v>
-      </x:c>
-      <x:c r="B18" s="17" t="n">
+      <x:c r="D20" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C18" s="17" t="n">
+      <x:c r="E20" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D18" s="17" t="n">
+      <x:c r="F20" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="64" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="63" t="str">
+        <x:v>U3</x:v>
+      </x:c>
+      <x:c r="B21" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C21" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="64" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E18" s="17" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="F18" s="17" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G18" s="17" t="n">
+      <x:c r="G21" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H18" s="18"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="6" t="str">
-        <x:v>G3</x:v>
-      </x:c>
-      <x:c r="B19" s="17" t="n">
+      <x:c r="H21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="63" t="str">
+        <x:v>VL</x:v>
+      </x:c>
+      <x:c r="B22" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D22" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C19" s="17" t="n">
+      <x:c r="E22" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D19" s="17" t="n">
+      <x:c r="F22" s="64" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E19" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F19" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G19" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H19" s="18"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="6" t="str">
-        <x:v>U1</x:v>
-      </x:c>
-      <x:c r="B20" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C20" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D20" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E20" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F20" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G20" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H20" s="18"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="6" t="str">
-        <x:v>U2</x:v>
-      </x:c>
-      <x:c r="B21" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C21" s="17" t="n">
+      <x:c r="G22" s="64" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D21" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E21" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F21" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G21" s="17" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="H21" s="18"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="6" t="str">
-        <x:v>U3</x:v>
-      </x:c>
-      <x:c r="B22" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C22" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D22" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E22" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F22" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G22" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H22" s="18"/>
+      <x:c r="H22"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="6" t="str">
-        <x:v>VL</x:v>
-      </x:c>
-      <x:c r="B23" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C23" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D23" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E23" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F23" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G23" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H23" s="18"/>
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+      <x:c r="G23"/>
+      <x:c r="H23"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
-      <x:c r="B24" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C24" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D24" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E24" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F24" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G24" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H24" s="18"/>
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+      <x:c r="G24"/>
+      <x:c r="H24"/>
     </x:row>
     <x:row r="25">
       <x:c r="B25"/>
@@ -11946,8 +11746,8 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C5" s="21" t="n">
-        <x:f>B5/SUM($B$5:$B$8)</x:f>
-        <x:v>0.03571428571428571</x:v>
+        <x:f>B5/SUM($B$5:$B$7)</x:f>
+        <x:v>0.038461538461538464</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11958,8 +11758,8 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="C6" s="21" t="n">
-        <x:f>B6/SUM($B$5:$B$8)</x:f>
-        <x:v>0.6964285714285714</x:v>
+        <x:f>B6/SUM($B$5:$B$7)</x:f>
+        <x:v>0.75</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -11970,21 +11770,14 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="C7" s="21" t="n">
-        <x:f>B7/SUM($B$5:$B$8)</x:f>
-        <x:v>0.19642857142857142</x:v>
+        <x:f>B7/SUM($B$5:$B$7)</x:f>
+        <x:v>0.21153846153846154</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="6" t="str">
-        <x:v>Robotics-first</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="21" t="n">
-        <x:f>B8/SUM($B$5:$B$8)</x:f>
-        <x:v>0.07142857142857142</x:v>
-      </x:c>
+      <x:c r="A8"/>
+      <x:c r="B8"/>
+      <x:c r="C8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9"/>
@@ -12062,7 +11855,7 @@
         <x:v>Researchers</x:v>
       </x:c>
       <x:c r="B5" s="6" t="n">
-        <x:v>56</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C5"/>
       <x:c r="D5" s="6" t="str">
@@ -12159,12 +11952,8 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F8"/>
-      <x:c r="G8" s="6" t="str">
-        <x:v>Robotics-first</x:v>
-      </x:c>
-      <x:c r="H8" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
+      <x:c r="G8" s="6"/>
+      <x:c r="H8" s="6"/>
       <x:c r="I8"/>
       <x:c r="J8" s="6" t="str">
         <x:v>U1</x:v>
@@ -12185,7 +11974,7 @@
         <x:v>U2</x:v>
       </x:c>
       <x:c r="E9" s="6" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F9"/>
       <x:c r="G9" s="6"/>
@@ -12228,14 +12017,14 @@
         <x:v>Single-paper bridges, not ranked</x:v>
       </x:c>
       <x:c r="B11" s="6" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C11"/>
       <x:c r="D11" s="6" t="str">
         <x:v>VL</x:v>
       </x:c>
       <x:c r="E11" s="6" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F11"/>
       <x:c r="G11"/>
@@ -12253,25 +12042,17 @@
         <x:v>Partial evidence rows</x:v>
       </x:c>
       <x:c r="B12" s="6" t="n">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C12"/>
-      <x:c r="D12" s="6" t="str">
-        <x:v>None</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="D12" s="6"/>
+      <x:c r="E12" s="6"/>
       <x:c r="F12"/>
       <x:c r="G12"/>
       <x:c r="H12"/>
       <x:c r="I12"/>
-      <x:c r="J12" t="str">
-        <x:v>None</x:v>
-      </x:c>
-      <x:c r="K12" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="J12"/>
+      <x:c r="K12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13"/>
@@ -12316,7 +12097,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="str">
-        <x:v>• One code axis maps video-origin architecture directly to robot role; model output is descriptive metadata, not a second code system.</x:v>
+        <x:v>— One code axis maps video-origin architecture directly to robot role; model output is descriptive metadata, not a second code system.</x:v>
       </x:c>
       <x:c r="B16" s="6"/>
       <x:c r="C16" s="6"/>
@@ -12331,7 +12112,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="str">
-        <x:v>• G1 researchers map mainly to planning (6), direct policy (4), and world simulation (3).</x:v>
+        <x:v>— G1 researchers map mainly to planning (6), direct policy (4), and world simulation (3).</x:v>
       </x:c>
       <x:c r="B17" s="6"/>
       <x:c r="C17" s="6"/>
@@ -12346,7 +12127,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="str">
-        <x:v>• Bridge Impact requires two distinct authored papers; single-paper bridges remain documented but are not ranked.</x:v>
+        <x:v>— Bridge Impact requires two distinct authored papers; single-paper bridges remain documented but are not ranked.</x:v>
       </x:c>
       <x:c r="B18" s="6"/>
       <x:c r="C18" s="6"/>
@@ -12361,7 +12142,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="6" t="str">
-        <x:v>• Tim Rocktäschel is excluded from the researcher sample because no physical-robot paper was verified; Genie remains a context paper.</x:v>
+        <x:v>— Four robotics-centered comparison cases were removed so the researcher denominator contains only verified video-to-robotics trajectories.</x:v>
       </x:c>
       <x:c r="B19" s="6"/>
       <x:c r="C19" s="6"/>
@@ -12376,7 +12157,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="6" t="str">
-        <x:v>• Counts describe this selected sample, not the full research population.</x:v>
+        <x:v>— Counts describe this selected sample, not the full research population.</x:v>
       </x:c>
       <x:c r="B20" s="6"/>
       <x:c r="C20" s="6"/>
@@ -12547,6 +12328,20 @@
         <x:v>No physical-robot paper was verified; virtual world-model and agent work alone does not meet the researcher inclusion rule</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>Kevin Black, Oier Mees, Pierre-Louis Guhur, Yunfan Jiang</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Robotics-centered comparison cases inside core researcher sample</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Excluded from core researcher sample; no empty-origin category retained</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>The published researcher denominator now contains only verified video-to-robotics trajectories. These four cases did not affect the ranked top 20.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>

</xml_diff>